<commit_message>
backlog update deferred PBI-041 and draft for enabler
</commit_message>
<xml_diff>
--- a/backlog/backlog.xlsx
+++ b/backlog/backlog.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="10668" windowHeight="9576"/>
+    <workbookView windowWidth="22188" windowHeight="9384"/>
   </bookViews>
   <sheets>
     <sheet name="backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">backlog!$A$1:$N$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">backlog!$A$1:$N$87</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1008" uniqueCount="535">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1055" uniqueCount="562">
   <si>
     <t>PBI-###</t>
   </si>
@@ -938,13 +938,16 @@
     <t>Action to be performed: build the admin form and user feedback for member organization registration. Why it is needed: administrators need a usable interface to create organizations and handle invalid input. Expected output: working form with validation messages and success state. Scope: form fields, submit flow, validation feedback, success and error states. Explicit exclusions: backend authorization and audit logging.</t>
   </si>
   <si>
-    <t>[ReqID: R03] Given valid registration data is entered, when the administrator submits the form, then the UI sends the request and displays a success result. | [ReqID: R03] Given invalid or duplicate data is entered, when submission is attempted, then the UI displays meaningful validation or error feedback.</t>
+    <t>[ReqID: R03] Given valid registration data is entered, when the administrator submits the form, then the UI sends the request and displays a success result aligned to the backend response. | [ReqID: R03] Given invalid or duplicate data is entered, when submission is attempted, then the UI displays meaningful validation or error feedback.</t>
   </si>
   <si>
     <t>Usability;Security;Maintainability</t>
   </si>
   <si>
-    <t>Important: Covers PBI-031 AC1 and AC2. Can run in parallel with PBI-040 after contract is stable. Evidence: screenshots, functional checks.</t>
+    <t>PBI-039;PBI-040;PBI-079;PBI-080;PBI-081;PBI-082</t>
+  </si>
+  <si>
+    <t>Important: Deferred pending approved frontend runway. Replace prior dependency chain with governed frontend prerequisites. Success-state messaging must align to the current backend membership workflow response model.</t>
   </si>
   <si>
     <t>PBI-042</t>
@@ -1635,6 +1638,84 @@
   </si>
   <si>
     <t>Important: Covers PBI-038 AC1 and AC2 plus DoD. Demo should show both intermediate and final decision histories.</t>
+  </si>
+  <si>
+    <t>PBI-079</t>
+  </si>
+  <si>
+    <t>Spike</t>
+  </si>
+  <si>
+    <t>Investigate governed frontend runway for repository-aligned UI work</t>
+  </si>
+  <si>
+    <t>Unknown / problem statement: the repository currently provides backend execution runway but no governed frontend execution boundary for Sprint UI work. Why a decision is needed now: PBI-041 cannot proceed safely without an approved frontend boundary, toolchain decision, and contract-consumer pattern. Investigation scope: frontend location, build/run/test commands, boundary ownership, contract-consumer rule, auth/session assumption, and minimum documentation updates. Explicit exclusions: no production-ready member onboarding form implementation. Approach: inspect current repo constraints, evaluate minimum frontend boundary options, and produce a documented recommendation.</t>
+  </si>
+  <si>
+    <t>[ReqID: R03] Given the spike timebox ends, when findings are reviewed, then a documented recommendation exists for whether frontend work proceeds now or remains deferred. | [ReqID: R03] Given a frontend boundary is recommended, when the spike closes, then minimum folder structure, commands, contract-consumer approach, and documentation impact are explicitly defined. | [ReqID: R03] Given PBI-041 depends on the outcome, when the spike closes, then follow-up backlog items and dependencies are identified.</t>
+  </si>
+  <si>
+    <t>Maintainability;Reliability;Architecture</t>
+  </si>
+  <si>
+    <t>Timebox: 2-3 calendar days. Exit Criteria: approved recommendation, minimum frontend boundary decision, run/build/test command decision, contract-consumer rule, follow-up PBIs. Important: This item exists to resolve the blocker before any resumed frontend delivery.</t>
+  </si>
+  <si>
+    <t>PBI-080</t>
+  </si>
+  <si>
+    <t>Enabler</t>
+  </si>
+  <si>
+    <t>Enable governed frontend application boundary for future Sprint UI work</t>
+  </si>
+  <si>
+    <t>Capability to be created or improved: establish a minimal governed frontend execution boundary inside the repository for future UI delivery. Why it is needed: frontend work should not proceed through ad hoc files or disconnected mock screens. Which future PBIs it enables: PBI-041 and later UI tasks under membership and shariah-review flows. Technical scope: frontend entry point, page shell, package scripts, build/run/test commands, minimal shared structure, and repo-aligned folder conventions. Explicit exclusions: completed member onboarding form behavior and advanced auth/session implementation.</t>
+  </si>
+  <si>
+    <t>[ReqID: R03] Given the approved runway decision exists, when the frontend boundary is created, then the repository contains a working frontend entry point and consistent local run/build/test flow. | [ReqID: R03] Given future UI tasks start, when contributors implement frontend work, then they do so inside the governed boundary rather than inventing a new structure. | [ReqID: R03] Given the boundary is reviewed, when the enabler is checked, then the scaffold and commands are documented and repeatable.</t>
+  </si>
+  <si>
+    <t>Important: Shared enablement item, not a child-only implementation detail of PBI-041. Evidence should include successful run/build output and scaffold tree.</t>
+  </si>
+  <si>
+    <t>PBI-081</t>
+  </si>
+  <si>
+    <t>Do define contract-consumer pattern and member onboarding page shell for future UI work</t>
+  </si>
+  <si>
+    <t>Action to be performed: define and implement the minimal frontend contract-consumer pattern and initial member onboarding page shell aligned to the existing backend membership contract. Why it is needed: future form work should consume backend contracts through an agreed pattern rather than ad hoc fetch logic. Expected output: onboarding page shell wired to a typed request layer or equivalent contract-aware client seam. Scope: page shell, request abstraction, request/response typing, success/error handling seam, and backend-consumer alignment. Explicit exclusions: final registration form UX, advanced auth enforcement, and completed frontend validation flows.</t>
+  </si>
+  <si>
+    <t>[ReqID: R03] Given the frontend boundary exists, when the page shell is reviewed, then there is a defined and reusable path to call member-organization creation. | [ReqID: R03] Given the backend contract is consumed, when success and error responses are handled, then the shell reflects the backend response model without ad hoc request code. | [ReqID: R03] Given later form work resumes, when submission behavior is added, then it plugs into the agreed client pattern.</t>
+  </si>
+  <si>
+    <t>Maintainability;Usability;Integration</t>
+  </si>
+  <si>
+    <t>PBI-079;PBI-080;PBI-039;PBI-040</t>
+  </si>
+  <si>
+    <t>Important: Direct unblocker for future PBI-041 resumption. Success-state design must align to backend-created organization lifecycle and not imply unsupported immediate activation.</t>
+  </si>
+  <si>
+    <t>PBI-082</t>
+  </si>
+  <si>
+    <t>Do align architecture and coding guidance for governed frontend boundary</t>
+  </si>
+  <si>
+    <t>Action to be performed: update repository architecture and coding guidance so future frontend work follows the same governed rules as the backend slice. Why it is needed: contributors should not rely on implicit chat memory or inconsistent local conventions for frontend implementation. Expected output: updated architecture, coding, and sprint execution guidance covering frontend boundary, folder rules, contract-first consumption, and test expectations. Scope: documentation alignment for the approved frontend boundary only. Explicit exclusions: broad SDLC rewrite and completed UI feature delivery.</t>
+  </si>
+  <si>
+    <t>[ReqID: R03] Given frontend runway is approved, when repository guidance is reviewed, then the frontend boundary and coding rules are explicit. | [ReqID: R03] Given future UI tasks are executed, when contributors implement frontend work, then documented conventions exist for structure, contract consumption, and test expectations.</t>
+  </si>
+  <si>
+    <t>Maintainability;Compliance;Architecture</t>
+  </si>
+  <si>
+    <t>Important: Update architecture guidance, coding rules, and sprint execution notes together so the repository does not contain conflicting delivery instructions.</t>
   </si>
 </sst>
 </file>
@@ -2306,11 +2387,25 @@
     <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="21">
+  <dxfs count="22">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FF64B5F6"/>
+          <bgColor theme="7" tint="0.4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFB74D"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF81C784"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2324,14 +2419,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FF81C784"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFB74D"/>
+          <bgColor rgb="FF64B5F6"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2528,25 +2616,25 @@
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
     <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="10"/>
-      <tableStyleElement type="headerRow" dxfId="9"/>
-      <tableStyleElement type="totalRow" dxfId="8"/>
-      <tableStyleElement type="firstColumn" dxfId="7"/>
-      <tableStyleElement type="lastColumn" dxfId="6"/>
-      <tableStyleElement type="firstRowStripe" dxfId="5"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="4"/>
+      <tableStyleElement type="wholeTable" dxfId="11"/>
+      <tableStyleElement type="headerRow" dxfId="10"/>
+      <tableStyleElement type="totalRow" dxfId="9"/>
+      <tableStyleElement type="firstColumn" dxfId="8"/>
+      <tableStyleElement type="lastColumn" dxfId="7"/>
+      <tableStyleElement type="firstRowStripe" dxfId="6"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="5"/>
     </tableStyle>
     <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="20"/>
-      <tableStyleElement type="totalRow" dxfId="19"/>
-      <tableStyleElement type="firstRowStripe" dxfId="18"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="17"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="16"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="15"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="14"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="13"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="12"/>
-      <tableStyleElement type="pageFieldValues" dxfId="11"/>
+      <tableStyleElement type="headerRow" dxfId="21"/>
+      <tableStyleElement type="totalRow" dxfId="20"/>
+      <tableStyleElement type="firstRowStripe" dxfId="19"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="18"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="17"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="16"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="15"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="14"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="13"/>
+      <tableStyleElement type="pageFieldValues" dxfId="12"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -2823,7 +2911,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:N79"/>
+  <dimension ref="A1:N83"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
@@ -3793,7 +3881,7 @@
         <v>34</v>
       </c>
       <c r="L23" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M23" t="s">
         <v>38</v>
@@ -4601,40 +4689,37 @@
       <c r="J42" t="s">
         <v>150</v>
       </c>
-      <c r="K42" t="s">
-        <v>247</v>
-      </c>
       <c r="L42" t="s">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="M42" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="N42" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="43" spans="1:14">
       <c r="A43" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B43" t="s">
         <v>287</v>
       </c>
       <c r="C43" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D43" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E43" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="F43" t="s">
         <v>42</v>
       </c>
       <c r="G43" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H43">
         <v>2</v>
@@ -4649,36 +4734,36 @@
         <v>247</v>
       </c>
       <c r="L43" t="s">
-        <v>45</v>
+        <v>291</v>
       </c>
       <c r="M43" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="N43" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="44" spans="1:14">
       <c r="A44" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B44" t="s">
         <v>287</v>
       </c>
       <c r="C44" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D44" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E44" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F44" t="s">
         <v>42</v>
       </c>
       <c r="G44" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H44">
         <v>2</v>
@@ -4693,30 +4778,30 @@
         <v>247</v>
       </c>
       <c r="L44" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M44" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="N44" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="45" spans="1:14">
       <c r="A45" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B45" t="s">
         <v>287</v>
       </c>
       <c r="C45" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D45" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E45" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F45" t="s">
         <v>42</v>
@@ -4743,24 +4828,24 @@
         <v>249</v>
       </c>
       <c r="N45" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="46" spans="1:14">
       <c r="A46" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B46" t="s">
         <v>287</v>
       </c>
       <c r="C46" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D46" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E46" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F46" t="s">
         <v>42</v>
@@ -4784,33 +4869,33 @@
         <v>35</v>
       </c>
       <c r="M46" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="N46" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="47" spans="1:14">
       <c r="A47" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B47" t="s">
         <v>287</v>
       </c>
       <c r="C47" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D47" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E47" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F47" t="s">
         <v>42</v>
       </c>
       <c r="G47" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="H47">
         <v>2</v>
@@ -4828,33 +4913,33 @@
         <v>35</v>
       </c>
       <c r="M47" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="N47" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="48" spans="1:14">
       <c r="A48" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B48" t="s">
         <v>287</v>
       </c>
       <c r="C48" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D48" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E48" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F48" t="s">
         <v>42</v>
       </c>
       <c r="G48" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H48">
         <v>2</v>
@@ -4872,33 +4957,33 @@
         <v>35</v>
       </c>
       <c r="M48" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="N48" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="49" spans="1:14">
       <c r="A49" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B49" t="s">
         <v>287</v>
       </c>
       <c r="C49" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D49" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E49" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="F49" t="s">
         <v>42</v>
       </c>
       <c r="G49" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H49">
         <v>2</v>
@@ -4916,27 +5001,27 @@
         <v>35</v>
       </c>
       <c r="M49" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="N49" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="50" spans="1:14">
       <c r="A50" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B50" t="s">
         <v>287</v>
       </c>
       <c r="C50" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D50" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="E50" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="F50" t="s">
         <v>42</v>
@@ -4951,7 +5036,7 @@
         <v>32</v>
       </c>
       <c r="J50" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="K50" t="s">
         <v>247</v>
@@ -4960,27 +5045,27 @@
         <v>35</v>
       </c>
       <c r="M50" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="N50" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="51" spans="1:14">
       <c r="A51" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B51" t="s">
         <v>287</v>
       </c>
       <c r="C51" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D51" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E51" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F51" t="s">
         <v>42</v>
@@ -5004,33 +5089,33 @@
         <v>35</v>
       </c>
       <c r="M51" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="N51" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="52" spans="1:14">
       <c r="A52" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B52" t="s">
         <v>287</v>
       </c>
       <c r="C52" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D52" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E52" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="F52" t="s">
         <v>42</v>
       </c>
       <c r="G52" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="H52">
         <v>2</v>
@@ -5048,33 +5133,33 @@
         <v>35</v>
       </c>
       <c r="M52" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="N52" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="53" spans="1:14">
       <c r="A53" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B53" t="s">
         <v>287</v>
       </c>
       <c r="C53" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="D53" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E53" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F53" t="s">
         <v>42</v>
       </c>
       <c r="G53" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H53">
         <v>2</v>
@@ -5092,33 +5177,33 @@
         <v>35</v>
       </c>
       <c r="M53" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="N53" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="54" spans="1:14">
       <c r="A54" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B54" t="s">
         <v>287</v>
       </c>
       <c r="C54" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D54" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="E54" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F54" t="s">
         <v>42</v>
       </c>
       <c r="G54" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H54">
         <v>2</v>
@@ -5136,27 +5221,27 @@
         <v>35</v>
       </c>
       <c r="M54" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="N54" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="55" spans="1:14">
       <c r="A55" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B55" t="s">
         <v>287</v>
       </c>
       <c r="C55" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="D55" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E55" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="F55" t="s">
         <v>42</v>
@@ -5171,7 +5256,7 @@
         <v>32</v>
       </c>
       <c r="J55" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="K55" t="s">
         <v>247</v>
@@ -5180,27 +5265,27 @@
         <v>35</v>
       </c>
       <c r="M55" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="N55" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="56" spans="1:14">
       <c r="A56" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B56" t="s">
         <v>287</v>
       </c>
       <c r="C56" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="D56" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="E56" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F56" t="s">
         <v>42</v>
@@ -5224,33 +5309,33 @@
         <v>35</v>
       </c>
       <c r="M56" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="N56" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="57" spans="1:14">
       <c r="A57" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B57" t="s">
         <v>287</v>
       </c>
       <c r="C57" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="D57" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="E57" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="F57" t="s">
         <v>42</v>
       </c>
       <c r="G57" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="H57">
         <v>2</v>
@@ -5268,33 +5353,33 @@
         <v>35</v>
       </c>
       <c r="M57" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="N57" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="58" spans="1:14">
       <c r="A58" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B58" t="s">
         <v>287</v>
       </c>
       <c r="C58" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="D58" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="E58" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="F58" t="s">
         <v>42</v>
       </c>
       <c r="G58" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="H58">
         <v>2</v>
@@ -5312,33 +5397,33 @@
         <v>35</v>
       </c>
       <c r="M58" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="N58" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="59" spans="1:14">
       <c r="A59" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B59" t="s">
         <v>287</v>
       </c>
       <c r="C59" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="D59" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="E59" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="F59" t="s">
         <v>42</v>
       </c>
       <c r="G59" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H59">
         <v>2</v>
@@ -5356,33 +5441,33 @@
         <v>35</v>
       </c>
       <c r="M59" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="N59" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="60" spans="1:14">
       <c r="A60" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B60" t="s">
         <v>287</v>
       </c>
       <c r="C60" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D60" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="E60" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="F60" t="s">
         <v>170</v>
       </c>
       <c r="G60" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="H60">
         <v>2</v>
@@ -5403,30 +5488,30 @@
         <v>264</v>
       </c>
       <c r="N60" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="61" spans="1:14">
       <c r="A61" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B61" t="s">
         <v>287</v>
       </c>
       <c r="C61" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D61" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="E61" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="F61" t="s">
         <v>170</v>
       </c>
       <c r="G61" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="H61">
         <v>3</v>
@@ -5444,33 +5529,33 @@
         <v>35</v>
       </c>
       <c r="M61" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="N61" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
     </row>
     <row r="62" spans="1:14">
       <c r="A62" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B62" t="s">
         <v>287</v>
       </c>
       <c r="C62" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D62" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="E62" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="F62" t="s">
         <v>170</v>
       </c>
       <c r="G62" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="H62">
         <v>2</v>
@@ -5488,27 +5573,27 @@
         <v>35</v>
       </c>
       <c r="M62" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="N62" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="63" spans="1:14">
       <c r="A63" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B63" t="s">
         <v>287</v>
       </c>
       <c r="C63" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="D63" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="E63" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="F63" t="s">
         <v>170</v>
@@ -5532,33 +5617,33 @@
         <v>35</v>
       </c>
       <c r="M63" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="N63" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
     </row>
     <row r="64" spans="1:14">
       <c r="A64" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B64" t="s">
         <v>287</v>
       </c>
       <c r="C64" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="D64" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="E64" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F64" t="s">
         <v>170</v>
       </c>
       <c r="G64" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H64">
         <v>2</v>
@@ -5576,33 +5661,33 @@
         <v>35</v>
       </c>
       <c r="M64" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="N64" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="65" spans="1:14">
       <c r="A65" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B65" t="s">
         <v>287</v>
       </c>
       <c r="C65" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="D65" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E65" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="F65" t="s">
         <v>170</v>
       </c>
       <c r="G65" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="H65">
         <v>2</v>
@@ -5620,33 +5705,33 @@
         <v>35</v>
       </c>
       <c r="M65" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="N65" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="66" spans="1:14">
       <c r="A66" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B66" t="s">
         <v>287</v>
       </c>
       <c r="C66" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="D66" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E66" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="F66" t="s">
         <v>170</v>
       </c>
       <c r="G66" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="H66">
         <v>3</v>
@@ -5664,33 +5749,33 @@
         <v>35</v>
       </c>
       <c r="M66" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="N66" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="67" spans="1:14">
       <c r="A67" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B67" t="s">
         <v>287</v>
       </c>
       <c r="C67" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="D67" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="E67" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="F67" t="s">
         <v>170</v>
       </c>
       <c r="G67" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="H67">
         <v>2</v>
@@ -5708,27 +5793,27 @@
         <v>35</v>
       </c>
       <c r="M67" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="N67" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
     <row r="68" spans="1:14">
       <c r="A68" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B68" t="s">
         <v>287</v>
       </c>
       <c r="C68" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="D68" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="E68" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="F68" t="s">
         <v>170</v>
@@ -5752,33 +5837,33 @@
         <v>35</v>
       </c>
       <c r="M68" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="N68" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
     </row>
     <row r="69" spans="1:14">
       <c r="A69" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B69" t="s">
         <v>287</v>
       </c>
       <c r="C69" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="D69" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="E69" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="F69" t="s">
         <v>170</v>
       </c>
       <c r="G69" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H69">
         <v>2</v>
@@ -5796,33 +5881,33 @@
         <v>35</v>
       </c>
       <c r="M69" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="N69" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
     </row>
     <row r="70" spans="1:14">
       <c r="A70" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="B70" t="s">
         <v>287</v>
       </c>
       <c r="C70" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="D70" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="E70" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="F70" t="s">
         <v>170</v>
       </c>
       <c r="G70" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="H70">
         <v>2</v>
@@ -5840,33 +5925,33 @@
         <v>35</v>
       </c>
       <c r="M70" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="N70" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
     </row>
     <row r="71" spans="1:14">
       <c r="A71" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B71" t="s">
         <v>287</v>
       </c>
       <c r="C71" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="D71" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="E71" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F71" t="s">
         <v>170</v>
       </c>
       <c r="G71" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="H71">
         <v>3</v>
@@ -5884,33 +5969,33 @@
         <v>35</v>
       </c>
       <c r="M71" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="N71" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
     </row>
     <row r="72" spans="1:14">
       <c r="A72" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B72" t="s">
         <v>287</v>
       </c>
       <c r="C72" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="D72" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="E72" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="F72" t="s">
         <v>170</v>
       </c>
       <c r="G72" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="H72">
         <v>2</v>
@@ -5928,27 +6013,27 @@
         <v>35</v>
       </c>
       <c r="M72" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="N72" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
     </row>
     <row r="73" spans="1:14">
       <c r="A73" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="B73" t="s">
         <v>287</v>
       </c>
       <c r="C73" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="D73" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="E73" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="F73" t="s">
         <v>170</v>
@@ -5972,33 +6057,33 @@
         <v>35</v>
       </c>
       <c r="M73" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="N73" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
     </row>
     <row r="74" spans="1:14">
       <c r="A74" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B74" t="s">
         <v>287</v>
       </c>
       <c r="C74" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="D74" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="E74" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="F74" t="s">
         <v>170</v>
       </c>
       <c r="G74" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H74">
         <v>2</v>
@@ -6016,33 +6101,33 @@
         <v>35</v>
       </c>
       <c r="M74" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="N74" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
     </row>
     <row r="75" spans="1:14">
       <c r="A75" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="B75" t="s">
         <v>287</v>
       </c>
       <c r="C75" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="D75" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="E75" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="F75" t="s">
         <v>170</v>
       </c>
       <c r="G75" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="H75">
         <v>2</v>
@@ -6051,7 +6136,7 @@
         <v>21</v>
       </c>
       <c r="J75" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="K75" t="s">
         <v>247</v>
@@ -6060,33 +6145,33 @@
         <v>35</v>
       </c>
       <c r="M75" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="N75" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
     </row>
     <row r="76" spans="1:14">
       <c r="A76" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B76" t="s">
         <v>287</v>
       </c>
       <c r="C76" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="D76" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="E76" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F76" t="s">
         <v>170</v>
       </c>
       <c r="G76" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="H76">
         <v>3</v>
@@ -6104,33 +6189,33 @@
         <v>35</v>
       </c>
       <c r="M76" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="N76" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
     </row>
     <row r="77" spans="1:14">
       <c r="A77" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B77" t="s">
         <v>287</v>
       </c>
       <c r="C77" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="D77" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="E77" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="F77" t="s">
         <v>170</v>
       </c>
       <c r="G77" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="H77">
         <v>2</v>
@@ -6148,27 +6233,27 @@
         <v>35</v>
       </c>
       <c r="M77" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="N77" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
     </row>
     <row r="78" spans="1:14">
       <c r="A78" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="B78" t="s">
         <v>287</v>
       </c>
       <c r="C78" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="D78" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="E78" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="F78" t="s">
         <v>170</v>
@@ -6192,33 +6277,33 @@
         <v>35</v>
       </c>
       <c r="M78" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="N78" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="79" spans="1:14">
       <c r="A79" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B79" t="s">
         <v>287</v>
       </c>
       <c r="C79" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="D79" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="E79" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="F79" t="s">
         <v>170</v>
       </c>
       <c r="G79" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H79">
         <v>2</v>
@@ -6236,33 +6321,205 @@
         <v>35</v>
       </c>
       <c r="M79" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="N79" t="s">
-        <v>534</v>
+        <v>535</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14">
+      <c r="A80" t="s">
+        <v>536</v>
+      </c>
+      <c r="B80" t="s">
+        <v>537</v>
+      </c>
+      <c r="C80" t="s">
+        <v>538</v>
+      </c>
+      <c r="D80" t="s">
+        <v>539</v>
+      </c>
+      <c r="E80" t="s">
+        <v>540</v>
+      </c>
+      <c r="F80" t="s">
+        <v>42</v>
+      </c>
+      <c r="G80" t="s">
+        <v>541</v>
+      </c>
+      <c r="H80">
+        <v>3</v>
+      </c>
+      <c r="I80" t="s">
+        <v>32</v>
+      </c>
+      <c r="J80" t="s">
+        <v>44</v>
+      </c>
+      <c r="L80" t="s">
+        <v>23</v>
+      </c>
+      <c r="M80" t="s">
+        <v>299</v>
+      </c>
+      <c r="N80" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14">
+      <c r="A81" t="s">
+        <v>543</v>
+      </c>
+      <c r="B81" t="s">
+        <v>544</v>
+      </c>
+      <c r="C81" t="s">
+        <v>545</v>
+      </c>
+      <c r="D81" t="s">
+        <v>546</v>
+      </c>
+      <c r="E81" t="s">
+        <v>547</v>
+      </c>
+      <c r="F81" t="s">
+        <v>42</v>
+      </c>
+      <c r="G81" t="s">
+        <v>541</v>
+      </c>
+      <c r="H81">
+        <v>3</v>
+      </c>
+      <c r="I81" t="s">
+        <v>32</v>
+      </c>
+      <c r="J81" t="s">
+        <v>150</v>
+      </c>
+      <c r="L81" t="s">
+        <v>23</v>
+      </c>
+      <c r="M81" t="s">
+        <v>536</v>
+      </c>
+      <c r="N81" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14">
+      <c r="A82" t="s">
+        <v>549</v>
+      </c>
+      <c r="B82" t="s">
+        <v>287</v>
+      </c>
+      <c r="C82" t="s">
+        <v>550</v>
+      </c>
+      <c r="D82" t="s">
+        <v>551</v>
+      </c>
+      <c r="E82" t="s">
+        <v>552</v>
+      </c>
+      <c r="F82" t="s">
+        <v>42</v>
+      </c>
+      <c r="G82" t="s">
+        <v>553</v>
+      </c>
+      <c r="H82">
+        <v>2</v>
+      </c>
+      <c r="I82" t="s">
+        <v>32</v>
+      </c>
+      <c r="J82" t="s">
+        <v>150</v>
+      </c>
+      <c r="L82" t="s">
+        <v>23</v>
+      </c>
+      <c r="M82" t="s">
+        <v>554</v>
+      </c>
+      <c r="N82" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14">
+      <c r="A83" t="s">
+        <v>556</v>
+      </c>
+      <c r="B83" t="s">
+        <v>287</v>
+      </c>
+      <c r="C83" t="s">
+        <v>557</v>
+      </c>
+      <c r="D83" t="s">
+        <v>558</v>
+      </c>
+      <c r="E83" t="s">
+        <v>559</v>
+      </c>
+      <c r="F83" t="s">
+        <v>42</v>
+      </c>
+      <c r="G83" t="s">
+        <v>560</v>
+      </c>
+      <c r="H83">
+        <v>1</v>
+      </c>
+      <c r="I83" t="s">
+        <v>32</v>
+      </c>
+      <c r="J83" t="s">
+        <v>44</v>
+      </c>
+      <c r="L83" t="s">
+        <v>23</v>
+      </c>
+      <c r="M83" t="s">
+        <v>536</v>
+      </c>
+      <c r="N83" t="s">
+        <v>561</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:N79" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:N87" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
+  <sortState ref="A2:N84">
+    <sortCondition ref="A2"/>
+  </sortState>
   <conditionalFormatting sqref="L$1:L$1048576">
-    <cfRule type="containsText" dxfId="0" priority="4" operator="between" text="Planned">
-      <formula>NOT(ISERROR(SEARCH("Planned",L1)))</formula>
+    <cfRule type="containsText" dxfId="0" priority="1" operator="between" text="In-Review">
+      <formula>NOT(ISERROR(SEARCH("In-Review",L1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="3" operator="between" text="Deferred">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L1:L84 L87:L1048576">
+    <cfRule type="containsText" dxfId="1" priority="2" operator="between" text="In-Progress">
+      <formula>NOT(ISERROR(SEARCH("In-Progress",L1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="3" operator="between" text="Completed">
+      <formula>NOT(ISERROR(SEARCH("Completed",L1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="4" operator="between" text="Deferred">
       <formula>NOT(ISERROR(SEARCH("Deferred",L1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="2" operator="between" text="Completed">
-      <formula>NOT(ISERROR(SEARCH("Completed",L1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="1" operator="between" text="In-Progress">
-      <formula>NOT(ISERROR(SEARCH("In-Progress",L1)))</formula>
+    <cfRule type="containsText" dxfId="4" priority="5" operator="between" text="Planned">
+      <formula>NOT(ISERROR(SEARCH("Planned",L1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L$1:L$1048576">
-      <formula1>"Planned,Deferred,In-Progress,Completed"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L1:L84 L87:L1048576">
+      <formula1>"Planned,Deferred,In-Progress,Completed,Draft"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
unwanted artifact clean up
</commit_message>
<xml_diff>
--- a/backlog/backlog.xlsx
+++ b/backlog/backlog.xlsx
@@ -4989,7 +4989,6 @@
       <c r="J32" t="s">
         <v>44</v>
       </c>
-      <c r="K32"/>
       <c r="L32" t="s">
         <v>247</v>
       </c>
@@ -5031,7 +5030,6 @@
       <c r="J33" t="s">
         <v>44</v>
       </c>
-      <c r="K33"/>
       <c r="L33" t="s">
         <v>45</v>
       </c>
@@ -5073,7 +5071,6 @@
       <c r="J34" t="s">
         <v>44</v>
       </c>
-      <c r="K34"/>
       <c r="L34" t="s">
         <v>45</v>
       </c>
@@ -5115,7 +5112,6 @@
       <c r="J35" t="s">
         <v>44</v>
       </c>
-      <c r="K35"/>
       <c r="L35" t="s">
         <v>35</v>
       </c>
@@ -5157,7 +5153,6 @@
       <c r="J36" t="s">
         <v>33</v>
       </c>
-      <c r="K36"/>
       <c r="L36" t="s">
         <v>45</v>
       </c>
@@ -5199,7 +5194,6 @@
       <c r="J37" t="s">
         <v>172</v>
       </c>
-      <c r="K37"/>
       <c r="L37" t="s">
         <v>35</v>
       </c>
@@ -5241,7 +5235,6 @@
       <c r="J38" t="s">
         <v>172</v>
       </c>
-      <c r="K38"/>
       <c r="L38" t="s">
         <v>35</v>
       </c>
@@ -5283,7 +5276,6 @@
       <c r="J39" t="s">
         <v>33</v>
       </c>
-      <c r="K39"/>
       <c r="L39" t="s">
         <v>35</v>
       </c>
@@ -5721,7 +5713,6 @@
       <c r="J49" t="s">
         <v>121</v>
       </c>
-      <c r="K49"/>
       <c r="L49" t="s">
         <v>45</v>
       </c>
@@ -5776,7 +5767,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="51" spans="1:14">
+    <row r="51" hidden="1" spans="1:14">
       <c r="A51" t="s">
         <v>359</v>
       </c>
@@ -5864,7 +5855,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="53" spans="1:14">
+    <row r="53" hidden="1" spans="1:14">
       <c r="A53" t="s">
         <v>372</v>
       </c>
@@ -5908,7 +5899,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="54" spans="1:14">
+    <row r="54" hidden="1" spans="1:14">
       <c r="A54" t="s">
         <v>378</v>
       </c>
@@ -5952,7 +5943,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="55" spans="1:14">
+    <row r="55" hidden="1" spans="1:14">
       <c r="A55" t="s">
         <v>384</v>
       </c>
@@ -6159,7 +6150,6 @@
       <c r="J59" t="s">
         <v>121</v>
       </c>
-      <c r="K59"/>
       <c r="L59" t="s">
         <v>35</v>
       </c>
@@ -6377,7 +6367,6 @@
       <c r="J64" t="s">
         <v>121</v>
       </c>
-      <c r="K64"/>
       <c r="L64" t="s">
         <v>45</v>
       </c>
@@ -6388,7 +6377,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="65" spans="1:14">
+    <row r="65" hidden="1" spans="1:14">
       <c r="A65" t="s">
         <v>447</v>
       </c>
@@ -6432,7 +6421,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="66" spans="1:14">
+    <row r="66" hidden="1" spans="1:14">
       <c r="A66" t="s">
         <v>453</v>
       </c>
@@ -6520,7 +6509,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="68" spans="1:14">
+    <row r="68" hidden="1" spans="1:14">
       <c r="A68" t="s">
         <v>465</v>
       </c>
@@ -6595,7 +6584,6 @@
       <c r="J69" t="s">
         <v>121</v>
       </c>
-      <c r="K69"/>
       <c r="L69" t="s">
         <v>35</v>
       </c>
@@ -6606,7 +6594,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="70" spans="1:14">
+    <row r="70" hidden="1" spans="1:14">
       <c r="A70" t="s">
         <v>477</v>
       </c>
@@ -6650,7 +6638,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="71" spans="1:14">
+    <row r="71" hidden="1" spans="1:14">
       <c r="A71" t="s">
         <v>483</v>
       </c>
@@ -6738,7 +6726,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="73" spans="1:14">
+    <row r="73" hidden="1" spans="1:14">
       <c r="A73" t="s">
         <v>496</v>
       </c>
@@ -6813,7 +6801,6 @@
       <c r="J74" t="s">
         <v>121</v>
       </c>
-      <c r="K74"/>
       <c r="L74" t="s">
         <v>35</v>
       </c>
@@ -6824,7 +6811,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="75" spans="1:14">
+    <row r="75" hidden="1" spans="1:14">
       <c r="A75" t="s">
         <v>508</v>
       </c>
@@ -6868,7 +6855,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="76" spans="1:14">
+    <row r="76" hidden="1" spans="1:14">
       <c r="A76" t="s">
         <v>515</v>
       </c>
@@ -6987,7 +6974,6 @@
       <c r="J78" t="s">
         <v>95</v>
       </c>
-      <c r="K78"/>
       <c r="L78" t="s">
         <v>35</v>
       </c>
@@ -7029,7 +7015,6 @@
       <c r="J79" t="s">
         <v>121</v>
       </c>
-      <c r="K79"/>
       <c r="L79" t="s">
         <v>35</v>
       </c>
@@ -7216,7 +7201,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="84" spans="1:14">
+    <row r="84" hidden="1" spans="1:14">
       <c r="A84" t="s">
         <v>566</v>
       </c>
@@ -7260,7 +7245,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="85" spans="1:14">
+    <row r="85" hidden="1" spans="1:14">
       <c r="A85" t="s">
         <v>574</v>
       </c>
@@ -7304,7 +7289,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="86" spans="1:14">
+    <row r="86" hidden="1" spans="1:14">
       <c r="A86" t="s">
         <v>580</v>
       </c>
@@ -7348,7 +7333,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="87" spans="1:14">
+    <row r="87" hidden="1" spans="1:14">
       <c r="A87" t="s">
         <v>586</v>
       </c>
@@ -7392,7 +7377,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="88" spans="1:14">
+    <row r="88" hidden="1" spans="1:14">
       <c r="A88" t="s">
         <v>593</v>
       </c>
@@ -7436,7 +7421,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="89" spans="1:14">
+    <row r="89" hidden="1" spans="1:14">
       <c r="A89" t="s">
         <v>599</v>
       </c>
@@ -7568,7 +7553,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="92" spans="1:14">
+    <row r="92" hidden="1" spans="1:14">
       <c r="A92" t="s">
         <v>619</v>
       </c>
@@ -7612,7 +7597,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="93" spans="1:14">
+    <row r="93" hidden="1" spans="1:14">
       <c r="A93" t="s">
         <v>626</v>
       </c>
@@ -7647,7 +7632,7 @@
         <v>363</v>
       </c>
       <c r="L93" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M93" t="s">
         <v>24</v>
@@ -7656,7 +7641,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="94" spans="1:14">
+    <row r="94" hidden="1" spans="1:14">
       <c r="A94" t="s">
         <v>633</v>
       </c>
@@ -7691,7 +7676,7 @@
         <v>363</v>
       </c>
       <c r="L94" t="s">
-        <v>35</v>
+        <v>293</v>
       </c>
       <c r="M94" t="s">
         <v>24</v>
@@ -7744,7 +7729,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="96" spans="1:14">
+    <row r="96" hidden="1" spans="1:14">
       <c r="A96" t="s">
         <v>646</v>
       </c>
@@ -7788,7 +7773,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="97" spans="1:14">
+    <row r="97" hidden="1" spans="1:14">
       <c r="A97" t="s">
         <v>652</v>
       </c>
@@ -7832,7 +7817,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="98" spans="1:14">
+    <row r="98" hidden="1" spans="1:14">
       <c r="A98" t="s">
         <v>658</v>
       </c>
@@ -7876,7 +7861,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="99" spans="1:14">
+    <row r="99" hidden="1" spans="1:14">
       <c r="A99" t="s">
         <v>665</v>
       </c>
@@ -7920,7 +7905,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="100" spans="1:14">
+    <row r="100" hidden="1" spans="1:14">
       <c r="A100" t="s">
         <v>672</v>
       </c>
@@ -7964,7 +7949,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="101" spans="1:14">
+    <row r="101" hidden="1" spans="1:14">
       <c r="A101" t="s">
         <v>679</v>
       </c>
@@ -8008,7 +7993,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="102" spans="1:14">
+    <row r="102" hidden="1" spans="1:14">
       <c r="A102" t="s">
         <v>686</v>
       </c>
@@ -8052,7 +8037,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="103" spans="1:14">
+    <row r="103" hidden="1" spans="1:14">
       <c r="A103" t="s">
         <v>693</v>
       </c>
@@ -8096,7 +8081,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="104" spans="1:14">
+    <row r="104" hidden="1" spans="1:14">
       <c r="A104" t="s">
         <v>700</v>
       </c>
@@ -8140,7 +8125,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="105" spans="1:14">
+    <row r="105" hidden="1" spans="1:14">
       <c r="A105" t="s">
         <v>707</v>
       </c>
@@ -8184,7 +8169,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="106" spans="1:14">
+    <row r="106" hidden="1" spans="1:14">
       <c r="A106" t="s">
         <v>713</v>
       </c>
@@ -8228,7 +8213,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="107" spans="1:14">
+    <row r="107" hidden="1" spans="1:14">
       <c r="A107" t="s">
         <v>719</v>
       </c>
@@ -8272,7 +8257,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="108" spans="1:14">
+    <row r="108" hidden="1" spans="1:14">
       <c r="A108" t="s">
         <v>726</v>
       </c>
@@ -8316,7 +8301,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="109" spans="1:14">
+    <row r="109" hidden="1" spans="1:14">
       <c r="A109" t="s">
         <v>733</v>
       </c>
@@ -8360,7 +8345,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="110" spans="1:14">
+    <row r="110" hidden="1" spans="1:14">
       <c r="A110" t="s">
         <v>740</v>
       </c>
@@ -8404,7 +8389,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="111" spans="1:14">
+    <row r="111" hidden="1" spans="1:14">
       <c r="A111" t="s">
         <v>747</v>
       </c>
@@ -8448,7 +8433,7 @@
         <v>752</v>
       </c>
     </row>
-    <row r="112" spans="1:14">
+    <row r="112" hidden="1" spans="1:14">
       <c r="A112" t="s">
         <v>753</v>
       </c>
@@ -8659,7 +8644,7 @@
         <v>363</v>
       </c>
       <c r="L116" t="s">
-        <v>35</v>
+        <v>293</v>
       </c>
       <c r="M116" t="s">
         <v>626</v>
@@ -8703,7 +8688,7 @@
         <v>363</v>
       </c>
       <c r="L117" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M117" t="s">
         <v>791</v>
@@ -8712,7 +8697,7 @@
         <v>792</v>
       </c>
     </row>
-    <row r="118" spans="1:14">
+    <row r="118" hidden="1" spans="1:14">
       <c r="A118" t="s">
         <v>793</v>
       </c>
@@ -8756,7 +8741,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="119" spans="1:14">
+    <row r="119" hidden="1" spans="1:14">
       <c r="A119" t="s">
         <v>799</v>
       </c>
@@ -8802,10 +8787,10 @@
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:N119" etc:filterBottomFollowUsedRange="0">
-    <filterColumn colId="10">
-      <filters>
-        <filter val="Sprint 2"/>
-      </filters>
+    <filterColumn colId="12">
+      <customFilters>
+        <customFilter operator="equal" val="*PBI-092*"/>
+      </customFilters>
     </filterColumn>
     <extLst/>
   </autoFilter>
@@ -8833,7 +8818,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L1:L77 L78:L119 L120:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L$1:L$1048576">
       <formula1>"Planned,Deferred,In-Progress,Completed,Draft,Blocked"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
[PBI-053] Add role-assignment test evidence and closeout note
</commit_message>
<xml_diff>
--- a/backlog/backlog.xlsx
+++ b/backlog/backlog.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="10668" windowHeight="9396"/>
+    <workbookView windowWidth="22188" windowHeight="9384"/>
   </bookViews>
   <sheets>
     <sheet name="backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">backlog!$A$1:$N$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">backlog!$A$1:$N$121</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1513" uniqueCount="806">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1527" uniqueCount="814">
   <si>
     <t>PBI-###</t>
   </si>
@@ -773,186 +773,186 @@
     <t>Security;Compliance;Maintainability</t>
   </si>
   <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Important: Story-level acceptance should not be marked Accepted/Done until PBI-083 is resolved and duplicate-prevention behavior is verified.</t>
+  </si>
+  <si>
+    <t>PBI-032</t>
+  </si>
+  <si>
+    <t>As an administrator, I want to define and maintain platform roles, so that access can be governed consistently</t>
+  </si>
+  <si>
+    <t>Context: role-based access requires a stable role catalogue before user assignment. Business problem: inconsistent role definitions weaken access governance. User role / actor: administrator. Expected behavior: administrator can create, update, and manage platform roles used for membership access control. Business value: establishes a reusable role model for secure access management. In scope: role creation, role update, role status management. Out of scope: user-role assignment and runtime access denial.</t>
+  </si>
+  <si>
+    <t>[ReqID: R03] Given an administrator defines a valid role, when the role is saved, then the platform stores the role for future assignment. | [ReqID: R03] Given a duplicate or invalid role definition is submitted, when save is attempted, then the platform rejects the change and returns a validation error.</t>
+  </si>
+  <si>
+    <t>DoR: Ready. PO Approval: Approved for Sprint 1 decomposition of PBI-003.</t>
+  </si>
+  <si>
+    <t>PBI-033</t>
+  </si>
+  <si>
+    <t>As an administrator, I want to assign platform roles to member users, so that each user can access only the functions required for their responsibilities</t>
+  </si>
+  <si>
+    <t>Context: once organizations and roles exist, users must be bound to those roles to support controlled access. Business problem: users without structured role assignment cannot be governed consistently. User role / actor: administrator. Expected behavior: administrator assigns, changes, or removes roles for users associated with member organizations. Business value: enables least-privilege access control. In scope: assign role, change role, remove role, membership validation. Out of scope: deactivation enforcement.</t>
+  </si>
+  <si>
+    <t>[ReqID: R03] Given a user belongs to a valid member organization and a valid role exists, when an administrator assigns the role, then the platform stores the assignment successfully. | [ReqID: R03] Given the user is not associated with a valid member organization or the role is invalid, when assignment is attempted, then the platform blocks the assignment and shows the reason.</t>
+  </si>
+  <si>
+    <t>PBI-003;PBI-031;PBI-032</t>
+  </si>
+  <si>
+    <t>PBI-034</t>
+  </si>
+  <si>
+    <t>As the platform, I want to block access for deactivated members, so that removed organizations and users cannot use protected functions</t>
+  </si>
+  <si>
+    <t>Context: membership and role management are incomplete without enforcement against deactivated members. Business problem: inactive members retaining access creates governance and security risk. User role / actor: system enforcement. Expected behavior: protected actions are denied when a member organization or user is deactivated. Business value: ensures access control reflects membership state. In scope: deactivation state check, denial of protected actions, error feedback. Out of scope: advanced non-repudiation analytics.</t>
+  </si>
+  <si>
+    <t>[ReqID: R03] Given a member organization or user is deactivated, when a protected action is attempted, then the platform denies access. | [ReqID: R03] Given an active member with a valid role attempts a protected action, when access is evaluated, then the platform allows the action to proceed.</t>
+  </si>
+  <si>
+    <t>Security;Compliance;Reliability</t>
+  </si>
+  <si>
+    <t>PBI-003;PBI-031;PBI-033</t>
+  </si>
+  <si>
+    <t>PBI-035</t>
+  </si>
+  <si>
+    <t>As a compliance coordinator, I want to submit a PLS item for Shariah review, so that governance starts from a formal and traceable request</t>
+  </si>
+  <si>
+    <t>Context: Shariah governance requires a formal starting point for review. Business problem: ad hoc review initiation makes approval workflow ambiguous and difficult to track. User role / actor: compliance coordinator. Expected behavior: coordinator submits a review request with the mandatory metadata for a PLS item. Business value: creates a controlled and traceable approval intake process. In scope: request creation, mandatory fields, initial workflow state. Out of scope: checklist completion and final decision.</t>
+  </si>
+  <si>
+    <t>[ReqID: R20] Given the required review-request data is complete, when the coordinator submits the request, then the platform creates a review record with initial Submitted status. | [ReqID: R20] Given mandatory review-request data is incomplete, when submission is attempted, then the platform blocks the request and shows validation errors.</t>
+  </si>
+  <si>
+    <t>Compliance;Audit;Security</t>
+  </si>
+  <si>
+    <t>DoR: Ready. PO Approval: Approved for Sprint 1 decomposition of PBI-020.</t>
+  </si>
+  <si>
+    <t>PBI-036</t>
+  </si>
+  <si>
+    <t>As a Shariah reviewer, I want to record the review checklist outcome, so that the basis of the governance decision is documented</t>
+  </si>
+  <si>
+    <t>Context: governance decisions require structured review evidence before approval can be finalized. Business problem: undocumented checklist completion weakens governance assurance. User role / actor: Shariah reviewer. Expected behavior: reviewer completes and saves the checklist findings for a submitted review item. Business value: makes the approval basis explicit and auditable. In scope: checklist completion, reviewer comments, review completion state. Out of scope: final approve reject conditional-approve transition.</t>
+  </si>
+  <si>
+    <t>[ReqID: R20] Given a submitted review item exists, when the reviewer completes the checklist with all required entries, then the platform stores the checklist outcome and reviewer comments. | [ReqID: R20] Given mandatory checklist entries are missing, when the reviewer attempts to save completion, then the platform blocks completion and shows validation errors.</t>
+  </si>
+  <si>
+    <t>PBI-020;PBI-035</t>
+  </si>
+  <si>
+    <t>PBI-037</t>
+  </si>
+  <si>
+    <t>As a Shariah reviewer, I want to record approve, reject, or conditional-approve decisions, so that governance outcomes are explicit and auditable</t>
+  </si>
+  <si>
+    <t>Context: the review workflow must end in a formal governance outcome. Business problem: without explicit decision capture, approval status cannot be relied upon. User role / actor: Shariah reviewer. Expected behavior: reviewer records the final decision with rationale or conditions where applicable. Business value: enables clear governance outcomes and later compliance verification. In scope: approve, reject, conditional approve, rationale capture, state transition. Out of scope: activation gating against PLS contract execution.</t>
+  </si>
+  <si>
+    <t>[ReqID: R20] Given a completed review checklist exists, when the reviewer records an approval decision, then the platform changes the item status to Approved and stores the decision metadata. | [ReqID: R20] Given the reviewer records a rejection or conditional approval, when the decision is saved, then the platform stores the rationale or conditions and updates the workflow state accordingly.</t>
+  </si>
+  <si>
+    <t>PBI-020;PBI-036</t>
+  </si>
+  <si>
+    <t>PBI-038</t>
+  </si>
+  <si>
+    <t>As a compliance coordinator, I want to view the current approval status and decision history, so that I can track governance progress and outcomes</t>
+  </si>
+  <si>
+    <t>Context: governance workflow participants need visibility into approval progress and results. Business problem: without a consolidated view, coordinators cannot follow up or confirm outcome state efficiently. User role / actor: compliance coordinator. Expected behavior: coordinator can view the latest status and prior review history of a PLS review item. Business value: improves workflow transparency and operational follow-up. In scope: status view, decision history, summary of review progression. Out of scope: regulator export and linkage to downstream contract execution.</t>
+  </si>
+  <si>
+    <t>[ReqID: R20] Given a review item exists, when the coordinator opens its details, then the platform displays the current approval status and prior review history. | [ReqID: R20] Given no final decision has been recorded yet, when the coordinator views the item, then the platform still shows the submitted and review-progress states without error.</t>
+  </si>
+  <si>
+    <t>Compliance;Audit;Usability;Security</t>
+  </si>
+  <si>
+    <t>PBI-020;PBI-035;PBI-037</t>
+  </si>
+  <si>
+    <t>PBI-039</t>
+  </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>Do define member organization schema, uniqueness rules, and membership status model</t>
+  </si>
+  <si>
+    <t>Action to be performed: define the member organization data model, required fields, uniqueness rules, and active or inactive lifecycle states. Why it is needed: downstream API, UI, and access-control tasks depend on stable data and state rules. Expected output: reviewed schema, validation rules, and request-response contract. Scope: entity fields, uniqueness rule, state values, API contract. Explicit exclusions: UI build and endpoint implementation.</t>
+  </si>
+  <si>
+    <t>[ReqID: R03] Given the schema draft is reviewed, when validation rules are checked, then required fields, uniqueness constraints, and status values are explicitly defined. | [ReqID: R03] Given downstream tasks consume the model, when implementation starts, then the request and response contract is stable enough for API and UI work.</t>
+  </si>
+  <si>
+    <t>Sprint 1</t>
+  </si>
+  <si>
+    <t>Important: Covers PBI-031 AC1 and AC2. Shared prerequisite for PBI-040 and PBI-041. Evidence: schema note, validation matrix, API contract.</t>
+  </si>
+  <si>
+    <t>PBI-040</t>
+  </si>
+  <si>
+    <t>Do implement member organization creation API and service validation</t>
+  </si>
+  <si>
+    <t>Action to be performed: build the backend endpoint and service logic for member organization creation with required validation and duplicate checks. Why it is needed: the story requires creation of unique active member organizations. Expected output: working create service with persistence and validation behavior. Scope: endpoint, service logic, required-field validation, duplicate prevention, persistence. Explicit exclusions: admin screen implementation.</t>
+  </si>
+  <si>
+    <t>[ReqID: R03] Given valid organization input is submitted, when the create service executes, then the organization is stored with a unique identifier and active status. | [ReqID: R03] Given missing or duplicate data is submitted, when validation runs, then the service rejects the request with the correct error response.</t>
+  </si>
+  <si>
+    <t>PBI-031;PBI-039</t>
+  </si>
+  <si>
+    <t>Important: Delivered slice completed current backend create flow, but duplicate-prevention remains incomplete in the implementation path and is now tracked explicitly by PBI-083.</t>
+  </si>
+  <si>
+    <t>PBI-041</t>
+  </si>
+  <si>
+    <t>Do implement administrator registration UI and error feedback for member onboarding</t>
+  </si>
+  <si>
+    <t>Action to be performed: build the admin form and user feedback for member organization registration. Why it is needed: administrators need a usable interface to create organizations and handle invalid input. Expected output: working form with validation messages and success state. Scope: form fields, submit flow, validation feedback, success and error states. Explicit exclusions: backend authorization and audit logging.</t>
+  </si>
+  <si>
+    <t>[ReqID: R03] Given valid registration data is entered, when the administrator submits the form, then the UI sends the request and displays a success result aligned to the backend response. | [ReqID: R03] Given invalid or duplicate data is entered, when submission is attempted, then the UI displays meaningful validation or error feedback.</t>
+  </si>
+  <si>
+    <t>Usability;Security;Maintainability</t>
+  </si>
+  <si>
+    <t>Sprint 2 (Optional)</t>
+  </si>
+  <si>
     <t>Blocked</t>
   </si>
   <si>
-    <t>Important: Story-level acceptance should not be marked Accepted/Done until PBI-083 is resolved and duplicate-prevention behavior is verified.</t>
-  </si>
-  <si>
-    <t>PBI-032</t>
-  </si>
-  <si>
-    <t>As an administrator, I want to define and maintain platform roles, so that access can be governed consistently</t>
-  </si>
-  <si>
-    <t>Context: role-based access requires a stable role catalogue before user assignment. Business problem: inconsistent role definitions weaken access governance. User role / actor: administrator. Expected behavior: administrator can create, update, and manage platform roles used for membership access control. Business value: establishes a reusable role model for secure access management. In scope: role creation, role update, role status management. Out of scope: user-role assignment and runtime access denial.</t>
-  </si>
-  <si>
-    <t>[ReqID: R03] Given an administrator defines a valid role, when the role is saved, then the platform stores the role for future assignment. | [ReqID: R03] Given a duplicate or invalid role definition is submitted, when save is attempted, then the platform rejects the change and returns a validation error.</t>
-  </si>
-  <si>
-    <t>DoR: Ready. PO Approval: Approved for Sprint 1 decomposition of PBI-003.</t>
-  </si>
-  <si>
-    <t>PBI-033</t>
-  </si>
-  <si>
-    <t>As an administrator, I want to assign platform roles to member users, so that each user can access only the functions required for their responsibilities</t>
-  </si>
-  <si>
-    <t>Context: once organizations and roles exist, users must be bound to those roles to support controlled access. Business problem: users without structured role assignment cannot be governed consistently. User role / actor: administrator. Expected behavior: administrator assigns, changes, or removes roles for users associated with member organizations. Business value: enables least-privilege access control. In scope: assign role, change role, remove role, membership validation. Out of scope: deactivation enforcement.</t>
-  </si>
-  <si>
-    <t>[ReqID: R03] Given a user belongs to a valid member organization and a valid role exists, when an administrator assigns the role, then the platform stores the assignment successfully. | [ReqID: R03] Given the user is not associated with a valid member organization or the role is invalid, when assignment is attempted, then the platform blocks the assignment and shows the reason.</t>
-  </si>
-  <si>
-    <t>PBI-003;PBI-031;PBI-032</t>
-  </si>
-  <si>
-    <t>PBI-034</t>
-  </si>
-  <si>
-    <t>As the platform, I want to block access for deactivated members, so that removed organizations and users cannot use protected functions</t>
-  </si>
-  <si>
-    <t>Context: membership and role management are incomplete without enforcement against deactivated members. Business problem: inactive members retaining access creates governance and security risk. User role / actor: system enforcement. Expected behavior: protected actions are denied when a member organization or user is deactivated. Business value: ensures access control reflects membership state. In scope: deactivation state check, denial of protected actions, error feedback. Out of scope: advanced non-repudiation analytics.</t>
-  </si>
-  <si>
-    <t>[ReqID: R03] Given a member organization or user is deactivated, when a protected action is attempted, then the platform denies access. | [ReqID: R03] Given an active member with a valid role attempts a protected action, when access is evaluated, then the platform allows the action to proceed.</t>
-  </si>
-  <si>
-    <t>Security;Compliance;Reliability</t>
-  </si>
-  <si>
-    <t>PBI-003;PBI-031;PBI-033</t>
-  </si>
-  <si>
-    <t>PBI-035</t>
-  </si>
-  <si>
-    <t>As a compliance coordinator, I want to submit a PLS item for Shariah review, so that governance starts from a formal and traceable request</t>
-  </si>
-  <si>
-    <t>Context: Shariah governance requires a formal starting point for review. Business problem: ad hoc review initiation makes approval workflow ambiguous and difficult to track. User role / actor: compliance coordinator. Expected behavior: coordinator submits a review request with the mandatory metadata for a PLS item. Business value: creates a controlled and traceable approval intake process. In scope: request creation, mandatory fields, initial workflow state. Out of scope: checklist completion and final decision.</t>
-  </si>
-  <si>
-    <t>[ReqID: R20] Given the required review-request data is complete, when the coordinator submits the request, then the platform creates a review record with initial Submitted status. | [ReqID: R20] Given mandatory review-request data is incomplete, when submission is attempted, then the platform blocks the request and shows validation errors.</t>
-  </si>
-  <si>
-    <t>Compliance;Audit;Security</t>
-  </si>
-  <si>
-    <t>DoR: Ready. PO Approval: Approved for Sprint 1 decomposition of PBI-020.</t>
-  </si>
-  <si>
-    <t>PBI-036</t>
-  </si>
-  <si>
-    <t>As a Shariah reviewer, I want to record the review checklist outcome, so that the basis of the governance decision is documented</t>
-  </si>
-  <si>
-    <t>Context: governance decisions require structured review evidence before approval can be finalized. Business problem: undocumented checklist completion weakens governance assurance. User role / actor: Shariah reviewer. Expected behavior: reviewer completes and saves the checklist findings for a submitted review item. Business value: makes the approval basis explicit and auditable. In scope: checklist completion, reviewer comments, review completion state. Out of scope: final approve reject conditional-approve transition.</t>
-  </si>
-  <si>
-    <t>[ReqID: R20] Given a submitted review item exists, when the reviewer completes the checklist with all required entries, then the platform stores the checklist outcome and reviewer comments. | [ReqID: R20] Given mandatory checklist entries are missing, when the reviewer attempts to save completion, then the platform blocks completion and shows validation errors.</t>
-  </si>
-  <si>
-    <t>PBI-020;PBI-035</t>
-  </si>
-  <si>
-    <t>PBI-037</t>
-  </si>
-  <si>
-    <t>As a Shariah reviewer, I want to record approve, reject, or conditional-approve decisions, so that governance outcomes are explicit and auditable</t>
-  </si>
-  <si>
-    <t>Context: the review workflow must end in a formal governance outcome. Business problem: without explicit decision capture, approval status cannot be relied upon. User role / actor: Shariah reviewer. Expected behavior: reviewer records the final decision with rationale or conditions where applicable. Business value: enables clear governance outcomes and later compliance verification. In scope: approve, reject, conditional approve, rationale capture, state transition. Out of scope: activation gating against PLS contract execution.</t>
-  </si>
-  <si>
-    <t>[ReqID: R20] Given a completed review checklist exists, when the reviewer records an approval decision, then the platform changes the item status to Approved and stores the decision metadata. | [ReqID: R20] Given the reviewer records a rejection or conditional approval, when the decision is saved, then the platform stores the rationale or conditions and updates the workflow state accordingly.</t>
-  </si>
-  <si>
-    <t>PBI-020;PBI-036</t>
-  </si>
-  <si>
-    <t>PBI-038</t>
-  </si>
-  <si>
-    <t>As a compliance coordinator, I want to view the current approval status and decision history, so that I can track governance progress and outcomes</t>
-  </si>
-  <si>
-    <t>Context: governance workflow participants need visibility into approval progress and results. Business problem: without a consolidated view, coordinators cannot follow up or confirm outcome state efficiently. User role / actor: compliance coordinator. Expected behavior: coordinator can view the latest status and prior review history of a PLS review item. Business value: improves workflow transparency and operational follow-up. In scope: status view, decision history, summary of review progression. Out of scope: regulator export and linkage to downstream contract execution.</t>
-  </si>
-  <si>
-    <t>[ReqID: R20] Given a review item exists, when the coordinator opens its details, then the platform displays the current approval status and prior review history. | [ReqID: R20] Given no final decision has been recorded yet, when the coordinator views the item, then the platform still shows the submitted and review-progress states without error.</t>
-  </si>
-  <si>
-    <t>Compliance;Audit;Usability;Security</t>
-  </si>
-  <si>
-    <t>PBI-020;PBI-035;PBI-037</t>
-  </si>
-  <si>
-    <t>PBI-039</t>
-  </si>
-  <si>
-    <t>Task</t>
-  </si>
-  <si>
-    <t>Do define member organization schema, uniqueness rules, and membership status model</t>
-  </si>
-  <si>
-    <t>Action to be performed: define the member organization data model, required fields, uniqueness rules, and active or inactive lifecycle states. Why it is needed: downstream API, UI, and access-control tasks depend on stable data and state rules. Expected output: reviewed schema, validation rules, and request-response contract. Scope: entity fields, uniqueness rule, state values, API contract. Explicit exclusions: UI build and endpoint implementation.</t>
-  </si>
-  <si>
-    <t>[ReqID: R03] Given the schema draft is reviewed, when validation rules are checked, then required fields, uniqueness constraints, and status values are explicitly defined. | [ReqID: R03] Given downstream tasks consume the model, when implementation starts, then the request and response contract is stable enough for API and UI work.</t>
-  </si>
-  <si>
-    <t>Sprint 1</t>
-  </si>
-  <si>
-    <t>Completed</t>
-  </si>
-  <si>
-    <t>Important: Covers PBI-031 AC1 and AC2. Shared prerequisite for PBI-040 and PBI-041. Evidence: schema note, validation matrix, API contract.</t>
-  </si>
-  <si>
-    <t>PBI-040</t>
-  </si>
-  <si>
-    <t>Do implement member organization creation API and service validation</t>
-  </si>
-  <si>
-    <t>Action to be performed: build the backend endpoint and service logic for member organization creation with required validation and duplicate checks. Why it is needed: the story requires creation of unique active member organizations. Expected output: working create service with persistence and validation behavior. Scope: endpoint, service logic, required-field validation, duplicate prevention, persistence. Explicit exclusions: admin screen implementation.</t>
-  </si>
-  <si>
-    <t>[ReqID: R03] Given valid organization input is submitted, when the create service executes, then the organization is stored with a unique identifier and active status. | [ReqID: R03] Given missing or duplicate data is submitted, when validation runs, then the service rejects the request with the correct error response.</t>
-  </si>
-  <si>
-    <t>PBI-031;PBI-039</t>
-  </si>
-  <si>
-    <t>Important: Delivered slice completed current backend create flow, but duplicate-prevention remains incomplete in the implementation path and is now tracked explicitly by PBI-083.</t>
-  </si>
-  <si>
-    <t>PBI-041</t>
-  </si>
-  <si>
-    <t>Do implement administrator registration UI and error feedback for member onboarding</t>
-  </si>
-  <si>
-    <t>Action to be performed: build the admin form and user feedback for member organization registration. Why it is needed: administrators need a usable interface to create organizations and handle invalid input. Expected output: working form with validation messages and success state. Scope: form fields, submit flow, validation feedback, success and error states. Explicit exclusions: backend authorization and audit logging.</t>
-  </si>
-  <si>
-    <t>[ReqID: R03] Given valid registration data is entered, when the administrator submits the form, then the UI sends the request and displays a success result aligned to the backend response. | [ReqID: R03] Given invalid or duplicate data is entered, when submission is attempted, then the UI displays meaningful validation or error feedback.</t>
-  </si>
-  <si>
-    <t>Usability;Security;Maintainability</t>
-  </si>
-  <si>
-    <t>Sprint 2 (Optional)</t>
-  </si>
-  <si>
     <t>PBI-039;PBI-040;PBI-079;PBI-080;PBI-081;PBI-082;PBI-083</t>
   </si>
   <si>
@@ -1808,7 +1808,7 @@
     <t>Security;Audit;Architecture;Maintainability</t>
   </si>
   <si>
-    <t>Timebox: 2-3 calendar days. Important: resolves the current drift between implemented header-based actor handling and intended trusted actor context.</t>
+    <t>Important: Durable docs now state the intended baseline more explicitly: protected writes must use server-derived authenticated actor context and not client-authored identity input. This Spike should now focus on inventorying actual current route usage, confirming the trusted request-context boundary, and defining the migration path from any temporary header-based behavior.</t>
   </si>
   <si>
     <t>PBI-087</t>
@@ -1826,7 +1826,7 @@
     <t>Security;Audit;Integration;Maintainability</t>
   </si>
   <si>
-    <t>Important: executable follow-up to PBI-086. Evidence should include middleware or plugin tests and route-consumption examples.</t>
+    <t>Important: Durable docs now define the interim contract expectation clearly enough to implement this without re-debating public semantics. This item should execute against the documented server-derived actor baseline and produce the reusable request-context boundary that later Wave 4 tasks consume.</t>
   </si>
   <si>
     <t>PBI-088</t>
@@ -1844,7 +1844,7 @@
     <t>PBI-062;PBI-086;PBI-087</t>
   </si>
   <si>
-    <t>Important: closes the current authorization-semantics gap in the Shariah submission flow.</t>
+    <t>Important: Durable docs now already fix one major ambiguity: submitter identity is server-derived, not client-authored. This item should focus only on tightening permission semantics for who may submit, not on re-opening actor-source contract design.</t>
   </si>
   <si>
     <t>PBI-089</t>
@@ -1886,7 +1886,7 @@
     <t>Audit;Compliance;Architecture;Security</t>
   </si>
   <si>
-    <t>Timebox: 2-3 calendar days. Important: resolves inconsistent denied-action audit behavior before broader hardening.</t>
+    <t>Important: Durable docs now include an interim audit baseline, so this Spike no longer starts from a blank page. Its purpose is to settle denied-action coverage, event-catalog boundaries, and route-application consistency before broad route hardening continues.</t>
   </si>
   <si>
     <t>PBI-091</t>
@@ -1907,7 +1907,7 @@
     <t>PBI-086;PBI-087;PBI-090</t>
   </si>
   <si>
-    <t>Important: cross-cutting implementation item; should be applied deliberately rather than piecemeal by future stories.</t>
+    <t>Important: Durable docs now provide a minimum audit baseline and actor-source expectation. This item should implement uniform route behavior on top of that baseline rather than inventing per-route audit semantics during execution.</t>
   </si>
   <si>
     <t>PBI-092</t>
@@ -1955,7 +1955,7 @@
     <t>Do refresh durable context docs to match implemented backend behavior and approved temporary scaffolding</t>
   </si>
   <si>
-    <t>Action to be performed: update durable context docs so they reflect implemented backend behavior, explicit temporary scaffolding, and approved Sprint 2 architecture decisions. Why it is needed: current docs are useful but behind the code in actor identity, authorization semantics, audit behavior, and some sprint-execution assumptions. Expected output: updated API contracts, architecture notes, coding rules, sprint execution notes, and state-model text where applicable. Scope: documentation refresh for implemented backend behavior and approved temporary/final boundaries. Explicit exclusions: broad SDLC rewrite.</t>
+    <t>Action to be performed: update durable context docs so they reflect implemented backend behavior, explicit temporary scaffolding, and approved Sprint 2 architecture decisions. Why it is needed: current docs are useful but behind the code in actor identity, authorization semantics, audit behavior, and some sprint-execution assumptions. Expected output: updated API contracts, architecture notes, coding rules, sprint execution notes, and state-model text where applicable. Scope: documentation refresh for implemented backend behavior and approved temporary or final boundaries. Explicit exclusions: broad SDLC rewrite.</t>
   </si>
   <si>
     <t>[ReqID: R03;R20;R22] Given Sprint 2 architecture decisions are approved, when the durable docs are refreshed, then current backend behavior and temporary scaffolding are documented accurately. | [ReqID: R03;R20;R22] Given contributors plan future PBIs, when they read the durable docs, then they do not rely on stale assumptions for actor identity, authorization, audit, or review-submission behavior.</t>
@@ -1967,7 +1967,7 @@
     <t>PBI-086;PBI-090</t>
   </si>
   <si>
-    <t>Important: should capture both implemented behavior and clearly-labeled temporary scaffolding to reduce Sprint 2 planning drift.</t>
+    <t>Important: Wave 3.5 focused doc-hardening pass applied before Wave 4. Durable docs now explicitly capture server-derived actor context for protected writes, Shariah submission actor handling, interim audit baseline, and current protected-action assumptions. Keep this item open until repo review/acceptance confirms the docs are the active source of truth.</t>
   </si>
   <si>
     <t>PBI-095</t>
@@ -1994,7 +1994,7 @@
     <t>Do harden role-assignment creation authorization</t>
   </si>
   <si>
-    <t>Action to be performed: define and implement explicit authorization on the role-assignment creation route using the approved actor boundary and assignment-validation prerequisites. Why it is needed: assignment creation behavior exists, but governance over who may create assignments is underdefined relative to security expectations. Expected output: protected assignment-creation authorization, negative/positive tests, and docs alignment. Scope: assignment-create authorization rule, route/service enforcement, automated coverage, and note updates. Explicit exclusions: broader UI work and full deactivation implementation.</t>
+    <t>Action to be performed: define and implement explicit authorization on the role-assignment creation route using the approved actor boundary and assignment-validation prerequisites. Why it is needed: assignment creation behavior exists, but governance over who may create assignments is underdefined relative to security expectations. Expected output: protected assignment-creation authorization, negative and positive tests, and docs alignment. Scope: assignment-create authorization rule, route/service enforcement, automated coverage, and note updates. Explicit exclusions: broader UI work and full deactivation implementation.</t>
   </si>
   <si>
     <t>[ReqID: R03;R22] Given an actor lacks the approved permission to create assignments, when assignment creation is attempted, then the backend rejects the request with the correct forbidden response. | [ReqID: R03;R22] Given an actor satisfies the approved authorization rule and assignment validation passes, when creation is attempted, then the backend still creates the assignment successfully. | [ReqID: R03;R22] Given the authorization is hardened, when tests and docs are reviewed, then the protected route behavior is covered and aligned.</t>
@@ -2003,7 +2003,7 @@
     <t>PBI-086;PBI-087;PBI-084;PBI-085;PBI-050</t>
   </si>
   <si>
-    <t>Important: this is separate from completing PBI-050 business validation; it hardens who may perform assignment creation.</t>
+    <t>Important: Durable docs now clarify that trusted actor identity must be server-derived for protected actions. This item should therefore focus on assignment-create permission rules and backend enforcement, not on inventing temporary actor semantics.</t>
   </si>
   <si>
     <t>PBI-097</t>
@@ -2150,7 +2150,7 @@
     <t>PBI-085;PBI-102;PBI-050</t>
   </si>
   <si>
-    <t>Important: this task resumes the blocked acceptance criteria of PBI-050. Evidence: service tests for invalid-user and non-member paths.</t>
+    <t>Important: this task resumes the blocked acceptance criteria of PBI-050. Evidence: service tests for invalid-user and non-member paths. Status: service-level validation slice complete, task not fully complete until runtime wiring and error mapping are added</t>
   </si>
   <si>
     <t>PBI-104</t>
@@ -2448,6 +2448,30 @@
   </si>
   <si>
     <t>Important: closes the deactivation-policy spike with an implementation-ready matrix.</t>
+  </si>
+  <si>
+    <t>PBI-119</t>
+  </si>
+  <si>
+    <t>Enable modular test-file structure for oversized test suites</t>
+  </si>
+  <si>
+    <t>Capability to be created or improved: refactor oversized test files into smaller, focused test units so the test suite is easier to read, maintain, and extend. Why it is needed: current test files have grown to roughly 4,000 lines each, which reduces readability, increases merge friction, and makes coverage gaps harder to manage. Which future PBIs it enables: safer backend changes, faster defect isolation, and clearer module-level regression ownership. Technical scope: split large test files by behavior or subdomain, preserve existing describe/test intent, update imports/helpers/shared fixtures as needed, and keep test execution behavior unchanged. Explicit exclusions: no intentional business-rule changes and no broad rewrite of passing test logic beyond structural refactoring.</t>
+  </si>
+  <si>
+    <t>[ReqID: R26] Given an oversized test file is selected for refactoring, when the split is completed, then the tests are reorganized into smaller focused files grouped by behavior, workflow, or validation concern. | [ReqID: R26] Given the refactoring is structural only, when the full test suite runs, then all previously covered scenarios still pass without changing intended business behavior. | [ReqID: R26] Given shared setup or helpers are needed after splitting, when the work is reviewed, then common fixtures/utilities are extracted or reused consistently instead of duplicated across files. | [ReqID: R26] Given contributors work on future test changes, when they open the refactored test area, then file boundaries are readable enough to locate relevant describe/test blocks without scanning one monolithic file.</t>
+  </si>
+  <si>
+    <t>Maintainability;Testability;Reliability</t>
+  </si>
+  <si>
+    <t>Draft</t>
+  </si>
+  <si>
+    <t>Important: target split should follow behavior-oriented boundaries, for example create-path, validation, duplicate/conflict, authorization, and state-transition coverage. Evidence: before/after file structure, passing full test suite, and note of any extracted shared test helpers. If refactoring spans many modules or exceeds 5 points, split by module or domain area rather than one backlog item.</t>
+  </si>
+  <si>
+    <t>`</t>
   </si>
 </sst>
 </file>
@@ -3651,7 +3675,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:N119"/>
+  <dimension ref="A1:N121"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
@@ -4958,7 +4982,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" hidden="1" spans="1:14">
+    <row r="32" spans="1:14">
       <c r="A32" t="s">
         <v>241</v>
       </c>
@@ -4993,13 +5017,13 @@
         <v>247</v>
       </c>
       <c r="M32" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="N32" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="33" hidden="1" spans="1:14">
+    <row r="33" spans="1:14">
       <c r="A33" t="s">
         <v>249</v>
       </c>
@@ -5040,7 +5064,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="34" hidden="1" spans="1:14">
+    <row r="34" spans="1:14">
       <c r="A34" t="s">
         <v>254</v>
       </c>
@@ -5081,7 +5105,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="35" hidden="1" spans="1:14">
+    <row r="35" spans="1:14">
       <c r="A35" t="s">
         <v>259</v>
       </c>
@@ -5122,7 +5146,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="36" hidden="1" spans="1:14">
+    <row r="36" spans="1:14">
       <c r="A36" t="s">
         <v>265</v>
       </c>
@@ -5163,7 +5187,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="37" hidden="1" spans="1:14">
+    <row r="37" spans="1:14">
       <c r="A37" t="s">
         <v>271</v>
       </c>
@@ -5204,7 +5228,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="38" hidden="1" spans="1:14">
+    <row r="38" spans="1:14">
       <c r="A38" t="s">
         <v>276</v>
       </c>
@@ -5245,7 +5269,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="39" hidden="1" spans="1:14">
+    <row r="39" spans="1:14">
       <c r="A39" t="s">
         <v>281</v>
       </c>
@@ -5286,7 +5310,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="40" hidden="1" spans="1:14">
+    <row r="40" spans="1:14">
       <c r="A40" t="s">
         <v>287</v>
       </c>
@@ -5321,30 +5345,30 @@
         <v>292</v>
       </c>
       <c r="L40" t="s">
-        <v>293</v>
+        <v>247</v>
       </c>
       <c r="M40" t="s">
         <v>241</v>
       </c>
       <c r="N40" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14">
+      <c r="A41" t="s">
         <v>294</v>
-      </c>
-    </row>
-    <row r="41" hidden="1" spans="1:14">
-      <c r="A41" t="s">
-        <v>295</v>
       </c>
       <c r="B41" t="s">
         <v>288</v>
       </c>
       <c r="C41" t="s">
+        <v>295</v>
+      </c>
+      <c r="D41" t="s">
         <v>296</v>
       </c>
-      <c r="D41" t="s">
+      <c r="E41" t="s">
         <v>297</v>
-      </c>
-      <c r="E41" t="s">
-        <v>298</v>
       </c>
       <c r="F41" t="s">
         <v>42</v>
@@ -5365,36 +5389,36 @@
         <v>292</v>
       </c>
       <c r="L41" t="s">
-        <v>293</v>
+        <v>247</v>
       </c>
       <c r="M41" t="s">
+        <v>298</v>
+      </c>
+      <c r="N41" t="s">
         <v>299</v>
       </c>
-      <c r="N41" t="s">
+    </row>
+    <row r="42" spans="1:14">
+      <c r="A42" t="s">
         <v>300</v>
-      </c>
-    </row>
-    <row r="42" hidden="1" spans="1:14">
-      <c r="A42" t="s">
-        <v>301</v>
       </c>
       <c r="B42" t="s">
         <v>288</v>
       </c>
       <c r="C42" t="s">
+        <v>301</v>
+      </c>
+      <c r="D42" t="s">
         <v>302</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
         <v>303</v>
-      </c>
-      <c r="E42" t="s">
-        <v>304</v>
       </c>
       <c r="F42" t="s">
         <v>42</v>
       </c>
       <c r="G42" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H42">
         <v>2</v>
@@ -5406,10 +5430,10 @@
         <v>150</v>
       </c>
       <c r="K42" t="s">
+        <v>305</v>
+      </c>
+      <c r="L42" t="s">
         <v>306</v>
-      </c>
-      <c r="L42" t="s">
-        <v>247</v>
       </c>
       <c r="M42" t="s">
         <v>307</v>
@@ -5418,7 +5442,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="43" hidden="1" spans="1:14">
+    <row r="43" spans="1:14">
       <c r="A43" t="s">
         <v>309</v>
       </c>
@@ -5453,7 +5477,7 @@
         <v>292</v>
       </c>
       <c r="L43" t="s">
-        <v>293</v>
+        <v>247</v>
       </c>
       <c r="M43" t="s">
         <v>314</v>
@@ -5462,7 +5486,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="44" hidden="1" spans="1:14">
+    <row r="44" spans="1:14">
       <c r="A44" t="s">
         <v>316</v>
       </c>
@@ -5497,7 +5521,7 @@
         <v>292</v>
       </c>
       <c r="L44" t="s">
-        <v>293</v>
+        <v>247</v>
       </c>
       <c r="M44" t="s">
         <v>321</v>
@@ -5506,7 +5530,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="45" hidden="1" spans="1:14">
+    <row r="45" spans="1:14">
       <c r="A45" t="s">
         <v>323</v>
       </c>
@@ -5541,7 +5565,7 @@
         <v>292</v>
       </c>
       <c r="L45" t="s">
-        <v>293</v>
+        <v>247</v>
       </c>
       <c r="M45" t="s">
         <v>249</v>
@@ -5550,7 +5574,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="46" hidden="1" spans="1:14">
+    <row r="46" spans="1:14">
       <c r="A46" t="s">
         <v>328</v>
       </c>
@@ -5585,7 +5609,7 @@
         <v>292</v>
       </c>
       <c r="L46" t="s">
-        <v>293</v>
+        <v>247</v>
       </c>
       <c r="M46" t="s">
         <v>332</v>
@@ -5594,7 +5618,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="47" hidden="1" spans="1:14">
+    <row r="47" spans="1:14">
       <c r="A47" t="s">
         <v>334</v>
       </c>
@@ -5626,10 +5650,10 @@
         <v>150</v>
       </c>
       <c r="K47" t="s">
+        <v>305</v>
+      </c>
+      <c r="L47" t="s">
         <v>306</v>
-      </c>
-      <c r="L47" t="s">
-        <v>247</v>
       </c>
       <c r="M47" t="s">
         <v>332</v>
@@ -5638,7 +5662,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="48" hidden="1" spans="1:14">
+    <row r="48" spans="1:14">
       <c r="A48" t="s">
         <v>340</v>
       </c>
@@ -5673,7 +5697,7 @@
         <v>292</v>
       </c>
       <c r="L48" t="s">
-        <v>293</v>
+        <v>247</v>
       </c>
       <c r="M48" t="s">
         <v>344</v>
@@ -5682,7 +5706,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="49" hidden="1" spans="1:14">
+    <row r="49" spans="1:14">
       <c r="A49" t="s">
         <v>346</v>
       </c>
@@ -5723,7 +5747,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="50" hidden="1" spans="1:14">
+    <row r="50" spans="1:14">
       <c r="A50" t="s">
         <v>352</v>
       </c>
@@ -5758,7 +5782,7 @@
         <v>292</v>
       </c>
       <c r="L50" t="s">
-        <v>293</v>
+        <v>247</v>
       </c>
       <c r="M50" t="s">
         <v>357</v>
@@ -5767,7 +5791,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="51" hidden="1" spans="1:14">
+    <row r="51" spans="1:14">
       <c r="A51" t="s">
         <v>359</v>
       </c>
@@ -5811,7 +5835,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="52" hidden="1" spans="1:14">
+    <row r="52" spans="1:14">
       <c r="A52" t="s">
         <v>366</v>
       </c>
@@ -5843,10 +5867,10 @@
         <v>150</v>
       </c>
       <c r="K52" t="s">
+        <v>305</v>
+      </c>
+      <c r="L52" t="s">
         <v>306</v>
-      </c>
-      <c r="L52" t="s">
-        <v>247</v>
       </c>
       <c r="M52" t="s">
         <v>370</v>
@@ -5855,7 +5879,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="53" hidden="1" spans="1:14">
+    <row r="53" spans="1:14">
       <c r="A53" t="s">
         <v>372</v>
       </c>
@@ -5890,7 +5914,7 @@
         <v>363</v>
       </c>
       <c r="L53" t="s">
-        <v>35</v>
+        <v>247</v>
       </c>
       <c r="M53" t="s">
         <v>376</v>
@@ -5899,7 +5923,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="54" hidden="1" spans="1:14">
+    <row r="54" spans="1:14">
       <c r="A54" t="s">
         <v>378</v>
       </c>
@@ -5934,7 +5958,7 @@
         <v>363</v>
       </c>
       <c r="L54" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M54" t="s">
         <v>382</v>
@@ -5943,7 +5967,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="55" hidden="1" spans="1:14">
+    <row r="55" spans="1:14">
       <c r="A55" t="s">
         <v>384</v>
       </c>
@@ -5987,7 +6011,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="56" hidden="1" spans="1:14">
+    <row r="56" spans="1:14">
       <c r="A56" t="s">
         <v>390</v>
       </c>
@@ -6019,7 +6043,7 @@
         <v>61</v>
       </c>
       <c r="K56" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="L56" t="s">
         <v>35</v>
@@ -6031,7 +6055,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="57" hidden="1" spans="1:14">
+    <row r="57" spans="1:14">
       <c r="A57" t="s">
         <v>396</v>
       </c>
@@ -6063,10 +6087,10 @@
         <v>150</v>
       </c>
       <c r="K57" t="s">
+        <v>305</v>
+      </c>
+      <c r="L57" t="s">
         <v>306</v>
-      </c>
-      <c r="L57" t="s">
-        <v>247</v>
       </c>
       <c r="M57" t="s">
         <v>401</v>
@@ -6075,7 +6099,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="58" hidden="1" spans="1:14">
+    <row r="58" spans="1:14">
       <c r="A58" t="s">
         <v>403</v>
       </c>
@@ -6107,7 +6131,7 @@
         <v>95</v>
       </c>
       <c r="K58" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="L58" t="s">
         <v>35</v>
@@ -6119,7 +6143,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="59" hidden="1" spans="1:14">
+    <row r="59" spans="1:14">
       <c r="A59" t="s">
         <v>410</v>
       </c>
@@ -6160,7 +6184,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="60" hidden="1" spans="1:14">
+    <row r="60" spans="1:14">
       <c r="A60" t="s">
         <v>416</v>
       </c>
@@ -6195,7 +6219,7 @@
         <v>292</v>
       </c>
       <c r="L60" t="s">
-        <v>293</v>
+        <v>247</v>
       </c>
       <c r="M60" t="s">
         <v>265</v>
@@ -6204,7 +6228,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="61" hidden="1" spans="1:14">
+    <row r="61" spans="1:14">
       <c r="A61" t="s">
         <v>422</v>
       </c>
@@ -6239,7 +6263,7 @@
         <v>292</v>
       </c>
       <c r="L61" t="s">
-        <v>293</v>
+        <v>247</v>
       </c>
       <c r="M61" t="s">
         <v>427</v>
@@ -6248,7 +6272,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="62" hidden="1" spans="1:14">
+    <row r="62" spans="1:14">
       <c r="A62" t="s">
         <v>429</v>
       </c>
@@ -6280,10 +6304,10 @@
         <v>150</v>
       </c>
       <c r="K62" t="s">
+        <v>305</v>
+      </c>
+      <c r="L62" t="s">
         <v>306</v>
-      </c>
-      <c r="L62" t="s">
-        <v>247</v>
       </c>
       <c r="M62" t="s">
         <v>427</v>
@@ -6292,7 +6316,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="63" hidden="1" spans="1:14">
+    <row r="63" spans="1:14">
       <c r="A63" t="s">
         <v>435</v>
       </c>
@@ -6327,7 +6351,7 @@
         <v>292</v>
       </c>
       <c r="L63" t="s">
-        <v>293</v>
+        <v>247</v>
       </c>
       <c r="M63" t="s">
         <v>439</v>
@@ -6336,7 +6360,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="64" hidden="1" spans="1:14">
+    <row r="64" spans="1:14">
       <c r="A64" t="s">
         <v>441</v>
       </c>
@@ -6377,7 +6401,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="65" hidden="1" spans="1:14">
+    <row r="65" spans="1:14">
       <c r="A65" t="s">
         <v>447</v>
       </c>
@@ -6421,7 +6445,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="66" hidden="1" spans="1:14">
+    <row r="66" spans="1:14">
       <c r="A66" t="s">
         <v>453</v>
       </c>
@@ -6465,7 +6489,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="67" hidden="1" spans="1:14">
+    <row r="67" spans="1:14">
       <c r="A67" t="s">
         <v>459</v>
       </c>
@@ -6497,10 +6521,10 @@
         <v>150</v>
       </c>
       <c r="K67" t="s">
+        <v>305</v>
+      </c>
+      <c r="L67" t="s">
         <v>306</v>
-      </c>
-      <c r="L67" t="s">
-        <v>247</v>
       </c>
       <c r="M67" t="s">
         <v>463</v>
@@ -6509,7 +6533,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="68" hidden="1" spans="1:14">
+    <row r="68" spans="1:14">
       <c r="A68" t="s">
         <v>465</v>
       </c>
@@ -6553,7 +6577,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="69" hidden="1" spans="1:14">
+    <row r="69" spans="1:14">
       <c r="A69" t="s">
         <v>471</v>
       </c>
@@ -6594,7 +6618,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="70" hidden="1" spans="1:14">
+    <row r="70" spans="1:14">
       <c r="A70" t="s">
         <v>477</v>
       </c>
@@ -6638,7 +6662,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="71" hidden="1" spans="1:14">
+    <row r="71" spans="1:14">
       <c r="A71" t="s">
         <v>483</v>
       </c>
@@ -6682,7 +6706,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="72" hidden="1" spans="1:14">
+    <row r="72" spans="1:14">
       <c r="A72" t="s">
         <v>490</v>
       </c>
@@ -6714,10 +6738,10 @@
         <v>150</v>
       </c>
       <c r="K72" t="s">
+        <v>305</v>
+      </c>
+      <c r="L72" t="s">
         <v>306</v>
-      </c>
-      <c r="L72" t="s">
-        <v>247</v>
       </c>
       <c r="M72" t="s">
         <v>494</v>
@@ -6726,7 +6750,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="73" hidden="1" spans="1:14">
+    <row r="73" spans="1:14">
       <c r="A73" t="s">
         <v>496</v>
       </c>
@@ -6770,7 +6794,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="74" hidden="1" spans="1:14">
+    <row r="74" spans="1:14">
       <c r="A74" t="s">
         <v>502</v>
       </c>
@@ -6811,7 +6835,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="75" hidden="1" spans="1:14">
+    <row r="75" spans="1:14">
       <c r="A75" t="s">
         <v>508</v>
       </c>
@@ -6855,7 +6879,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="76" hidden="1" spans="1:14">
+    <row r="76" spans="1:14">
       <c r="A76" t="s">
         <v>515</v>
       </c>
@@ -6899,7 +6923,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="77" hidden="1" spans="1:14">
+    <row r="77" spans="1:14">
       <c r="A77" t="s">
         <v>522</v>
       </c>
@@ -6931,10 +6955,10 @@
         <v>150</v>
       </c>
       <c r="K77" t="s">
+        <v>305</v>
+      </c>
+      <c r="L77" t="s">
         <v>306</v>
-      </c>
-      <c r="L77" t="s">
-        <v>247</v>
       </c>
       <c r="M77" t="s">
         <v>526</v>
@@ -6943,7 +6967,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="78" hidden="1" spans="1:14">
+    <row r="78" spans="1:14">
       <c r="A78" t="s">
         <v>528</v>
       </c>
@@ -6984,7 +7008,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="79" hidden="1" spans="1:14">
+    <row r="79" spans="1:14">
       <c r="A79" t="s">
         <v>534</v>
       </c>
@@ -7025,7 +7049,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="80" hidden="1" spans="1:14">
+    <row r="80" spans="1:14">
       <c r="A80" t="s">
         <v>540</v>
       </c>
@@ -7057,19 +7081,19 @@
         <v>44</v>
       </c>
       <c r="K80" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="L80" t="s">
         <v>35</v>
       </c>
       <c r="M80" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="N80" t="s">
         <v>546</v>
       </c>
     </row>
-    <row r="81" hidden="1" spans="1:14">
+    <row r="81" spans="1:14">
       <c r="A81" t="s">
         <v>547</v>
       </c>
@@ -7101,7 +7125,7 @@
         <v>150</v>
       </c>
       <c r="K81" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="L81" t="s">
         <v>35</v>
@@ -7113,7 +7137,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="82" hidden="1" spans="1:14">
+    <row r="82" spans="1:14">
       <c r="A82" t="s">
         <v>553</v>
       </c>
@@ -7145,7 +7169,7 @@
         <v>150</v>
       </c>
       <c r="K82" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="L82" t="s">
         <v>35</v>
@@ -7157,7 +7181,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="83" hidden="1" spans="1:14">
+    <row r="83" spans="1:14">
       <c r="A83" t="s">
         <v>560</v>
       </c>
@@ -7189,7 +7213,7 @@
         <v>44</v>
       </c>
       <c r="K83" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="L83" t="s">
         <v>35</v>
@@ -7201,7 +7225,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="84" hidden="1" spans="1:14">
+    <row r="84" spans="1:14">
       <c r="A84" t="s">
         <v>566</v>
       </c>
@@ -7236,7 +7260,7 @@
         <v>363</v>
       </c>
       <c r="L84" t="s">
-        <v>35</v>
+        <v>247</v>
       </c>
       <c r="M84" t="s">
         <v>572</v>
@@ -7245,7 +7269,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="85" hidden="1" spans="1:14">
+    <row r="85" spans="1:14">
       <c r="A85" t="s">
         <v>574</v>
       </c>
@@ -7280,7 +7304,7 @@
         <v>363</v>
       </c>
       <c r="L85" t="s">
-        <v>35</v>
+        <v>247</v>
       </c>
       <c r="M85" t="s">
         <v>359</v>
@@ -7289,7 +7313,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="86" hidden="1" spans="1:14">
+    <row r="86" spans="1:14">
       <c r="A86" t="s">
         <v>580</v>
       </c>
@@ -7324,7 +7348,7 @@
         <v>363</v>
       </c>
       <c r="L86" t="s">
-        <v>35</v>
+        <v>247</v>
       </c>
       <c r="M86" t="s">
         <v>574</v>
@@ -7333,7 +7357,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="87" hidden="1" spans="1:14">
+    <row r="87" spans="1:14">
       <c r="A87" t="s">
         <v>586</v>
       </c>
@@ -7377,7 +7401,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="88" hidden="1" spans="1:14">
+    <row r="88" spans="1:14">
       <c r="A88" t="s">
         <v>593</v>
       </c>
@@ -7421,7 +7445,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="89" hidden="1" spans="1:14">
+    <row r="89" spans="1:14">
       <c r="A89" t="s">
         <v>599</v>
       </c>
@@ -7465,7 +7489,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="90" hidden="1" spans="1:14">
+    <row r="90" spans="1:14">
       <c r="A90" t="s">
         <v>605</v>
       </c>
@@ -7497,7 +7521,7 @@
         <v>44</v>
       </c>
       <c r="K90" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="L90" t="s">
         <v>35</v>
@@ -7509,7 +7533,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="91" hidden="1" spans="1:14">
+    <row r="91" spans="1:14">
       <c r="A91" t="s">
         <v>612</v>
       </c>
@@ -7541,7 +7565,7 @@
         <v>95</v>
       </c>
       <c r="K91" t="s">
-        <v>306</v>
+        <v>363</v>
       </c>
       <c r="L91" t="s">
         <v>35</v>
@@ -7553,7 +7577,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="92" hidden="1" spans="1:14">
+    <row r="92" spans="1:14">
       <c r="A92" t="s">
         <v>619</v>
       </c>
@@ -7597,7 +7621,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="93" hidden="1" spans="1:14">
+    <row r="93" spans="1:14">
       <c r="A93" t="s">
         <v>626</v>
       </c>
@@ -7632,7 +7656,7 @@
         <v>363</v>
       </c>
       <c r="L93" t="s">
-        <v>45</v>
+        <v>247</v>
       </c>
       <c r="M93" t="s">
         <v>24</v>
@@ -7641,7 +7665,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="94" hidden="1" spans="1:14">
+    <row r="94" spans="1:14">
       <c r="A94" t="s">
         <v>633</v>
       </c>
@@ -7676,7 +7700,7 @@
         <v>363</v>
       </c>
       <c r="L94" t="s">
-        <v>293</v>
+        <v>247</v>
       </c>
       <c r="M94" t="s">
         <v>24</v>
@@ -7685,7 +7709,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="95" hidden="1" spans="1:14">
+    <row r="95" spans="1:14">
       <c r="A95" t="s">
         <v>639</v>
       </c>
@@ -7717,10 +7741,10 @@
         <v>44</v>
       </c>
       <c r="K95" t="s">
-        <v>306</v>
+        <v>363</v>
       </c>
       <c r="L95" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M95" t="s">
         <v>644</v>
@@ -7729,7 +7753,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="96" hidden="1" spans="1:14">
+    <row r="96" spans="1:14">
       <c r="A96" t="s">
         <v>646</v>
       </c>
@@ -7773,7 +7797,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="97" hidden="1" spans="1:14">
+    <row r="97" spans="1:14">
       <c r="A97" t="s">
         <v>652</v>
       </c>
@@ -7817,7 +7841,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="98" hidden="1" spans="1:14">
+    <row r="98" spans="1:14">
       <c r="A98" t="s">
         <v>658</v>
       </c>
@@ -7852,7 +7876,7 @@
         <v>363</v>
       </c>
       <c r="L98" t="s">
-        <v>293</v>
+        <v>247</v>
       </c>
       <c r="M98" t="s">
         <v>24</v>
@@ -7861,7 +7885,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="99" hidden="1" spans="1:14">
+    <row r="99" spans="1:14">
       <c r="A99" t="s">
         <v>665</v>
       </c>
@@ -7896,7 +7920,7 @@
         <v>363</v>
       </c>
       <c r="L99" t="s">
-        <v>35</v>
+        <v>247</v>
       </c>
       <c r="M99" t="s">
         <v>670</v>
@@ -7905,7 +7929,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="100" hidden="1" spans="1:14">
+    <row r="100" spans="1:14">
       <c r="A100" t="s">
         <v>672</v>
       </c>
@@ -7940,7 +7964,7 @@
         <v>363</v>
       </c>
       <c r="L100" t="s">
-        <v>35</v>
+        <v>247</v>
       </c>
       <c r="M100" t="s">
         <v>677</v>
@@ -7949,7 +7973,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="101" hidden="1" spans="1:14">
+    <row r="101" spans="1:14">
       <c r="A101" t="s">
         <v>679</v>
       </c>
@@ -7984,7 +8008,7 @@
         <v>363</v>
       </c>
       <c r="L101" t="s">
-        <v>35</v>
+        <v>247</v>
       </c>
       <c r="M101" t="s">
         <v>684</v>
@@ -7993,7 +8017,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="102" hidden="1" spans="1:14">
+    <row r="102" spans="1:14">
       <c r="A102" t="s">
         <v>686</v>
       </c>
@@ -8028,7 +8052,7 @@
         <v>363</v>
       </c>
       <c r="L102" t="s">
-        <v>35</v>
+        <v>247</v>
       </c>
       <c r="M102" t="s">
         <v>691</v>
@@ -8037,7 +8061,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="103" hidden="1" spans="1:14">
+    <row r="103" spans="1:14">
       <c r="A103" t="s">
         <v>693</v>
       </c>
@@ -8072,7 +8096,7 @@
         <v>363</v>
       </c>
       <c r="L103" t="s">
-        <v>35</v>
+        <v>247</v>
       </c>
       <c r="M103" t="s">
         <v>698</v>
@@ -8081,7 +8105,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="104" hidden="1" spans="1:14">
+    <row r="104" spans="1:14">
       <c r="A104" t="s">
         <v>700</v>
       </c>
@@ -8116,7 +8140,7 @@
         <v>363</v>
       </c>
       <c r="L104" t="s">
-        <v>35</v>
+        <v>247</v>
       </c>
       <c r="M104" t="s">
         <v>705</v>
@@ -8125,7 +8149,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="105" hidden="1" spans="1:14">
+    <row r="105" spans="1:14">
       <c r="A105" t="s">
         <v>707</v>
       </c>
@@ -8160,7 +8184,7 @@
         <v>363</v>
       </c>
       <c r="L105" t="s">
-        <v>35</v>
+        <v>247</v>
       </c>
       <c r="M105" t="s">
         <v>711</v>
@@ -8169,7 +8193,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="106" hidden="1" spans="1:14">
+    <row r="106" spans="1:14">
       <c r="A106" t="s">
         <v>713</v>
       </c>
@@ -8213,7 +8237,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="107" hidden="1" spans="1:14">
+    <row r="107" spans="1:14">
       <c r="A107" t="s">
         <v>719</v>
       </c>
@@ -8257,7 +8281,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="108" hidden="1" spans="1:14">
+    <row r="108" spans="1:14">
       <c r="A108" t="s">
         <v>726</v>
       </c>
@@ -8301,7 +8325,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="109" hidden="1" spans="1:14">
+    <row r="109" spans="1:14">
       <c r="A109" t="s">
         <v>733</v>
       </c>
@@ -8345,7 +8369,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="110" hidden="1" spans="1:14">
+    <row r="110" spans="1:14">
       <c r="A110" t="s">
         <v>740</v>
       </c>
@@ -8389,7 +8413,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="111" hidden="1" spans="1:14">
+    <row r="111" spans="1:14">
       <c r="A111" t="s">
         <v>747</v>
       </c>
@@ -8433,7 +8457,7 @@
         <v>752</v>
       </c>
     </row>
-    <row r="112" hidden="1" spans="1:14">
+    <row r="112" spans="1:14">
       <c r="A112" t="s">
         <v>753</v>
       </c>
@@ -8477,7 +8501,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="113" hidden="1" spans="1:14">
+    <row r="113" spans="1:14">
       <c r="A113" t="s">
         <v>760</v>
       </c>
@@ -8509,7 +8533,7 @@
         <v>44</v>
       </c>
       <c r="K113" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="L113" t="s">
         <v>35</v>
@@ -8521,7 +8545,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="114" hidden="1" spans="1:14">
+    <row r="114" spans="1:14">
       <c r="A114" t="s">
         <v>766</v>
       </c>
@@ -8553,7 +8577,7 @@
         <v>61</v>
       </c>
       <c r="K114" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="L114" t="s">
         <v>35</v>
@@ -8565,7 +8589,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="115" hidden="1" spans="1:14">
+    <row r="115" spans="1:14">
       <c r="A115" t="s">
         <v>773</v>
       </c>
@@ -8597,7 +8621,7 @@
         <v>61</v>
       </c>
       <c r="K115" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="L115" t="s">
         <v>35</v>
@@ -8644,7 +8668,7 @@
         <v>363</v>
       </c>
       <c r="L116" t="s">
-        <v>293</v>
+        <v>247</v>
       </c>
       <c r="M116" t="s">
         <v>626</v>
@@ -8688,7 +8712,7 @@
         <v>363</v>
       </c>
       <c r="L117" t="s">
-        <v>45</v>
+        <v>247</v>
       </c>
       <c r="M117" t="s">
         <v>791</v>
@@ -8697,7 +8721,7 @@
         <v>792</v>
       </c>
     </row>
-    <row r="118" hidden="1" spans="1:14">
+    <row r="118" spans="1:14">
       <c r="A118" t="s">
         <v>793</v>
       </c>
@@ -8741,7 +8765,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="119" hidden="1" spans="1:14">
+    <row r="119" spans="1:14">
       <c r="A119" t="s">
         <v>799</v>
       </c>
@@ -8785,12 +8809,65 @@
         <v>805</v>
       </c>
     </row>
+    <row r="120" spans="1:14">
+      <c r="A120" t="s">
+        <v>806</v>
+      </c>
+      <c r="B120" t="s">
+        <v>548</v>
+      </c>
+      <c r="C120" t="s">
+        <v>807</v>
+      </c>
+      <c r="D120" t="s">
+        <v>808</v>
+      </c>
+      <c r="E120" t="s">
+        <v>809</v>
+      </c>
+      <c r="F120" t="s">
+        <v>211</v>
+      </c>
+      <c r="G120" t="s">
+        <v>810</v>
+      </c>
+      <c r="H120">
+        <v>3</v>
+      </c>
+      <c r="I120" t="s">
+        <v>21</v>
+      </c>
+      <c r="J120" t="s">
+        <v>44</v>
+      </c>
+      <c r="K120" t="s">
+        <v>363</v>
+      </c>
+      <c r="L120" t="s">
+        <v>811</v>
+      </c>
+      <c r="M120" t="s">
+        <v>24</v>
+      </c>
+      <c r="N120" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="121" spans="1:14">
+      <c r="D121" t="s">
+        <v>813</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:N119" etc:filterBottomFollowUsedRange="0">
-    <filterColumn colId="12">
-      <customFilters>
-        <customFilter operator="equal" val="*PBI-092*"/>
-      </customFilters>
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:N121" etc:filterBottomFollowUsedRange="0">
+    <filterColumn colId="1">
+      <filters blank="1">
+        <filter val="Enabler"/>
+        <filter val="Spike"/>
+        <filter val="Bug"/>
+        <filter val="Story"/>
+        <filter val="Task"/>
+      </filters>
     </filterColumn>
     <extLst/>
   </autoFilter>

</xml_diff>

<commit_message>
[PBI-108] Migrate protected route consumers to trusted actor context
</commit_message>
<xml_diff>
--- a/backlog/backlog.xlsx
+++ b/backlog/backlog.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9384"/>
+    <workbookView windowWidth="12420" windowHeight="4716"/>
   </bookViews>
   <sheets>
     <sheet name="backlog" sheetId="1" r:id="rId1"/>
@@ -4982,7 +4982,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:14">
+    <row r="32" hidden="1" spans="1:14">
       <c r="A32" t="s">
         <v>241</v>
       </c>
@@ -5023,7 +5023,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="33" spans="1:14">
+    <row r="33" hidden="1" spans="1:14">
       <c r="A33" t="s">
         <v>249</v>
       </c>
@@ -5064,7 +5064,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="34" spans="1:14">
+    <row r="34" hidden="1" spans="1:14">
       <c r="A34" t="s">
         <v>254</v>
       </c>
@@ -5105,7 +5105,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="35" spans="1:14">
+    <row r="35" hidden="1" spans="1:14">
       <c r="A35" t="s">
         <v>259</v>
       </c>
@@ -5146,7 +5146,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="36" spans="1:14">
+    <row r="36" hidden="1" spans="1:14">
       <c r="A36" t="s">
         <v>265</v>
       </c>
@@ -5187,7 +5187,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="37" spans="1:14">
+    <row r="37" hidden="1" spans="1:14">
       <c r="A37" t="s">
         <v>271</v>
       </c>
@@ -5228,7 +5228,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="38" spans="1:14">
+    <row r="38" hidden="1" spans="1:14">
       <c r="A38" t="s">
         <v>276</v>
       </c>
@@ -5269,7 +5269,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="39" spans="1:14">
+    <row r="39" hidden="1" spans="1:14">
       <c r="A39" t="s">
         <v>281</v>
       </c>
@@ -5310,7 +5310,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="40" spans="1:14">
+    <row r="40" hidden="1" spans="1:14">
       <c r="A40" t="s">
         <v>287</v>
       </c>
@@ -5354,7 +5354,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="41" spans="1:14">
+    <row r="41" hidden="1" spans="1:14">
       <c r="A41" t="s">
         <v>294</v>
       </c>
@@ -5398,7 +5398,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="42" spans="1:14">
+    <row r="42" hidden="1" spans="1:14">
       <c r="A42" t="s">
         <v>300</v>
       </c>
@@ -5442,7 +5442,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="43" spans="1:14">
+    <row r="43" hidden="1" spans="1:14">
       <c r="A43" t="s">
         <v>309</v>
       </c>
@@ -5486,7 +5486,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="44" spans="1:14">
+    <row r="44" hidden="1" spans="1:14">
       <c r="A44" t="s">
         <v>316</v>
       </c>
@@ -5530,7 +5530,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="45" spans="1:14">
+    <row r="45" hidden="1" spans="1:14">
       <c r="A45" t="s">
         <v>323</v>
       </c>
@@ -5574,7 +5574,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="46" spans="1:14">
+    <row r="46" hidden="1" spans="1:14">
       <c r="A46" t="s">
         <v>328</v>
       </c>
@@ -5618,7 +5618,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="47" spans="1:14">
+    <row r="47" hidden="1" spans="1:14">
       <c r="A47" t="s">
         <v>334</v>
       </c>
@@ -5662,7 +5662,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="48" spans="1:14">
+    <row r="48" hidden="1" spans="1:14">
       <c r="A48" t="s">
         <v>340</v>
       </c>
@@ -5706,7 +5706,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="49" spans="1:14">
+    <row r="49" hidden="1" spans="1:14">
       <c r="A49" t="s">
         <v>346</v>
       </c>
@@ -5747,7 +5747,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="50" spans="1:14">
+    <row r="50" hidden="1" spans="1:14">
       <c r="A50" t="s">
         <v>352</v>
       </c>
@@ -5791,7 +5791,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="51" spans="1:14">
+    <row r="51" hidden="1" spans="1:14">
       <c r="A51" t="s">
         <v>359</v>
       </c>
@@ -5835,7 +5835,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="52" spans="1:14">
+    <row r="52" hidden="1" spans="1:14">
       <c r="A52" t="s">
         <v>366</v>
       </c>
@@ -5879,7 +5879,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="53" spans="1:14">
+    <row r="53" hidden="1" spans="1:14">
       <c r="A53" t="s">
         <v>372</v>
       </c>
@@ -5923,7 +5923,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="54" spans="1:14">
+    <row r="54" hidden="1" spans="1:14">
       <c r="A54" t="s">
         <v>378</v>
       </c>
@@ -5958,7 +5958,7 @@
         <v>363</v>
       </c>
       <c r="L54" t="s">
-        <v>45</v>
+        <v>247</v>
       </c>
       <c r="M54" t="s">
         <v>382</v>
@@ -5967,7 +5967,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="55" spans="1:14">
+    <row r="55" hidden="1" spans="1:14">
       <c r="A55" t="s">
         <v>384</v>
       </c>
@@ -6011,7 +6011,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="56" spans="1:14">
+    <row r="56" hidden="1" spans="1:14">
       <c r="A56" t="s">
         <v>390</v>
       </c>
@@ -6055,7 +6055,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="57" spans="1:14">
+    <row r="57" hidden="1" spans="1:14">
       <c r="A57" t="s">
         <v>396</v>
       </c>
@@ -6099,7 +6099,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="58" spans="1:14">
+    <row r="58" hidden="1" spans="1:14">
       <c r="A58" t="s">
         <v>403</v>
       </c>
@@ -6143,7 +6143,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="59" spans="1:14">
+    <row r="59" hidden="1" spans="1:14">
       <c r="A59" t="s">
         <v>410</v>
       </c>
@@ -6184,7 +6184,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="60" spans="1:14">
+    <row r="60" hidden="1" spans="1:14">
       <c r="A60" t="s">
         <v>416</v>
       </c>
@@ -6228,7 +6228,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="61" spans="1:14">
+    <row r="61" hidden="1" spans="1:14">
       <c r="A61" t="s">
         <v>422</v>
       </c>
@@ -6272,7 +6272,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="62" spans="1:14">
+    <row r="62" hidden="1" spans="1:14">
       <c r="A62" t="s">
         <v>429</v>
       </c>
@@ -6316,7 +6316,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="63" spans="1:14">
+    <row r="63" hidden="1" spans="1:14">
       <c r="A63" t="s">
         <v>435</v>
       </c>
@@ -6360,7 +6360,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="64" spans="1:14">
+    <row r="64" hidden="1" spans="1:14">
       <c r="A64" t="s">
         <v>441</v>
       </c>
@@ -6401,7 +6401,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="65" spans="1:14">
+    <row r="65" hidden="1" spans="1:14">
       <c r="A65" t="s">
         <v>447</v>
       </c>
@@ -6445,7 +6445,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="66" spans="1:14">
+    <row r="66" hidden="1" spans="1:14">
       <c r="A66" t="s">
         <v>453</v>
       </c>
@@ -6489,7 +6489,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="67" spans="1:14">
+    <row r="67" hidden="1" spans="1:14">
       <c r="A67" t="s">
         <v>459</v>
       </c>
@@ -6533,7 +6533,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="68" spans="1:14">
+    <row r="68" hidden="1" spans="1:14">
       <c r="A68" t="s">
         <v>465</v>
       </c>
@@ -6577,7 +6577,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="69" spans="1:14">
+    <row r="69" hidden="1" spans="1:14">
       <c r="A69" t="s">
         <v>471</v>
       </c>
@@ -6618,7 +6618,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="70" spans="1:14">
+    <row r="70" hidden="1" spans="1:14">
       <c r="A70" t="s">
         <v>477</v>
       </c>
@@ -6662,7 +6662,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="71" spans="1:14">
+    <row r="71" hidden="1" spans="1:14">
       <c r="A71" t="s">
         <v>483</v>
       </c>
@@ -6706,7 +6706,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="72" spans="1:14">
+    <row r="72" hidden="1" spans="1:14">
       <c r="A72" t="s">
         <v>490</v>
       </c>
@@ -6750,7 +6750,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="73" spans="1:14">
+    <row r="73" hidden="1" spans="1:14">
       <c r="A73" t="s">
         <v>496</v>
       </c>
@@ -6794,7 +6794,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="74" spans="1:14">
+    <row r="74" hidden="1" spans="1:14">
       <c r="A74" t="s">
         <v>502</v>
       </c>
@@ -6835,7 +6835,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="75" spans="1:14">
+    <row r="75" hidden="1" spans="1:14">
       <c r="A75" t="s">
         <v>508</v>
       </c>
@@ -6879,7 +6879,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="76" spans="1:14">
+    <row r="76" hidden="1" spans="1:14">
       <c r="A76" t="s">
         <v>515</v>
       </c>
@@ -6923,7 +6923,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="77" spans="1:14">
+    <row r="77" hidden="1" spans="1:14">
       <c r="A77" t="s">
         <v>522</v>
       </c>
@@ -6967,7 +6967,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="78" spans="1:14">
+    <row r="78" hidden="1" spans="1:14">
       <c r="A78" t="s">
         <v>528</v>
       </c>
@@ -7008,7 +7008,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="79" spans="1:14">
+    <row r="79" hidden="1" spans="1:14">
       <c r="A79" t="s">
         <v>534</v>
       </c>
@@ -7049,7 +7049,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="80" spans="1:14">
+    <row r="80" hidden="1" spans="1:14">
       <c r="A80" t="s">
         <v>540</v>
       </c>
@@ -7093,7 +7093,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="81" spans="1:14">
+    <row r="81" hidden="1" spans="1:14">
       <c r="A81" t="s">
         <v>547</v>
       </c>
@@ -7137,7 +7137,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="82" spans="1:14">
+    <row r="82" hidden="1" spans="1:14">
       <c r="A82" t="s">
         <v>553</v>
       </c>
@@ -7181,7 +7181,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="83" spans="1:14">
+    <row r="83" hidden="1" spans="1:14">
       <c r="A83" t="s">
         <v>560</v>
       </c>
@@ -7225,7 +7225,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="84" spans="1:14">
+    <row r="84" hidden="1" spans="1:14">
       <c r="A84" t="s">
         <v>566</v>
       </c>
@@ -7269,7 +7269,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="85" spans="1:14">
+    <row r="85" hidden="1" spans="1:14">
       <c r="A85" t="s">
         <v>574</v>
       </c>
@@ -7313,7 +7313,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="86" spans="1:14">
+    <row r="86" hidden="1" spans="1:14">
       <c r="A86" t="s">
         <v>580</v>
       </c>
@@ -7357,7 +7357,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="87" spans="1:14">
+    <row r="87" hidden="1" spans="1:14">
       <c r="A87" t="s">
         <v>586</v>
       </c>
@@ -7401,7 +7401,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="88" spans="1:14">
+    <row r="88" hidden="1" spans="1:14">
       <c r="A88" t="s">
         <v>593</v>
       </c>
@@ -7480,7 +7480,7 @@
         <v>363</v>
       </c>
       <c r="L89" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M89" t="s">
         <v>603</v>
@@ -7489,7 +7489,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="90" spans="1:14">
+    <row r="90" hidden="1" spans="1:14">
       <c r="A90" t="s">
         <v>605</v>
       </c>
@@ -7533,7 +7533,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="91" spans="1:14">
+    <row r="91" hidden="1" spans="1:14">
       <c r="A91" t="s">
         <v>612</v>
       </c>
@@ -7612,7 +7612,7 @@
         <v>363</v>
       </c>
       <c r="L92" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M92" t="s">
         <v>624</v>
@@ -7621,7 +7621,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="93" spans="1:14">
+    <row r="93" hidden="1" spans="1:14">
       <c r="A93" t="s">
         <v>626</v>
       </c>
@@ -7665,7 +7665,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="94" spans="1:14">
+    <row r="94" hidden="1" spans="1:14">
       <c r="A94" t="s">
         <v>633</v>
       </c>
@@ -7709,7 +7709,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="95" spans="1:14">
+    <row r="95" hidden="1" spans="1:14">
       <c r="A95" t="s">
         <v>639</v>
       </c>
@@ -7744,7 +7744,7 @@
         <v>363</v>
       </c>
       <c r="L95" t="s">
-        <v>45</v>
+        <v>247</v>
       </c>
       <c r="M95" t="s">
         <v>644</v>
@@ -7753,7 +7753,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="96" spans="1:14">
+    <row r="96" hidden="1" spans="1:14">
       <c r="A96" t="s">
         <v>646</v>
       </c>
@@ -7832,7 +7832,7 @@
         <v>363</v>
       </c>
       <c r="L97" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M97" t="s">
         <v>656</v>
@@ -7841,7 +7841,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="98" spans="1:14">
+    <row r="98" hidden="1" spans="1:14">
       <c r="A98" t="s">
         <v>658</v>
       </c>
@@ -7885,7 +7885,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="99" spans="1:14">
+    <row r="99" hidden="1" spans="1:14">
       <c r="A99" t="s">
         <v>665</v>
       </c>
@@ -7929,7 +7929,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="100" spans="1:14">
+    <row r="100" hidden="1" spans="1:14">
       <c r="A100" t="s">
         <v>672</v>
       </c>
@@ -7973,7 +7973,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="101" spans="1:14">
+    <row r="101" hidden="1" spans="1:14">
       <c r="A101" t="s">
         <v>679</v>
       </c>
@@ -8017,7 +8017,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="102" spans="1:14">
+    <row r="102" hidden="1" spans="1:14">
       <c r="A102" t="s">
         <v>686</v>
       </c>
@@ -8061,7 +8061,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="103" spans="1:14">
+    <row r="103" hidden="1" spans="1:14">
       <c r="A103" t="s">
         <v>693</v>
       </c>
@@ -8105,7 +8105,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="104" spans="1:14">
+    <row r="104" hidden="1" spans="1:14">
       <c r="A104" t="s">
         <v>700</v>
       </c>
@@ -8149,7 +8149,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="105" spans="1:14">
+    <row r="105" hidden="1" spans="1:14">
       <c r="A105" t="s">
         <v>707</v>
       </c>
@@ -8228,7 +8228,7 @@
         <v>363</v>
       </c>
       <c r="L106" t="s">
-        <v>35</v>
+        <v>247</v>
       </c>
       <c r="M106" t="s">
         <v>586</v>
@@ -8272,7 +8272,7 @@
         <v>363</v>
       </c>
       <c r="L107" t="s">
-        <v>35</v>
+        <v>247</v>
       </c>
       <c r="M107" t="s">
         <v>724</v>
@@ -8316,7 +8316,7 @@
         <v>363</v>
       </c>
       <c r="L108" t="s">
-        <v>35</v>
+        <v>247</v>
       </c>
       <c r="M108" t="s">
         <v>731</v>
@@ -8360,7 +8360,7 @@
         <v>363</v>
       </c>
       <c r="L109" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M109" t="s">
         <v>738</v>
@@ -8404,7 +8404,7 @@
         <v>363</v>
       </c>
       <c r="L110" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M110" t="s">
         <v>745</v>
@@ -8448,7 +8448,7 @@
         <v>363</v>
       </c>
       <c r="L111" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M111" t="s">
         <v>612</v>
@@ -8492,7 +8492,7 @@
         <v>363</v>
       </c>
       <c r="L112" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M112" t="s">
         <v>758</v>
@@ -8501,7 +8501,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="113" spans="1:14">
+    <row r="113" hidden="1" spans="1:14">
       <c r="A113" t="s">
         <v>760</v>
       </c>
@@ -8545,7 +8545,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="114" spans="1:14">
+    <row r="114" hidden="1" spans="1:14">
       <c r="A114" t="s">
         <v>766</v>
       </c>
@@ -8589,7 +8589,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="115" spans="1:14">
+    <row r="115" hidden="1" spans="1:14">
       <c r="A115" t="s">
         <v>773</v>
       </c>
@@ -8633,7 +8633,7 @@
         <v>779</v>
       </c>
     </row>
-    <row r="116" spans="1:14">
+    <row r="116" hidden="1" spans="1:14">
       <c r="A116" t="s">
         <v>780</v>
       </c>
@@ -8677,7 +8677,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="117" spans="1:14">
+    <row r="117" hidden="1" spans="1:14">
       <c r="A117" t="s">
         <v>786</v>
       </c>
@@ -8721,7 +8721,7 @@
         <v>792</v>
       </c>
     </row>
-    <row r="118" spans="1:14">
+    <row r="118" hidden="1" spans="1:14">
       <c r="A118" t="s">
         <v>793</v>
       </c>
@@ -8765,7 +8765,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="119" spans="1:14">
+    <row r="119" hidden="1" spans="1:14">
       <c r="A119" t="s">
         <v>799</v>
       </c>
@@ -8809,7 +8809,7 @@
         <v>805</v>
       </c>
     </row>
-    <row r="120" spans="1:14">
+    <row r="120" hidden="1" spans="1:14">
       <c r="A120" t="s">
         <v>806</v>
       </c>
@@ -8853,20 +8853,25 @@
         <v>812</v>
       </c>
     </row>
-    <row r="121" spans="1:14">
+    <row r="121" hidden="1" spans="1:14">
       <c r="D121" t="s">
         <v>813</v>
       </c>
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:N121" etc:filterBottomFollowUsedRange="0">
-    <filterColumn colId="1">
-      <filters blank="1">
-        <filter val="Enabler"/>
-        <filter val="Spike"/>
-        <filter val="Bug"/>
-        <filter val="Story"/>
-        <filter val="Task"/>
+    <filterColumn colId="0">
+      <filters>
+        <filter val="PBI-110"/>
+        <filter val="PBI-091"/>
+        <filter val="PBI-111"/>
+        <filter val="PBI-105"/>
+        <filter val="PBI-096"/>
+        <filter val="PBI-106"/>
+        <filter val="PBI-107"/>
+        <filter val="PBI-088"/>
+        <filter val="PBI-108"/>
+        <filter val="PBI-109"/>
       </filters>
     </filterColumn>
     <extLst/>

</xml_diff>

<commit_message>
[PBI-067] Implement checklist access control, audit logging, and state-transition guards
</commit_message>
<xml_diff>
--- a/backlog/backlog.xlsx
+++ b/backlog/backlog.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="12420" windowHeight="4716"/>
+    <workbookView windowWidth="13548" windowHeight="4716"/>
   </bookViews>
   <sheets>
     <sheet name="backlog" sheetId="1" r:id="rId1"/>
@@ -773,144 +773,144 @@
     <t>Security;Compliance;Maintainability</t>
   </si>
   <si>
+    <t>Important: Story-level acceptance should not be marked Accepted/Done until PBI-083 is resolved and duplicate-prevention behavior is verified.</t>
+  </si>
+  <si>
+    <t>PBI-032</t>
+  </si>
+  <si>
+    <t>As an administrator, I want to define and maintain platform roles, so that access can be governed consistently</t>
+  </si>
+  <si>
+    <t>Context: role-based access requires a stable role catalogue before user assignment. Business problem: inconsistent role definitions weaken access governance. User role / actor: administrator. Expected behavior: administrator can create, update, and manage platform roles used for membership access control. Business value: establishes a reusable role model for secure access management. In scope: role creation, role update, role status management. Out of scope: user-role assignment and runtime access denial.</t>
+  </si>
+  <si>
+    <t>[ReqID: R03] Given an administrator defines a valid role, when the role is saved, then the platform stores the role for future assignment. | [ReqID: R03] Given a duplicate or invalid role definition is submitted, when save is attempted, then the platform rejects the change and returns a validation error.</t>
+  </si>
+  <si>
+    <t>DoR: Ready. PO Approval: Approved for Sprint 1 decomposition of PBI-003.</t>
+  </si>
+  <si>
+    <t>PBI-033</t>
+  </si>
+  <si>
+    <t>As an administrator, I want to assign platform roles to member users, so that each user can access only the functions required for their responsibilities</t>
+  </si>
+  <si>
+    <t>Context: once organizations and roles exist, users must be bound to those roles to support controlled access. Business problem: users without structured role assignment cannot be governed consistently. User role / actor: administrator. Expected behavior: administrator assigns, changes, or removes roles for users associated with member organizations. Business value: enables least-privilege access control. In scope: assign role, change role, remove role, membership validation. Out of scope: deactivation enforcement.</t>
+  </si>
+  <si>
+    <t>[ReqID: R03] Given a user belongs to a valid member organization and a valid role exists, when an administrator assigns the role, then the platform stores the assignment successfully. | [ReqID: R03] Given the user is not associated with a valid member organization or the role is invalid, when assignment is attempted, then the platform blocks the assignment and shows the reason.</t>
+  </si>
+  <si>
+    <t>PBI-003;PBI-031;PBI-032</t>
+  </si>
+  <si>
+    <t>PBI-034</t>
+  </si>
+  <si>
+    <t>As the platform, I want to block access for deactivated members, so that removed organizations and users cannot use protected functions</t>
+  </si>
+  <si>
+    <t>Context: membership and role management are incomplete without enforcement against deactivated members. Business problem: inactive members retaining access creates governance and security risk. User role / actor: system enforcement. Expected behavior: protected actions are denied when a member organization or user is deactivated. Business value: ensures access control reflects membership state. In scope: deactivation state check, denial of protected actions, error feedback. Out of scope: advanced non-repudiation analytics.</t>
+  </si>
+  <si>
+    <t>[ReqID: R03] Given a member organization or user is deactivated, when a protected action is attempted, then the platform denies access. | [ReqID: R03] Given an active member with a valid role attempts a protected action, when access is evaluated, then the platform allows the action to proceed.</t>
+  </si>
+  <si>
+    <t>Security;Compliance;Reliability</t>
+  </si>
+  <si>
+    <t>PBI-003;PBI-031;PBI-033</t>
+  </si>
+  <si>
+    <t>PBI-035</t>
+  </si>
+  <si>
+    <t>As a compliance coordinator, I want to submit a PLS item for Shariah review, so that governance starts from a formal and traceable request</t>
+  </si>
+  <si>
+    <t>Context: Shariah governance requires a formal starting point for review. Business problem: ad hoc review initiation makes approval workflow ambiguous and difficult to track. User role / actor: compliance coordinator. Expected behavior: coordinator submits a review request with the mandatory metadata for a PLS item. Business value: creates a controlled and traceable approval intake process. In scope: request creation, mandatory fields, initial workflow state. Out of scope: checklist completion and final decision.</t>
+  </si>
+  <si>
+    <t>[ReqID: R20] Given the required review-request data is complete, when the coordinator submits the request, then the platform creates a review record with initial Submitted status. | [ReqID: R20] Given mandatory review-request data is incomplete, when submission is attempted, then the platform blocks the request and shows validation errors.</t>
+  </si>
+  <si>
+    <t>Compliance;Audit;Security</t>
+  </si>
+  <si>
+    <t>DoR: Ready. PO Approval: Approved for Sprint 1 decomposition of PBI-020.</t>
+  </si>
+  <si>
+    <t>PBI-036</t>
+  </si>
+  <si>
+    <t>As a Shariah reviewer, I want to record the review checklist outcome, so that the basis of the governance decision is documented</t>
+  </si>
+  <si>
+    <t>Context: governance decisions require structured review evidence before approval can be finalized. Business problem: undocumented checklist completion weakens governance assurance. User role / actor: Shariah reviewer. Expected behavior: reviewer completes and saves the checklist findings for a submitted review item. Business value: makes the approval basis explicit and auditable. In scope: checklist completion, reviewer comments, review completion state. Out of scope: final approve reject conditional-approve transition.</t>
+  </si>
+  <si>
+    <t>[ReqID: R20] Given a submitted review item exists, when the reviewer completes the checklist with all required entries, then the platform stores the checklist outcome and reviewer comments. | [ReqID: R20] Given mandatory checklist entries are missing, when the reviewer attempts to save completion, then the platform blocks completion and shows validation errors.</t>
+  </si>
+  <si>
+    <t>PBI-020;PBI-035</t>
+  </si>
+  <si>
+    <t>PBI-037</t>
+  </si>
+  <si>
+    <t>As a Shariah reviewer, I want to record approve, reject, or conditional-approve decisions, so that governance outcomes are explicit and auditable</t>
+  </si>
+  <si>
+    <t>Context: the review workflow must end in a formal governance outcome. Business problem: without explicit decision capture, approval status cannot be relied upon. User role / actor: Shariah reviewer. Expected behavior: reviewer records the final decision with rationale or conditions where applicable. Business value: enables clear governance outcomes and later compliance verification. In scope: approve, reject, conditional approve, rationale capture, state transition. Out of scope: activation gating against PLS contract execution.</t>
+  </si>
+  <si>
+    <t>[ReqID: R20] Given a completed review checklist exists, when the reviewer records an approval decision, then the platform changes the item status to Approved and stores the decision metadata. | [ReqID: R20] Given the reviewer records a rejection or conditional approval, when the decision is saved, then the platform stores the rationale or conditions and updates the workflow state accordingly.</t>
+  </si>
+  <si>
+    <t>PBI-020;PBI-036</t>
+  </si>
+  <si>
+    <t>PBI-038</t>
+  </si>
+  <si>
+    <t>As a compliance coordinator, I want to view the current approval status and decision history, so that I can track governance progress and outcomes</t>
+  </si>
+  <si>
+    <t>Context: governance workflow participants need visibility into approval progress and results. Business problem: without a consolidated view, coordinators cannot follow up or confirm outcome state efficiently. User role / actor: compliance coordinator. Expected behavior: coordinator can view the latest status and prior review history of a PLS review item. Business value: improves workflow transparency and operational follow-up. In scope: status view, decision history, summary of review progression. Out of scope: regulator export and linkage to downstream contract execution.</t>
+  </si>
+  <si>
+    <t>[ReqID: R20] Given a review item exists, when the coordinator opens its details, then the platform displays the current approval status and prior review history. | [ReqID: R20] Given no final decision has been recorded yet, when the coordinator views the item, then the platform still shows the submitted and review-progress states without error.</t>
+  </si>
+  <si>
+    <t>Compliance;Audit;Usability;Security</t>
+  </si>
+  <si>
+    <t>PBI-020;PBI-035;PBI-037</t>
+  </si>
+  <si>
+    <t>PBI-039</t>
+  </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>Do define member organization schema, uniqueness rules, and membership status model</t>
+  </si>
+  <si>
+    <t>Action to be performed: define the member organization data model, required fields, uniqueness rules, and active or inactive lifecycle states. Why it is needed: downstream API, UI, and access-control tasks depend on stable data and state rules. Expected output: reviewed schema, validation rules, and request-response contract. Scope: entity fields, uniqueness rule, state values, API contract. Explicit exclusions: UI build and endpoint implementation.</t>
+  </si>
+  <si>
+    <t>[ReqID: R03] Given the schema draft is reviewed, when validation rules are checked, then required fields, uniqueness constraints, and status values are explicitly defined. | [ReqID: R03] Given downstream tasks consume the model, when implementation starts, then the request and response contract is stable enough for API and UI work.</t>
+  </si>
+  <si>
+    <t>Sprint 1</t>
+  </si>
+  <si>
     <t>Completed</t>
   </si>
   <si>
-    <t>Important: Story-level acceptance should not be marked Accepted/Done until PBI-083 is resolved and duplicate-prevention behavior is verified.</t>
-  </si>
-  <si>
-    <t>PBI-032</t>
-  </si>
-  <si>
-    <t>As an administrator, I want to define and maintain platform roles, so that access can be governed consistently</t>
-  </si>
-  <si>
-    <t>Context: role-based access requires a stable role catalogue before user assignment. Business problem: inconsistent role definitions weaken access governance. User role / actor: administrator. Expected behavior: administrator can create, update, and manage platform roles used for membership access control. Business value: establishes a reusable role model for secure access management. In scope: role creation, role update, role status management. Out of scope: user-role assignment and runtime access denial.</t>
-  </si>
-  <si>
-    <t>[ReqID: R03] Given an administrator defines a valid role, when the role is saved, then the platform stores the role for future assignment. | [ReqID: R03] Given a duplicate or invalid role definition is submitted, when save is attempted, then the platform rejects the change and returns a validation error.</t>
-  </si>
-  <si>
-    <t>DoR: Ready. PO Approval: Approved for Sprint 1 decomposition of PBI-003.</t>
-  </si>
-  <si>
-    <t>PBI-033</t>
-  </si>
-  <si>
-    <t>As an administrator, I want to assign platform roles to member users, so that each user can access only the functions required for their responsibilities</t>
-  </si>
-  <si>
-    <t>Context: once organizations and roles exist, users must be bound to those roles to support controlled access. Business problem: users without structured role assignment cannot be governed consistently. User role / actor: administrator. Expected behavior: administrator assigns, changes, or removes roles for users associated with member organizations. Business value: enables least-privilege access control. In scope: assign role, change role, remove role, membership validation. Out of scope: deactivation enforcement.</t>
-  </si>
-  <si>
-    <t>[ReqID: R03] Given a user belongs to a valid member organization and a valid role exists, when an administrator assigns the role, then the platform stores the assignment successfully. | [ReqID: R03] Given the user is not associated with a valid member organization or the role is invalid, when assignment is attempted, then the platform blocks the assignment and shows the reason.</t>
-  </si>
-  <si>
-    <t>PBI-003;PBI-031;PBI-032</t>
-  </si>
-  <si>
-    <t>PBI-034</t>
-  </si>
-  <si>
-    <t>As the platform, I want to block access for deactivated members, so that removed organizations and users cannot use protected functions</t>
-  </si>
-  <si>
-    <t>Context: membership and role management are incomplete without enforcement against deactivated members. Business problem: inactive members retaining access creates governance and security risk. User role / actor: system enforcement. Expected behavior: protected actions are denied when a member organization or user is deactivated. Business value: ensures access control reflects membership state. In scope: deactivation state check, denial of protected actions, error feedback. Out of scope: advanced non-repudiation analytics.</t>
-  </si>
-  <si>
-    <t>[ReqID: R03] Given a member organization or user is deactivated, when a protected action is attempted, then the platform denies access. | [ReqID: R03] Given an active member with a valid role attempts a protected action, when access is evaluated, then the platform allows the action to proceed.</t>
-  </si>
-  <si>
-    <t>Security;Compliance;Reliability</t>
-  </si>
-  <si>
-    <t>PBI-003;PBI-031;PBI-033</t>
-  </si>
-  <si>
-    <t>PBI-035</t>
-  </si>
-  <si>
-    <t>As a compliance coordinator, I want to submit a PLS item for Shariah review, so that governance starts from a formal and traceable request</t>
-  </si>
-  <si>
-    <t>Context: Shariah governance requires a formal starting point for review. Business problem: ad hoc review initiation makes approval workflow ambiguous and difficult to track. User role / actor: compliance coordinator. Expected behavior: coordinator submits a review request with the mandatory metadata for a PLS item. Business value: creates a controlled and traceable approval intake process. In scope: request creation, mandatory fields, initial workflow state. Out of scope: checklist completion and final decision.</t>
-  </si>
-  <si>
-    <t>[ReqID: R20] Given the required review-request data is complete, when the coordinator submits the request, then the platform creates a review record with initial Submitted status. | [ReqID: R20] Given mandatory review-request data is incomplete, when submission is attempted, then the platform blocks the request and shows validation errors.</t>
-  </si>
-  <si>
-    <t>Compliance;Audit;Security</t>
-  </si>
-  <si>
-    <t>DoR: Ready. PO Approval: Approved for Sprint 1 decomposition of PBI-020.</t>
-  </si>
-  <si>
-    <t>PBI-036</t>
-  </si>
-  <si>
-    <t>As a Shariah reviewer, I want to record the review checklist outcome, so that the basis of the governance decision is documented</t>
-  </si>
-  <si>
-    <t>Context: governance decisions require structured review evidence before approval can be finalized. Business problem: undocumented checklist completion weakens governance assurance. User role / actor: Shariah reviewer. Expected behavior: reviewer completes and saves the checklist findings for a submitted review item. Business value: makes the approval basis explicit and auditable. In scope: checklist completion, reviewer comments, review completion state. Out of scope: final approve reject conditional-approve transition.</t>
-  </si>
-  <si>
-    <t>[ReqID: R20] Given a submitted review item exists, when the reviewer completes the checklist with all required entries, then the platform stores the checklist outcome and reviewer comments. | [ReqID: R20] Given mandatory checklist entries are missing, when the reviewer attempts to save completion, then the platform blocks completion and shows validation errors.</t>
-  </si>
-  <si>
-    <t>PBI-020;PBI-035</t>
-  </si>
-  <si>
-    <t>PBI-037</t>
-  </si>
-  <si>
-    <t>As a Shariah reviewer, I want to record approve, reject, or conditional-approve decisions, so that governance outcomes are explicit and auditable</t>
-  </si>
-  <si>
-    <t>Context: the review workflow must end in a formal governance outcome. Business problem: without explicit decision capture, approval status cannot be relied upon. User role / actor: Shariah reviewer. Expected behavior: reviewer records the final decision with rationale or conditions where applicable. Business value: enables clear governance outcomes and later compliance verification. In scope: approve, reject, conditional approve, rationale capture, state transition. Out of scope: activation gating against PLS contract execution.</t>
-  </si>
-  <si>
-    <t>[ReqID: R20] Given a completed review checklist exists, when the reviewer records an approval decision, then the platform changes the item status to Approved and stores the decision metadata. | [ReqID: R20] Given the reviewer records a rejection or conditional approval, when the decision is saved, then the platform stores the rationale or conditions and updates the workflow state accordingly.</t>
-  </si>
-  <si>
-    <t>PBI-020;PBI-036</t>
-  </si>
-  <si>
-    <t>PBI-038</t>
-  </si>
-  <si>
-    <t>As a compliance coordinator, I want to view the current approval status and decision history, so that I can track governance progress and outcomes</t>
-  </si>
-  <si>
-    <t>Context: governance workflow participants need visibility into approval progress and results. Business problem: without a consolidated view, coordinators cannot follow up or confirm outcome state efficiently. User role / actor: compliance coordinator. Expected behavior: coordinator can view the latest status and prior review history of a PLS review item. Business value: improves workflow transparency and operational follow-up. In scope: status view, decision history, summary of review progression. Out of scope: regulator export and linkage to downstream contract execution.</t>
-  </si>
-  <si>
-    <t>[ReqID: R20] Given a review item exists, when the coordinator opens its details, then the platform displays the current approval status and prior review history. | [ReqID: R20] Given no final decision has been recorded yet, when the coordinator views the item, then the platform still shows the submitted and review-progress states without error.</t>
-  </si>
-  <si>
-    <t>Compliance;Audit;Usability;Security</t>
-  </si>
-  <si>
-    <t>PBI-020;PBI-035;PBI-037</t>
-  </si>
-  <si>
-    <t>PBI-039</t>
-  </si>
-  <si>
-    <t>Task</t>
-  </si>
-  <si>
-    <t>Do define member organization schema, uniqueness rules, and membership status model</t>
-  </si>
-  <si>
-    <t>Action to be performed: define the member organization data model, required fields, uniqueness rules, and active or inactive lifecycle states. Why it is needed: downstream API, UI, and access-control tasks depend on stable data and state rules. Expected output: reviewed schema, validation rules, and request-response contract. Scope: entity fields, uniqueness rule, state values, API contract. Explicit exclusions: UI build and endpoint implementation.</t>
-  </si>
-  <si>
-    <t>[ReqID: R03] Given the schema draft is reviewed, when validation rules are checked, then required fields, uniqueness constraints, and status values are explicitly defined. | [ReqID: R03] Given downstream tasks consume the model, when implementation starts, then the request and response contract is stable enough for API and UI work.</t>
-  </si>
-  <si>
-    <t>Sprint 1</t>
-  </si>
-  <si>
     <t>Important: Covers PBI-031 AC1 and AC2. Shared prerequisite for PBI-040 and PBI-041. Evidence: schema note, validation matrix, API contract.</t>
   </si>
   <si>
@@ -953,7 +953,7 @@
     <t>Blocked</t>
   </si>
   <si>
-    <t>PBI-039;PBI-040;PBI-079;PBI-080;PBI-081;PBI-082;PBI-083</t>
+    <t>PBI-031;PBI-039;PBI-040;PBI-079;PBI-080;PBI-081;PBI-082;PBI-083</t>
   </si>
   <si>
     <t>Important: Covers PBI-031 AC1 and AC2. Can run in parallel with PBI-040 after contract is stable. Evidence: screenshots, functional checks. When resumed, this task must consume the backend duplicate-conflict response semantics introduced by PBI-083.</t>
@@ -5014,30 +5014,30 @@
         <v>44</v>
       </c>
       <c r="L32" t="s">
-        <v>247</v>
+        <v>45</v>
       </c>
       <c r="M32" t="s">
         <v>38</v>
       </c>
       <c r="N32" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="33" hidden="1" spans="1:14">
       <c r="A33" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B33" t="s">
         <v>242</v>
       </c>
       <c r="C33" t="s">
+        <v>249</v>
+      </c>
+      <c r="D33" t="s">
         <v>250</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
         <v>251</v>
-      </c>
-      <c r="E33" t="s">
-        <v>252</v>
       </c>
       <c r="F33" t="s">
         <v>42</v>
@@ -5061,24 +5061,24 @@
         <v>38</v>
       </c>
       <c r="N33" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="34" hidden="1" spans="1:14">
       <c r="A34" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B34" t="s">
         <v>242</v>
       </c>
       <c r="C34" t="s">
+        <v>254</v>
+      </c>
+      <c r="D34" t="s">
         <v>255</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
         <v>256</v>
-      </c>
-      <c r="E34" t="s">
-        <v>257</v>
       </c>
       <c r="F34" t="s">
         <v>42</v>
@@ -5099,33 +5099,33 @@
         <v>45</v>
       </c>
       <c r="M34" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="N34" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="35" hidden="1" spans="1:14">
       <c r="A35" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B35" t="s">
         <v>242</v>
       </c>
       <c r="C35" t="s">
+        <v>259</v>
+      </c>
+      <c r="D35" t="s">
         <v>260</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
         <v>261</v>
-      </c>
-      <c r="E35" t="s">
-        <v>262</v>
       </c>
       <c r="F35" t="s">
         <v>42</v>
       </c>
       <c r="G35" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="H35">
         <v>5</v>
@@ -5140,33 +5140,33 @@
         <v>35</v>
       </c>
       <c r="M35" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="N35" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="36" hidden="1" spans="1:14">
       <c r="A36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B36" t="s">
         <v>242</v>
       </c>
       <c r="C36" t="s">
+        <v>265</v>
+      </c>
+      <c r="D36" t="s">
         <v>266</v>
       </c>
-      <c r="D36" t="s">
+      <c r="E36" t="s">
         <v>267</v>
-      </c>
-      <c r="E36" t="s">
-        <v>268</v>
       </c>
       <c r="F36" t="s">
         <v>170</v>
       </c>
       <c r="G36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="H36">
         <v>3</v>
@@ -5184,30 +5184,30 @@
         <v>166</v>
       </c>
       <c r="N36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="37" hidden="1" spans="1:14">
       <c r="A37" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B37" t="s">
         <v>242</v>
       </c>
       <c r="C37" t="s">
+        <v>271</v>
+      </c>
+      <c r="D37" t="s">
         <v>272</v>
       </c>
-      <c r="D37" t="s">
+      <c r="E37" t="s">
         <v>273</v>
-      </c>
-      <c r="E37" t="s">
-        <v>274</v>
       </c>
       <c r="F37" t="s">
         <v>170</v>
       </c>
       <c r="G37" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="H37">
         <v>3</v>
@@ -5222,33 +5222,33 @@
         <v>35</v>
       </c>
       <c r="M37" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N37" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="38" hidden="1" spans="1:14">
       <c r="A38" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B38" t="s">
         <v>242</v>
       </c>
       <c r="C38" t="s">
+        <v>276</v>
+      </c>
+      <c r="D38" t="s">
         <v>277</v>
       </c>
-      <c r="D38" t="s">
+      <c r="E38" t="s">
         <v>278</v>
-      </c>
-      <c r="E38" t="s">
-        <v>279</v>
       </c>
       <c r="F38" t="s">
         <v>170</v>
       </c>
       <c r="G38" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="H38">
         <v>3</v>
@@ -5263,33 +5263,33 @@
         <v>35</v>
       </c>
       <c r="M38" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="N38" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="39" hidden="1" spans="1:14">
       <c r="A39" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B39" t="s">
         <v>242</v>
       </c>
       <c r="C39" t="s">
+        <v>281</v>
+      </c>
+      <c r="D39" t="s">
         <v>282</v>
       </c>
-      <c r="D39" t="s">
+      <c r="E39" t="s">
         <v>283</v>
-      </c>
-      <c r="E39" t="s">
-        <v>284</v>
       </c>
       <c r="F39" t="s">
         <v>170</v>
       </c>
       <c r="G39" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="H39">
         <v>2</v>
@@ -5304,27 +5304,27 @@
         <v>35</v>
       </c>
       <c r="M39" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="N39" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="40" hidden="1" spans="1:14">
       <c r="A40" t="s">
+        <v>286</v>
+      </c>
+      <c r="B40" t="s">
         <v>287</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
         <v>288</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40" t="s">
         <v>289</v>
       </c>
-      <c r="D40" t="s">
+      <c r="E40" t="s">
         <v>290</v>
-      </c>
-      <c r="E40" t="s">
-        <v>291</v>
       </c>
       <c r="F40" t="s">
         <v>42</v>
@@ -5342,10 +5342,10 @@
         <v>44</v>
       </c>
       <c r="K40" t="s">
+        <v>291</v>
+      </c>
+      <c r="L40" t="s">
         <v>292</v>
-      </c>
-      <c r="L40" t="s">
-        <v>247</v>
       </c>
       <c r="M40" t="s">
         <v>241</v>
@@ -5359,7 +5359,7 @@
         <v>294</v>
       </c>
       <c r="B41" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C41" t="s">
         <v>295</v>
@@ -5374,7 +5374,7 @@
         <v>42</v>
       </c>
       <c r="G41" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="H41">
         <v>3</v>
@@ -5386,10 +5386,10 @@
         <v>61</v>
       </c>
       <c r="K41" t="s">
+        <v>291</v>
+      </c>
+      <c r="L41" t="s">
         <v>292</v>
-      </c>
-      <c r="L41" t="s">
-        <v>247</v>
       </c>
       <c r="M41" t="s">
         <v>298</v>
@@ -5403,7 +5403,7 @@
         <v>300</v>
       </c>
       <c r="B42" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C42" t="s">
         <v>301</v>
@@ -5447,7 +5447,7 @@
         <v>309</v>
       </c>
       <c r="B43" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C43" t="s">
         <v>310</v>
@@ -5474,10 +5474,10 @@
         <v>95</v>
       </c>
       <c r="K43" t="s">
+        <v>291</v>
+      </c>
+      <c r="L43" t="s">
         <v>292</v>
-      </c>
-      <c r="L43" t="s">
-        <v>247</v>
       </c>
       <c r="M43" t="s">
         <v>314</v>
@@ -5491,7 +5491,7 @@
         <v>316</v>
       </c>
       <c r="B44" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C44" t="s">
         <v>317</v>
@@ -5518,10 +5518,10 @@
         <v>121</v>
       </c>
       <c r="K44" t="s">
+        <v>291</v>
+      </c>
+      <c r="L44" t="s">
         <v>292</v>
-      </c>
-      <c r="L44" t="s">
-        <v>247</v>
       </c>
       <c r="M44" t="s">
         <v>321</v>
@@ -5535,7 +5535,7 @@
         <v>323</v>
       </c>
       <c r="B45" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C45" t="s">
         <v>324</v>
@@ -5562,13 +5562,13 @@
         <v>44</v>
       </c>
       <c r="K45" t="s">
+        <v>291</v>
+      </c>
+      <c r="L45" t="s">
         <v>292</v>
       </c>
-      <c r="L45" t="s">
-        <v>247</v>
-      </c>
       <c r="M45" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="N45" t="s">
         <v>327</v>
@@ -5579,7 +5579,7 @@
         <v>328</v>
       </c>
       <c r="B46" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C46" t="s">
         <v>329</v>
@@ -5594,7 +5594,7 @@
         <v>42</v>
       </c>
       <c r="G46" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="H46">
         <v>3</v>
@@ -5606,10 +5606,10 @@
         <v>61</v>
       </c>
       <c r="K46" t="s">
+        <v>291</v>
+      </c>
+      <c r="L46" t="s">
         <v>292</v>
-      </c>
-      <c r="L46" t="s">
-        <v>247</v>
       </c>
       <c r="M46" t="s">
         <v>332</v>
@@ -5623,7 +5623,7 @@
         <v>334</v>
       </c>
       <c r="B47" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C47" t="s">
         <v>335</v>
@@ -5667,7 +5667,7 @@
         <v>340</v>
       </c>
       <c r="B48" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C48" t="s">
         <v>341</v>
@@ -5694,10 +5694,10 @@
         <v>95</v>
       </c>
       <c r="K48" t="s">
+        <v>291</v>
+      </c>
+      <c r="L48" t="s">
         <v>292</v>
-      </c>
-      <c r="L48" t="s">
-        <v>247</v>
       </c>
       <c r="M48" t="s">
         <v>344</v>
@@ -5711,7 +5711,7 @@
         <v>346</v>
       </c>
       <c r="B49" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C49" t="s">
         <v>347</v>
@@ -5752,7 +5752,7 @@
         <v>352</v>
       </c>
       <c r="B50" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C50" t="s">
         <v>353</v>
@@ -5779,10 +5779,10 @@
         <v>356</v>
       </c>
       <c r="K50" t="s">
+        <v>291</v>
+      </c>
+      <c r="L50" t="s">
         <v>292</v>
-      </c>
-      <c r="L50" t="s">
-        <v>247</v>
       </c>
       <c r="M50" t="s">
         <v>357</v>
@@ -5796,7 +5796,7 @@
         <v>359</v>
       </c>
       <c r="B51" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C51" t="s">
         <v>360</v>
@@ -5826,7 +5826,7 @@
         <v>363</v>
       </c>
       <c r="L51" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M51" t="s">
         <v>364</v>
@@ -5840,7 +5840,7 @@
         <v>366</v>
       </c>
       <c r="B52" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C52" t="s">
         <v>367</v>
@@ -5884,7 +5884,7 @@
         <v>372</v>
       </c>
       <c r="B53" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C53" t="s">
         <v>373</v>
@@ -5914,7 +5914,7 @@
         <v>363</v>
       </c>
       <c r="L53" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M53" t="s">
         <v>376</v>
@@ -5928,7 +5928,7 @@
         <v>378</v>
       </c>
       <c r="B54" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C54" t="s">
         <v>379</v>
@@ -5958,7 +5958,7 @@
         <v>363</v>
       </c>
       <c r="L54" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M54" t="s">
         <v>382</v>
@@ -5972,7 +5972,7 @@
         <v>384</v>
       </c>
       <c r="B55" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C55" t="s">
         <v>385</v>
@@ -6016,7 +6016,7 @@
         <v>390</v>
       </c>
       <c r="B56" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C56" t="s">
         <v>391</v>
@@ -6031,7 +6031,7 @@
         <v>42</v>
       </c>
       <c r="G56" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="H56">
         <v>3</v>
@@ -6060,7 +6060,7 @@
         <v>396</v>
       </c>
       <c r="B57" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C57" t="s">
         <v>397</v>
@@ -6104,7 +6104,7 @@
         <v>403</v>
       </c>
       <c r="B58" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C58" t="s">
         <v>404</v>
@@ -6148,7 +6148,7 @@
         <v>410</v>
       </c>
       <c r="B59" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C59" t="s">
         <v>411</v>
@@ -6189,7 +6189,7 @@
         <v>416</v>
       </c>
       <c r="B60" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C60" t="s">
         <v>417</v>
@@ -6216,13 +6216,13 @@
         <v>33</v>
       </c>
       <c r="K60" t="s">
+        <v>291</v>
+      </c>
+      <c r="L60" t="s">
         <v>292</v>
       </c>
-      <c r="L60" t="s">
-        <v>247</v>
-      </c>
       <c r="M60" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="N60" t="s">
         <v>421</v>
@@ -6233,7 +6233,7 @@
         <v>422</v>
       </c>
       <c r="B61" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C61" t="s">
         <v>423</v>
@@ -6260,10 +6260,10 @@
         <v>61</v>
       </c>
       <c r="K61" t="s">
+        <v>291</v>
+      </c>
+      <c r="L61" t="s">
         <v>292</v>
-      </c>
-      <c r="L61" t="s">
-        <v>247</v>
       </c>
       <c r="M61" t="s">
         <v>427</v>
@@ -6277,7 +6277,7 @@
         <v>429</v>
       </c>
       <c r="B62" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C62" t="s">
         <v>430</v>
@@ -6321,7 +6321,7 @@
         <v>435</v>
       </c>
       <c r="B63" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C63" t="s">
         <v>436</v>
@@ -6336,7 +6336,7 @@
         <v>170</v>
       </c>
       <c r="G63" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="H63">
         <v>2</v>
@@ -6348,10 +6348,10 @@
         <v>95</v>
       </c>
       <c r="K63" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="L63" t="s">
-        <v>247</v>
+        <v>45</v>
       </c>
       <c r="M63" t="s">
         <v>439</v>
@@ -6365,7 +6365,7 @@
         <v>441</v>
       </c>
       <c r="B64" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C64" t="s">
         <v>442</v>
@@ -6401,12 +6401,12 @@
         <v>446</v>
       </c>
     </row>
-    <row r="65" hidden="1" spans="1:14">
+    <row r="65" spans="1:14">
       <c r="A65" t="s">
         <v>447</v>
       </c>
       <c r="B65" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C65" t="s">
         <v>448</v>
@@ -6436,7 +6436,7 @@
         <v>363</v>
       </c>
       <c r="L65" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M65" t="s">
         <v>451</v>
@@ -6445,12 +6445,12 @@
         <v>452</v>
       </c>
     </row>
-    <row r="66" hidden="1" spans="1:14">
+    <row r="66" spans="1:14">
       <c r="A66" t="s">
         <v>453</v>
       </c>
       <c r="B66" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C66" t="s">
         <v>454</v>
@@ -6480,7 +6480,7 @@
         <v>363</v>
       </c>
       <c r="L66" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M66" t="s">
         <v>457</v>
@@ -6494,7 +6494,7 @@
         <v>459</v>
       </c>
       <c r="B67" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C67" t="s">
         <v>460</v>
@@ -6533,12 +6533,12 @@
         <v>464</v>
       </c>
     </row>
-    <row r="68" hidden="1" spans="1:14">
+    <row r="68" spans="1:14">
       <c r="A68" t="s">
         <v>465</v>
       </c>
       <c r="B68" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C68" t="s">
         <v>466</v>
@@ -6553,7 +6553,7 @@
         <v>170</v>
       </c>
       <c r="G68" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="H68">
         <v>2</v>
@@ -6568,7 +6568,7 @@
         <v>363</v>
       </c>
       <c r="L68" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M68" t="s">
         <v>469</v>
@@ -6582,7 +6582,7 @@
         <v>471</v>
       </c>
       <c r="B69" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C69" t="s">
         <v>472</v>
@@ -6618,12 +6618,12 @@
         <v>476</v>
       </c>
     </row>
-    <row r="70" hidden="1" spans="1:14">
+    <row r="70" spans="1:14">
       <c r="A70" t="s">
         <v>477</v>
       </c>
       <c r="B70" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C70" t="s">
         <v>478</v>
@@ -6653,7 +6653,7 @@
         <v>363</v>
       </c>
       <c r="L70" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M70" t="s">
         <v>481</v>
@@ -6662,12 +6662,12 @@
         <v>482</v>
       </c>
     </row>
-    <row r="71" hidden="1" spans="1:14">
+    <row r="71" spans="1:14">
       <c r="A71" t="s">
         <v>483</v>
       </c>
       <c r="B71" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C71" t="s">
         <v>484</v>
@@ -6697,7 +6697,7 @@
         <v>363</v>
       </c>
       <c r="L71" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M71" t="s">
         <v>488</v>
@@ -6711,7 +6711,7 @@
         <v>490</v>
       </c>
       <c r="B72" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C72" t="s">
         <v>491</v>
@@ -6750,12 +6750,12 @@
         <v>495</v>
       </c>
     </row>
-    <row r="73" hidden="1" spans="1:14">
+    <row r="73" spans="1:14">
       <c r="A73" t="s">
         <v>496</v>
       </c>
       <c r="B73" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C73" t="s">
         <v>497</v>
@@ -6770,7 +6770,7 @@
         <v>170</v>
       </c>
       <c r="G73" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="H73">
         <v>2</v>
@@ -6785,7 +6785,7 @@
         <v>363</v>
       </c>
       <c r="L73" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M73" t="s">
         <v>500</v>
@@ -6799,7 +6799,7 @@
         <v>502</v>
       </c>
       <c r="B74" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C74" t="s">
         <v>503</v>
@@ -6835,12 +6835,12 @@
         <v>507</v>
       </c>
     </row>
-    <row r="75" hidden="1" spans="1:14">
+    <row r="75" spans="1:14">
       <c r="A75" t="s">
         <v>508</v>
       </c>
       <c r="B75" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C75" t="s">
         <v>509</v>
@@ -6870,7 +6870,7 @@
         <v>363</v>
       </c>
       <c r="L75" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M75" t="s">
         <v>513</v>
@@ -6879,12 +6879,12 @@
         <v>514</v>
       </c>
     </row>
-    <row r="76" hidden="1" spans="1:14">
+    <row r="76" spans="1:14">
       <c r="A76" t="s">
         <v>515</v>
       </c>
       <c r="B76" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C76" t="s">
         <v>516</v>
@@ -6914,7 +6914,7 @@
         <v>363</v>
       </c>
       <c r="L76" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M76" t="s">
         <v>520</v>
@@ -6928,7 +6928,7 @@
         <v>522</v>
       </c>
       <c r="B77" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C77" t="s">
         <v>523</v>
@@ -6972,7 +6972,7 @@
         <v>528</v>
       </c>
       <c r="B78" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C78" t="s">
         <v>529</v>
@@ -6987,7 +6987,7 @@
         <v>170</v>
       </c>
       <c r="G78" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="H78">
         <v>2</v>
@@ -7013,7 +7013,7 @@
         <v>534</v>
       </c>
       <c r="B79" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C79" t="s">
         <v>535</v>
@@ -7142,7 +7142,7 @@
         <v>553</v>
       </c>
       <c r="B82" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C82" t="s">
         <v>554</v>
@@ -7186,7 +7186,7 @@
         <v>560</v>
       </c>
       <c r="B83" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C83" t="s">
         <v>561</v>
@@ -7260,7 +7260,7 @@
         <v>363</v>
       </c>
       <c r="L84" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M84" t="s">
         <v>572</v>
@@ -7304,7 +7304,7 @@
         <v>363</v>
       </c>
       <c r="L85" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M85" t="s">
         <v>359</v>
@@ -7348,7 +7348,7 @@
         <v>363</v>
       </c>
       <c r="L86" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M86" t="s">
         <v>574</v>
@@ -7392,7 +7392,7 @@
         <v>363</v>
       </c>
       <c r="L87" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M87" t="s">
         <v>24</v>
@@ -7445,12 +7445,12 @@
         <v>598</v>
       </c>
     </row>
-    <row r="89" spans="1:14">
+    <row r="89" hidden="1" spans="1:14">
       <c r="A89" t="s">
         <v>599</v>
       </c>
       <c r="B89" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C89" t="s">
         <v>600</v>
@@ -7480,7 +7480,7 @@
         <v>363</v>
       </c>
       <c r="L89" t="s">
-        <v>45</v>
+        <v>292</v>
       </c>
       <c r="M89" t="s">
         <v>603</v>
@@ -7489,7 +7489,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="90" hidden="1" spans="1:14">
+    <row r="90" spans="1:14">
       <c r="A90" t="s">
         <v>605</v>
       </c>
@@ -7524,7 +7524,7 @@
         <v>305</v>
       </c>
       <c r="L90" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M90" t="s">
         <v>24</v>
@@ -7568,7 +7568,7 @@
         <v>363</v>
       </c>
       <c r="L91" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M91" t="s">
         <v>24</v>
@@ -7577,7 +7577,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="92" spans="1:14">
+    <row r="92" hidden="1" spans="1:14">
       <c r="A92" t="s">
         <v>619</v>
       </c>
@@ -7656,7 +7656,7 @@
         <v>363</v>
       </c>
       <c r="L93" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M93" t="s">
         <v>24</v>
@@ -7670,7 +7670,7 @@
         <v>633</v>
       </c>
       <c r="B94" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C94" t="s">
         <v>634</v>
@@ -7700,7 +7700,7 @@
         <v>363</v>
       </c>
       <c r="L94" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M94" t="s">
         <v>24</v>
@@ -7714,7 +7714,7 @@
         <v>639</v>
       </c>
       <c r="B95" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C95" t="s">
         <v>640</v>
@@ -7744,7 +7744,7 @@
         <v>363</v>
       </c>
       <c r="L95" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M95" t="s">
         <v>644</v>
@@ -7797,12 +7797,12 @@
         <v>651</v>
       </c>
     </row>
-    <row r="97" spans="1:14">
+    <row r="97" hidden="1" spans="1:14">
       <c r="A97" t="s">
         <v>652</v>
       </c>
       <c r="B97" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C97" t="s">
         <v>653</v>
@@ -7832,7 +7832,7 @@
         <v>363</v>
       </c>
       <c r="L97" t="s">
-        <v>45</v>
+        <v>292</v>
       </c>
       <c r="M97" t="s">
         <v>656</v>
@@ -7846,7 +7846,7 @@
         <v>658</v>
       </c>
       <c r="B98" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C98" t="s">
         <v>659</v>
@@ -7876,7 +7876,7 @@
         <v>363</v>
       </c>
       <c r="L98" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M98" t="s">
         <v>24</v>
@@ -7890,7 +7890,7 @@
         <v>665</v>
       </c>
       <c r="B99" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C99" t="s">
         <v>666</v>
@@ -7920,7 +7920,7 @@
         <v>363</v>
       </c>
       <c r="L99" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M99" t="s">
         <v>670</v>
@@ -7934,7 +7934,7 @@
         <v>672</v>
       </c>
       <c r="B100" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C100" t="s">
         <v>673</v>
@@ -7964,7 +7964,7 @@
         <v>363</v>
       </c>
       <c r="L100" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M100" t="s">
         <v>677</v>
@@ -7978,7 +7978,7 @@
         <v>679</v>
       </c>
       <c r="B101" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C101" t="s">
         <v>680</v>
@@ -8008,7 +8008,7 @@
         <v>363</v>
       </c>
       <c r="L101" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M101" t="s">
         <v>684</v>
@@ -8022,7 +8022,7 @@
         <v>686</v>
       </c>
       <c r="B102" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C102" t="s">
         <v>687</v>
@@ -8052,7 +8052,7 @@
         <v>363</v>
       </c>
       <c r="L102" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M102" t="s">
         <v>691</v>
@@ -8066,7 +8066,7 @@
         <v>693</v>
       </c>
       <c r="B103" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C103" t="s">
         <v>694</v>
@@ -8096,7 +8096,7 @@
         <v>363</v>
       </c>
       <c r="L103" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M103" t="s">
         <v>698</v>
@@ -8110,7 +8110,7 @@
         <v>700</v>
       </c>
       <c r="B104" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C104" t="s">
         <v>701</v>
@@ -8140,7 +8140,7 @@
         <v>363</v>
       </c>
       <c r="L104" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M104" t="s">
         <v>705</v>
@@ -8154,7 +8154,7 @@
         <v>707</v>
       </c>
       <c r="B105" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C105" t="s">
         <v>708</v>
@@ -8184,7 +8184,7 @@
         <v>363</v>
       </c>
       <c r="L105" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M105" t="s">
         <v>711</v>
@@ -8193,12 +8193,12 @@
         <v>712</v>
       </c>
     </row>
-    <row r="106" spans="1:14">
+    <row r="106" hidden="1" spans="1:14">
       <c r="A106" t="s">
         <v>713</v>
       </c>
       <c r="B106" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C106" t="s">
         <v>714</v>
@@ -8228,7 +8228,7 @@
         <v>363</v>
       </c>
       <c r="L106" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M106" t="s">
         <v>586</v>
@@ -8237,12 +8237,12 @@
         <v>718</v>
       </c>
     </row>
-    <row r="107" spans="1:14">
+    <row r="107" hidden="1" spans="1:14">
       <c r="A107" t="s">
         <v>719</v>
       </c>
       <c r="B107" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C107" t="s">
         <v>720</v>
@@ -8272,7 +8272,7 @@
         <v>363</v>
       </c>
       <c r="L107" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M107" t="s">
         <v>724</v>
@@ -8281,12 +8281,12 @@
         <v>725</v>
       </c>
     </row>
-    <row r="108" spans="1:14">
+    <row r="108" hidden="1" spans="1:14">
       <c r="A108" t="s">
         <v>726</v>
       </c>
       <c r="B108" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C108" t="s">
         <v>727</v>
@@ -8316,7 +8316,7 @@
         <v>363</v>
       </c>
       <c r="L108" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M108" t="s">
         <v>731</v>
@@ -8325,12 +8325,12 @@
         <v>732</v>
       </c>
     </row>
-    <row r="109" spans="1:14">
+    <row r="109" hidden="1" spans="1:14">
       <c r="A109" t="s">
         <v>733</v>
       </c>
       <c r="B109" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C109" t="s">
         <v>734</v>
@@ -8360,7 +8360,7 @@
         <v>363</v>
       </c>
       <c r="L109" t="s">
-        <v>45</v>
+        <v>292</v>
       </c>
       <c r="M109" t="s">
         <v>738</v>
@@ -8369,12 +8369,12 @@
         <v>739</v>
       </c>
     </row>
-    <row r="110" spans="1:14">
+    <row r="110" hidden="1" spans="1:14">
       <c r="A110" t="s">
         <v>740</v>
       </c>
       <c r="B110" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C110" t="s">
         <v>741</v>
@@ -8404,7 +8404,7 @@
         <v>363</v>
       </c>
       <c r="L110" t="s">
-        <v>45</v>
+        <v>292</v>
       </c>
       <c r="M110" t="s">
         <v>745</v>
@@ -8413,12 +8413,12 @@
         <v>746</v>
       </c>
     </row>
-    <row r="111" spans="1:14">
+    <row r="111" hidden="1" spans="1:14">
       <c r="A111" t="s">
         <v>747</v>
       </c>
       <c r="B111" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C111" t="s">
         <v>748</v>
@@ -8448,7 +8448,7 @@
         <v>363</v>
       </c>
       <c r="L111" t="s">
-        <v>45</v>
+        <v>292</v>
       </c>
       <c r="M111" t="s">
         <v>612</v>
@@ -8457,12 +8457,12 @@
         <v>752</v>
       </c>
     </row>
-    <row r="112" spans="1:14">
+    <row r="112" hidden="1" spans="1:14">
       <c r="A112" t="s">
         <v>753</v>
       </c>
       <c r="B112" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C112" t="s">
         <v>754</v>
@@ -8492,7 +8492,7 @@
         <v>363</v>
       </c>
       <c r="L112" t="s">
-        <v>45</v>
+        <v>292</v>
       </c>
       <c r="M112" t="s">
         <v>758</v>
@@ -8506,7 +8506,7 @@
         <v>760</v>
       </c>
       <c r="B113" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C113" t="s">
         <v>761</v>
@@ -8550,7 +8550,7 @@
         <v>766</v>
       </c>
       <c r="B114" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C114" t="s">
         <v>767</v>
@@ -8594,7 +8594,7 @@
         <v>773</v>
       </c>
       <c r="B115" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C115" t="s">
         <v>774</v>
@@ -8638,7 +8638,7 @@
         <v>780</v>
       </c>
       <c r="B116" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C116" t="s">
         <v>781</v>
@@ -8668,7 +8668,7 @@
         <v>363</v>
       </c>
       <c r="L116" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M116" t="s">
         <v>626</v>
@@ -8682,7 +8682,7 @@
         <v>786</v>
       </c>
       <c r="B117" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C117" t="s">
         <v>787</v>
@@ -8712,7 +8712,7 @@
         <v>363</v>
       </c>
       <c r="L117" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="M117" t="s">
         <v>791</v>
@@ -8726,7 +8726,7 @@
         <v>793</v>
       </c>
       <c r="B118" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C118" t="s">
         <v>794</v>
@@ -8770,7 +8770,7 @@
         <v>799</v>
       </c>
       <c r="B119" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C119" t="s">
         <v>800</v>
@@ -8862,16 +8862,15 @@
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:N121" etc:filterBottomFollowUsedRange="0">
     <filterColumn colId="0">
       <filters>
-        <filter val="PBI-110"/>
-        <filter val="PBI-091"/>
-        <filter val="PBI-111"/>
-        <filter val="PBI-105"/>
-        <filter val="PBI-096"/>
-        <filter val="PBI-106"/>
-        <filter val="PBI-107"/>
-        <filter val="PBI-088"/>
-        <filter val="PBI-108"/>
-        <filter val="PBI-109"/>
+        <filter val="PBI-070"/>
+        <filter val="PBI-072"/>
+        <filter val="PBI-064"/>
+        <filter val="PBI-074"/>
+        <filter val="PBI-065"/>
+        <filter val="PBI-075"/>
+        <filter val="PBI-067"/>
+        <filter val="PBI-069"/>
+        <filter val="PBI-089"/>
       </filters>
     </filterColumn>
     <extLst/>
@@ -8900,7 +8899,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L$1:L$1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L67 L68 L69 L72 L73 L74 L90 L1:L64 L65:L66 L70:L71 L75:L76 L77:L89 L91:L1048576">
       <formula1>"Planned,Deferred,In-Progress,Completed,Draft,Blocked"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
[PBI-089] Enable modular test-file structure for oversized test suites
</commit_message>
<xml_diff>
--- a/backlog/backlog.xlsx
+++ b/backlog/backlog.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="13548" windowHeight="4716"/>
+    <workbookView windowWidth="22188" windowHeight="9384"/>
   </bookViews>
   <sheets>
     <sheet name="backlog" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1527" uniqueCount="814">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1527" uniqueCount="813">
   <si>
     <t>PBI-###</t>
   </si>
@@ -2463,9 +2463,6 @@
   </si>
   <si>
     <t>Maintainability;Testability;Reliability</t>
-  </si>
-  <si>
-    <t>Draft</t>
   </si>
   <si>
     <t>Important: target split should follow behavior-oriented boundaries, for example create-path, validation, duplicate/conflict, authorization, and state-transition coverage. Evidence: before/after file structure, passing full test suite, and note of any extracted shared test helpers. If refactoring spans many modules or exceeds 5 points, split by module or domain area rather than one backlog item.</t>
@@ -5791,7 +5788,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="51" hidden="1" spans="1:14">
+    <row r="51" spans="1:14">
       <c r="A51" t="s">
         <v>359</v>
       </c>
@@ -5879,7 +5876,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="53" hidden="1" spans="1:14">
+    <row r="53" spans="1:14">
       <c r="A53" t="s">
         <v>372</v>
       </c>
@@ -5923,7 +5920,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="54" hidden="1" spans="1:14">
+    <row r="54" spans="1:14">
       <c r="A54" t="s">
         <v>378</v>
       </c>
@@ -5967,7 +5964,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="55" hidden="1" spans="1:14">
+    <row r="55" spans="1:14">
       <c r="A55" t="s">
         <v>384</v>
       </c>
@@ -6436,7 +6433,7 @@
         <v>363</v>
       </c>
       <c r="L65" t="s">
-        <v>45</v>
+        <v>292</v>
       </c>
       <c r="M65" t="s">
         <v>451</v>
@@ -6480,7 +6477,7 @@
         <v>363</v>
       </c>
       <c r="L66" t="s">
-        <v>45</v>
+        <v>292</v>
       </c>
       <c r="M66" t="s">
         <v>457</v>
@@ -6568,7 +6565,7 @@
         <v>363</v>
       </c>
       <c r="L68" t="s">
-        <v>45</v>
+        <v>292</v>
       </c>
       <c r="M68" t="s">
         <v>469</v>
@@ -6653,7 +6650,7 @@
         <v>363</v>
       </c>
       <c r="L70" t="s">
-        <v>45</v>
+        <v>292</v>
       </c>
       <c r="M70" t="s">
         <v>481</v>
@@ -6697,7 +6694,7 @@
         <v>363</v>
       </c>
       <c r="L71" t="s">
-        <v>45</v>
+        <v>292</v>
       </c>
       <c r="M71" t="s">
         <v>488</v>
@@ -6785,7 +6782,7 @@
         <v>363</v>
       </c>
       <c r="L73" t="s">
-        <v>45</v>
+        <v>292</v>
       </c>
       <c r="M73" t="s">
         <v>500</v>
@@ -6870,7 +6867,7 @@
         <v>363</v>
       </c>
       <c r="L75" t="s">
-        <v>45</v>
+        <v>292</v>
       </c>
       <c r="M75" t="s">
         <v>513</v>
@@ -6914,7 +6911,7 @@
         <v>363</v>
       </c>
       <c r="L76" t="s">
-        <v>45</v>
+        <v>292</v>
       </c>
       <c r="M76" t="s">
         <v>520</v>
@@ -7225,7 +7222,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="84" hidden="1" spans="1:14">
+    <row r="84" spans="1:14">
       <c r="A84" t="s">
         <v>566</v>
       </c>
@@ -7269,7 +7266,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="85" hidden="1" spans="1:14">
+    <row r="85" spans="1:14">
       <c r="A85" t="s">
         <v>574</v>
       </c>
@@ -7313,7 +7310,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="86" hidden="1" spans="1:14">
+    <row r="86" spans="1:14">
       <c r="A86" t="s">
         <v>580</v>
       </c>
@@ -7357,7 +7354,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="87" hidden="1" spans="1:14">
+    <row r="87" spans="1:14">
       <c r="A87" t="s">
         <v>586</v>
       </c>
@@ -7401,7 +7398,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="88" hidden="1" spans="1:14">
+    <row r="88" spans="1:14">
       <c r="A88" t="s">
         <v>593</v>
       </c>
@@ -7445,7 +7442,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="89" hidden="1" spans="1:14">
+    <row r="89" spans="1:14">
       <c r="A89" t="s">
         <v>599</v>
       </c>
@@ -7489,7 +7486,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="90" spans="1:14">
+    <row r="90" hidden="1" spans="1:14">
       <c r="A90" t="s">
         <v>605</v>
       </c>
@@ -7533,7 +7530,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="91" hidden="1" spans="1:14">
+    <row r="91" spans="1:14">
       <c r="A91" t="s">
         <v>612</v>
       </c>
@@ -7577,7 +7574,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="92" hidden="1" spans="1:14">
+    <row r="92" spans="1:14">
       <c r="A92" t="s">
         <v>619</v>
       </c>
@@ -7621,7 +7618,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="93" hidden="1" spans="1:14">
+    <row r="93" spans="1:14">
       <c r="A93" t="s">
         <v>626</v>
       </c>
@@ -7665,7 +7662,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="94" hidden="1" spans="1:14">
+    <row r="94" spans="1:14">
       <c r="A94" t="s">
         <v>633</v>
       </c>
@@ -7709,7 +7706,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="95" hidden="1" spans="1:14">
+    <row r="95" spans="1:14">
       <c r="A95" t="s">
         <v>639</v>
       </c>
@@ -7753,7 +7750,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="96" hidden="1" spans="1:14">
+    <row r="96" spans="1:14">
       <c r="A96" t="s">
         <v>646</v>
       </c>
@@ -7797,7 +7794,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="97" hidden="1" spans="1:14">
+    <row r="97" spans="1:14">
       <c r="A97" t="s">
         <v>652</v>
       </c>
@@ -7841,7 +7838,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="98" hidden="1" spans="1:14">
+    <row r="98" spans="1:14">
       <c r="A98" t="s">
         <v>658</v>
       </c>
@@ -7885,7 +7882,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="99" hidden="1" spans="1:14">
+    <row r="99" spans="1:14">
       <c r="A99" t="s">
         <v>665</v>
       </c>
@@ -7929,7 +7926,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="100" hidden="1" spans="1:14">
+    <row r="100" spans="1:14">
       <c r="A100" t="s">
         <v>672</v>
       </c>
@@ -7973,7 +7970,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="101" hidden="1" spans="1:14">
+    <row r="101" spans="1:14">
       <c r="A101" t="s">
         <v>679</v>
       </c>
@@ -8017,7 +8014,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="102" hidden="1" spans="1:14">
+    <row r="102" spans="1:14">
       <c r="A102" t="s">
         <v>686</v>
       </c>
@@ -8061,7 +8058,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="103" hidden="1" spans="1:14">
+    <row r="103" spans="1:14">
       <c r="A103" t="s">
         <v>693</v>
       </c>
@@ -8105,7 +8102,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="104" hidden="1" spans="1:14">
+    <row r="104" spans="1:14">
       <c r="A104" t="s">
         <v>700</v>
       </c>
@@ -8149,7 +8146,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="105" hidden="1" spans="1:14">
+    <row r="105" spans="1:14">
       <c r="A105" t="s">
         <v>707</v>
       </c>
@@ -8193,7 +8190,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="106" hidden="1" spans="1:14">
+    <row r="106" spans="1:14">
       <c r="A106" t="s">
         <v>713</v>
       </c>
@@ -8237,7 +8234,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="107" hidden="1" spans="1:14">
+    <row r="107" spans="1:14">
       <c r="A107" t="s">
         <v>719</v>
       </c>
@@ -8281,7 +8278,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="108" hidden="1" spans="1:14">
+    <row r="108" spans="1:14">
       <c r="A108" t="s">
         <v>726</v>
       </c>
@@ -8325,7 +8322,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="109" hidden="1" spans="1:14">
+    <row r="109" spans="1:14">
       <c r="A109" t="s">
         <v>733</v>
       </c>
@@ -8369,7 +8366,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="110" hidden="1" spans="1:14">
+    <row r="110" spans="1:14">
       <c r="A110" t="s">
         <v>740</v>
       </c>
@@ -8413,7 +8410,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="111" hidden="1" spans="1:14">
+    <row r="111" spans="1:14">
       <c r="A111" t="s">
         <v>747</v>
       </c>
@@ -8457,7 +8454,7 @@
         <v>752</v>
       </c>
     </row>
-    <row r="112" hidden="1" spans="1:14">
+    <row r="112" spans="1:14">
       <c r="A112" t="s">
         <v>753</v>
       </c>
@@ -8633,7 +8630,7 @@
         <v>779</v>
       </c>
     </row>
-    <row r="116" hidden="1" spans="1:14">
+    <row r="116" spans="1:14">
       <c r="A116" t="s">
         <v>780</v>
       </c>
@@ -8677,7 +8674,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="117" hidden="1" spans="1:14">
+    <row r="117" spans="1:14">
       <c r="A117" t="s">
         <v>786</v>
       </c>
@@ -8721,7 +8718,7 @@
         <v>792</v>
       </c>
     </row>
-    <row r="118" hidden="1" spans="1:14">
+    <row r="118" spans="1:14">
       <c r="A118" t="s">
         <v>793</v>
       </c>
@@ -8765,7 +8762,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="119" hidden="1" spans="1:14">
+    <row r="119" spans="1:14">
       <c r="A119" t="s">
         <v>799</v>
       </c>
@@ -8809,7 +8806,7 @@
         <v>805</v>
       </c>
     </row>
-    <row r="120" hidden="1" spans="1:14">
+    <row r="120" spans="1:14">
       <c r="A120" t="s">
         <v>806</v>
       </c>
@@ -8844,33 +8841,25 @@
         <v>363</v>
       </c>
       <c r="L120" t="s">
-        <v>811</v>
+        <v>292</v>
       </c>
       <c r="M120" t="s">
         <v>24</v>
       </c>
       <c r="N120" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
     </row>
     <row r="121" hidden="1" spans="1:14">
       <c r="D121" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:N121" etc:filterBottomFollowUsedRange="0">
-    <filterColumn colId="0">
+    <filterColumn colId="10">
       <filters>
-        <filter val="PBI-070"/>
-        <filter val="PBI-072"/>
-        <filter val="PBI-064"/>
-        <filter val="PBI-074"/>
-        <filter val="PBI-065"/>
-        <filter val="PBI-075"/>
-        <filter val="PBI-067"/>
-        <filter val="PBI-069"/>
-        <filter val="PBI-089"/>
+        <filter val="Sprint 2"/>
       </filters>
     </filterColumn>
     <extLst/>
@@ -8899,7 +8888,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L67 L68 L69 L72 L73 L74 L90 L1:L64 L65:L66 L70:L71 L75:L76 L77:L89 L91:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L$1:L$1048576">
       <formula1>"Planned,Deferred,In-Progress,Completed,Draft,Blocked"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
[PBI-079, PBI-082, PBI-080, PBI-081]
</commit_message>
<xml_diff>
--- a/backlog/backlog.xlsx
+++ b/backlog/backlog.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1527" uniqueCount="814">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1527" uniqueCount="813">
   <si>
     <t>PBI-###</t>
   </si>
@@ -948,9 +948,6 @@
   </si>
   <si>
     <t>Sprint 3</t>
-  </si>
-  <si>
-    <t>Blocked</t>
   </si>
   <si>
     <t>PBI-031;PBI-039;PBI-040;PBI-079;PBI-080;PBI-081;PBI-082;PBI-083</t>
@@ -3674,7 +3671,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:N121"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
@@ -3722,7 +3719,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" hidden="1" spans="1:14">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -3763,7 +3760,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" hidden="1" spans="1:14">
       <c r="A3" t="s">
         <v>26</v>
       </c>
@@ -3807,7 +3804,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" hidden="1" spans="1:14">
       <c r="A4" t="s">
         <v>38</v>
       </c>
@@ -3851,7 +3848,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" hidden="1" spans="1:14">
       <c r="A5" t="s">
         <v>47</v>
       </c>
@@ -3892,7 +3889,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" hidden="1" spans="1:14">
       <c r="A6" t="s">
         <v>55</v>
       </c>
@@ -3936,7 +3933,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7" hidden="1" spans="1:14">
       <c r="A7" t="s">
         <v>63</v>
       </c>
@@ -3980,7 +3977,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" hidden="1" spans="1:14">
       <c r="A8" t="s">
         <v>72</v>
       </c>
@@ -4024,7 +4021,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9" hidden="1" spans="1:14">
       <c r="A9" t="s">
         <v>81</v>
       </c>
@@ -4068,7 +4065,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10" hidden="1" spans="1:14">
       <c r="A10" t="s">
         <v>89</v>
       </c>
@@ -4109,7 +4106,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" hidden="1" spans="1:14">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -4150,7 +4147,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:14">
+    <row r="12" hidden="1" spans="1:14">
       <c r="A12" t="s">
         <v>102</v>
       </c>
@@ -4191,7 +4188,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="13" spans="1:14">
+    <row r="13" hidden="1" spans="1:14">
       <c r="A13" t="s">
         <v>109</v>
       </c>
@@ -4232,7 +4229,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" hidden="1" spans="1:14">
       <c r="A14" t="s">
         <v>115</v>
       </c>
@@ -4273,7 +4270,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:14">
+    <row r="15" hidden="1" spans="1:14">
       <c r="A15" t="s">
         <v>123</v>
       </c>
@@ -4314,7 +4311,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:14">
+    <row r="16" hidden="1" spans="1:14">
       <c r="A16" t="s">
         <v>130</v>
       </c>
@@ -4358,7 +4355,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="17" spans="1:14">
+    <row r="17" hidden="1" spans="1:14">
       <c r="A17" t="s">
         <v>138</v>
       </c>
@@ -4399,7 +4396,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:14">
+    <row r="18" hidden="1" spans="1:14">
       <c r="A18" t="s">
         <v>144</v>
       </c>
@@ -4443,7 +4440,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="19" spans="1:14">
+    <row r="19" hidden="1" spans="1:14">
       <c r="A19" t="s">
         <v>152</v>
       </c>
@@ -4484,7 +4481,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:14">
+    <row r="20" hidden="1" spans="1:14">
       <c r="A20" t="s">
         <v>159</v>
       </c>
@@ -4525,7 +4522,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:14">
+    <row r="21" hidden="1" spans="1:14">
       <c r="A21" t="s">
         <v>166</v>
       </c>
@@ -4569,7 +4566,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="22" spans="1:14">
+    <row r="22" hidden="1" spans="1:14">
       <c r="A22" t="s">
         <v>174</v>
       </c>
@@ -4610,7 +4607,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:14">
+    <row r="23" hidden="1" spans="1:14">
       <c r="A23" t="s">
         <v>165</v>
       </c>
@@ -4654,7 +4651,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="24" spans="1:14">
+    <row r="24" hidden="1" spans="1:14">
       <c r="A24" t="s">
         <v>187</v>
       </c>
@@ -4695,7 +4692,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="25" spans="1:14">
+    <row r="25" hidden="1" spans="1:14">
       <c r="A25" t="s">
         <v>194</v>
       </c>
@@ -4736,7 +4733,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:14">
+    <row r="26" hidden="1" spans="1:14">
       <c r="A26" t="s">
         <v>122</v>
       </c>
@@ -4777,7 +4774,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:14">
+    <row r="27" hidden="1" spans="1:14">
       <c r="A27" t="s">
         <v>207</v>
       </c>
@@ -4818,7 +4815,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:14">
+    <row r="28" hidden="1" spans="1:14">
       <c r="A28" t="s">
         <v>213</v>
       </c>
@@ -4859,7 +4856,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:14">
+    <row r="29" hidden="1" spans="1:14">
       <c r="A29" t="s">
         <v>220</v>
       </c>
@@ -4900,7 +4897,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:14">
+    <row r="30" hidden="1" spans="1:14">
       <c r="A30" t="s">
         <v>227</v>
       </c>
@@ -4941,7 +4938,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="31" spans="1:14">
+    <row r="31" hidden="1" spans="1:14">
       <c r="A31" t="s">
         <v>234</v>
       </c>
@@ -4982,7 +4979,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:14">
+    <row r="32" hidden="1" spans="1:14">
       <c r="A32" t="s">
         <v>241</v>
       </c>
@@ -5023,7 +5020,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="33" spans="1:14">
+    <row r="33" hidden="1" spans="1:14">
       <c r="A33" t="s">
         <v>248</v>
       </c>
@@ -5064,7 +5061,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="34" spans="1:14">
+    <row r="34" hidden="1" spans="1:14">
       <c r="A34" t="s">
         <v>253</v>
       </c>
@@ -5105,7 +5102,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="35" spans="1:14">
+    <row r="35" hidden="1" spans="1:14">
       <c r="A35" t="s">
         <v>258</v>
       </c>
@@ -5146,7 +5143,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="36" spans="1:14">
+    <row r="36" hidden="1" spans="1:14">
       <c r="A36" t="s">
         <v>264</v>
       </c>
@@ -5187,7 +5184,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="37" spans="1:14">
+    <row r="37" hidden="1" spans="1:14">
       <c r="A37" t="s">
         <v>270</v>
       </c>
@@ -5228,7 +5225,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="38" spans="1:14">
+    <row r="38" hidden="1" spans="1:14">
       <c r="A38" t="s">
         <v>275</v>
       </c>
@@ -5269,7 +5266,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="39" spans="1:14">
+    <row r="39" hidden="1" spans="1:14">
       <c r="A39" t="s">
         <v>280</v>
       </c>
@@ -5310,7 +5307,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="40" spans="1:14">
+    <row r="40" hidden="1" spans="1:14">
       <c r="A40" t="s">
         <v>286</v>
       </c>
@@ -5354,7 +5351,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="41" spans="1:14">
+    <row r="41" hidden="1" spans="1:14">
       <c r="A41" t="s">
         <v>294</v>
       </c>
@@ -5433,36 +5430,36 @@
         <v>305</v>
       </c>
       <c r="L42" t="s">
+        <v>35</v>
+      </c>
+      <c r="M42" t="s">
         <v>306</v>
       </c>
-      <c r="M42" t="s">
+      <c r="N42" t="s">
         <v>307</v>
       </c>
-      <c r="N42" t="s">
+    </row>
+    <row r="43" hidden="1" spans="1:14">
+      <c r="A43" t="s">
         <v>308</v>
-      </c>
-    </row>
-    <row r="43" spans="1:14">
-      <c r="A43" t="s">
-        <v>309</v>
       </c>
       <c r="B43" t="s">
         <v>287</v>
       </c>
       <c r="C43" t="s">
+        <v>309</v>
+      </c>
+      <c r="D43" t="s">
         <v>310</v>
       </c>
-      <c r="D43" t="s">
+      <c r="E43" t="s">
         <v>311</v>
-      </c>
-      <c r="E43" t="s">
-        <v>312</v>
       </c>
       <c r="F43" t="s">
         <v>42</v>
       </c>
       <c r="G43" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H43">
         <v>2</v>
@@ -5480,33 +5477,33 @@
         <v>292</v>
       </c>
       <c r="M43" t="s">
+        <v>313</v>
+      </c>
+      <c r="N43" t="s">
         <v>314</v>
       </c>
-      <c r="N43" t="s">
+    </row>
+    <row r="44" hidden="1" spans="1:14">
+      <c r="A44" t="s">
         <v>315</v>
-      </c>
-    </row>
-    <row r="44" spans="1:14">
-      <c r="A44" t="s">
-        <v>316</v>
       </c>
       <c r="B44" t="s">
         <v>287</v>
       </c>
       <c r="C44" t="s">
+        <v>316</v>
+      </c>
+      <c r="D44" t="s">
         <v>317</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>318</v>
-      </c>
-      <c r="E44" t="s">
-        <v>319</v>
       </c>
       <c r="F44" t="s">
         <v>42</v>
       </c>
       <c r="G44" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H44">
         <v>2</v>
@@ -5521,30 +5518,30 @@
         <v>291</v>
       </c>
       <c r="L44" t="s">
-        <v>292</v>
+        <v>45</v>
       </c>
       <c r="M44" t="s">
+        <v>320</v>
+      </c>
+      <c r="N44" t="s">
         <v>321</v>
       </c>
-      <c r="N44" t="s">
+    </row>
+    <row r="45" hidden="1" spans="1:14">
+      <c r="A45" t="s">
         <v>322</v>
-      </c>
-    </row>
-    <row r="45" spans="1:14">
-      <c r="A45" t="s">
-        <v>323</v>
       </c>
       <c r="B45" t="s">
         <v>287</v>
       </c>
       <c r="C45" t="s">
+        <v>323</v>
+      </c>
+      <c r="D45" t="s">
         <v>324</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>325</v>
-      </c>
-      <c r="E45" t="s">
-        <v>326</v>
       </c>
       <c r="F45" t="s">
         <v>42</v>
@@ -5571,24 +5568,24 @@
         <v>248</v>
       </c>
       <c r="N45" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="46" hidden="1" spans="1:14">
+      <c r="A46" t="s">
         <v>327</v>
-      </c>
-    </row>
-    <row r="46" spans="1:14">
-      <c r="A46" t="s">
-        <v>328</v>
       </c>
       <c r="B46" t="s">
         <v>287</v>
       </c>
       <c r="C46" t="s">
+        <v>328</v>
+      </c>
+      <c r="D46" t="s">
         <v>329</v>
       </c>
-      <c r="D46" t="s">
+      <c r="E46" t="s">
         <v>330</v>
-      </c>
-      <c r="E46" t="s">
-        <v>331</v>
       </c>
       <c r="F46" t="s">
         <v>42</v>
@@ -5612,33 +5609,33 @@
         <v>292</v>
       </c>
       <c r="M46" t="s">
+        <v>331</v>
+      </c>
+      <c r="N46" t="s">
         <v>332</v>
-      </c>
-      <c r="N46" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="47" spans="1:14">
       <c r="A47" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B47" t="s">
         <v>287</v>
       </c>
       <c r="C47" t="s">
+        <v>334</v>
+      </c>
+      <c r="D47" t="s">
         <v>335</v>
       </c>
-      <c r="D47" t="s">
+      <c r="E47" t="s">
         <v>336</v>
-      </c>
-      <c r="E47" t="s">
-        <v>337</v>
       </c>
       <c r="F47" t="s">
         <v>42</v>
       </c>
       <c r="G47" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="H47">
         <v>2</v>
@@ -5653,36 +5650,36 @@
         <v>305</v>
       </c>
       <c r="L47" t="s">
-        <v>306</v>
+        <v>35</v>
       </c>
       <c r="M47" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="N47" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="48" hidden="1" spans="1:14">
+      <c r="A48" t="s">
         <v>339</v>
-      </c>
-    </row>
-    <row r="48" spans="1:14">
-      <c r="A48" t="s">
-        <v>340</v>
       </c>
       <c r="B48" t="s">
         <v>287</v>
       </c>
       <c r="C48" t="s">
+        <v>340</v>
+      </c>
+      <c r="D48" t="s">
         <v>341</v>
       </c>
-      <c r="D48" t="s">
+      <c r="E48" t="s">
         <v>342</v>
-      </c>
-      <c r="E48" t="s">
-        <v>343</v>
       </c>
       <c r="F48" t="s">
         <v>42</v>
       </c>
       <c r="G48" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H48">
         <v>2</v>
@@ -5700,33 +5697,33 @@
         <v>292</v>
       </c>
       <c r="M48" t="s">
+        <v>343</v>
+      </c>
+      <c r="N48" t="s">
         <v>344</v>
       </c>
-      <c r="N48" t="s">
+    </row>
+    <row r="49" hidden="1" spans="1:14">
+      <c r="A49" t="s">
         <v>345</v>
-      </c>
-    </row>
-    <row r="49" spans="1:14">
-      <c r="A49" t="s">
-        <v>346</v>
       </c>
       <c r="B49" t="s">
         <v>287</v>
       </c>
       <c r="C49" t="s">
+        <v>346</v>
+      </c>
+      <c r="D49" t="s">
         <v>347</v>
       </c>
-      <c r="D49" t="s">
+      <c r="E49" t="s">
         <v>348</v>
-      </c>
-      <c r="E49" t="s">
-        <v>349</v>
       </c>
       <c r="F49" t="s">
         <v>42</v>
       </c>
       <c r="G49" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H49">
         <v>2</v>
@@ -5741,27 +5738,27 @@
         <v>45</v>
       </c>
       <c r="M49" t="s">
+        <v>349</v>
+      </c>
+      <c r="N49" t="s">
         <v>350</v>
       </c>
-      <c r="N49" t="s">
+    </row>
+    <row r="50" hidden="1" spans="1:14">
+      <c r="A50" t="s">
         <v>351</v>
-      </c>
-    </row>
-    <row r="50" spans="1:14">
-      <c r="A50" t="s">
-        <v>352</v>
       </c>
       <c r="B50" t="s">
         <v>287</v>
       </c>
       <c r="C50" t="s">
+        <v>352</v>
+      </c>
+      <c r="D50" t="s">
         <v>353</v>
       </c>
-      <c r="D50" t="s">
+      <c r="E50" t="s">
         <v>354</v>
-      </c>
-      <c r="E50" t="s">
-        <v>355</v>
       </c>
       <c r="F50" t="s">
         <v>42</v>
@@ -5776,7 +5773,7 @@
         <v>32</v>
       </c>
       <c r="J50" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="K50" t="s">
         <v>291</v>
@@ -5785,27 +5782,27 @@
         <v>292</v>
       </c>
       <c r="M50" t="s">
+        <v>356</v>
+      </c>
+      <c r="N50" t="s">
         <v>357</v>
       </c>
-      <c r="N50" t="s">
+    </row>
+    <row r="51" hidden="1" spans="1:14">
+      <c r="A51" t="s">
         <v>358</v>
-      </c>
-    </row>
-    <row r="51" spans="1:14">
-      <c r="A51" t="s">
-        <v>359</v>
       </c>
       <c r="B51" t="s">
         <v>287</v>
       </c>
       <c r="C51" t="s">
+        <v>359</v>
+      </c>
+      <c r="D51" t="s">
         <v>360</v>
       </c>
-      <c r="D51" t="s">
+      <c r="E51" t="s">
         <v>361</v>
-      </c>
-      <c r="E51" t="s">
-        <v>362</v>
       </c>
       <c r="F51" t="s">
         <v>42</v>
@@ -5823,39 +5820,39 @@
         <v>61</v>
       </c>
       <c r="K51" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L51" t="s">
         <v>292</v>
       </c>
       <c r="M51" t="s">
+        <v>363</v>
+      </c>
+      <c r="N51" t="s">
         <v>364</v>
-      </c>
-      <c r="N51" t="s">
-        <v>365</v>
       </c>
     </row>
     <row r="52" spans="1:14">
       <c r="A52" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B52" t="s">
         <v>287</v>
       </c>
       <c r="C52" t="s">
+        <v>366</v>
+      </c>
+      <c r="D52" t="s">
         <v>367</v>
       </c>
-      <c r="D52" t="s">
+      <c r="E52" t="s">
         <v>368</v>
-      </c>
-      <c r="E52" t="s">
-        <v>369</v>
       </c>
       <c r="F52" t="s">
         <v>42</v>
       </c>
       <c r="G52" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="H52">
         <v>2</v>
@@ -5870,36 +5867,36 @@
         <v>305</v>
       </c>
       <c r="L52" t="s">
-        <v>306</v>
+        <v>35</v>
       </c>
       <c r="M52" t="s">
+        <v>369</v>
+      </c>
+      <c r="N52" t="s">
         <v>370</v>
       </c>
-      <c r="N52" t="s">
+    </row>
+    <row r="53" hidden="1" spans="1:14">
+      <c r="A53" t="s">
         <v>371</v>
-      </c>
-    </row>
-    <row r="53" spans="1:14">
-      <c r="A53" t="s">
-        <v>372</v>
       </c>
       <c r="B53" t="s">
         <v>287</v>
       </c>
       <c r="C53" t="s">
+        <v>372</v>
+      </c>
+      <c r="D53" t="s">
         <v>373</v>
       </c>
-      <c r="D53" t="s">
+      <c r="E53" t="s">
         <v>374</v>
-      </c>
-      <c r="E53" t="s">
-        <v>375</v>
       </c>
       <c r="F53" t="s">
         <v>42</v>
       </c>
       <c r="G53" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H53">
         <v>2</v>
@@ -5911,39 +5908,39 @@
         <v>95</v>
       </c>
       <c r="K53" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L53" t="s">
         <v>292</v>
       </c>
       <c r="M53" t="s">
+        <v>375</v>
+      </c>
+      <c r="N53" t="s">
         <v>376</v>
       </c>
-      <c r="N53" t="s">
+    </row>
+    <row r="54" hidden="1" spans="1:14">
+      <c r="A54" t="s">
         <v>377</v>
-      </c>
-    </row>
-    <row r="54" spans="1:14">
-      <c r="A54" t="s">
-        <v>378</v>
       </c>
       <c r="B54" t="s">
         <v>287</v>
       </c>
       <c r="C54" t="s">
+        <v>378</v>
+      </c>
+      <c r="D54" t="s">
         <v>379</v>
       </c>
-      <c r="D54" t="s">
+      <c r="E54" t="s">
         <v>380</v>
-      </c>
-      <c r="E54" t="s">
-        <v>381</v>
       </c>
       <c r="F54" t="s">
         <v>42</v>
       </c>
       <c r="G54" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H54">
         <v>2</v>
@@ -5955,33 +5952,33 @@
         <v>121</v>
       </c>
       <c r="K54" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L54" t="s">
         <v>292</v>
       </c>
       <c r="M54" t="s">
+        <v>381</v>
+      </c>
+      <c r="N54" t="s">
         <v>382</v>
       </c>
-      <c r="N54" t="s">
+    </row>
+    <row r="55" hidden="1" spans="1:14">
+      <c r="A55" t="s">
         <v>383</v>
-      </c>
-    </row>
-    <row r="55" spans="1:14">
-      <c r="A55" t="s">
-        <v>384</v>
       </c>
       <c r="B55" t="s">
         <v>287</v>
       </c>
       <c r="C55" t="s">
+        <v>384</v>
+      </c>
+      <c r="D55" t="s">
         <v>385</v>
       </c>
-      <c r="D55" t="s">
+      <c r="E55" t="s">
         <v>386</v>
-      </c>
-      <c r="E55" t="s">
-        <v>387</v>
       </c>
       <c r="F55" t="s">
         <v>42</v>
@@ -5996,36 +5993,36 @@
         <v>32</v>
       </c>
       <c r="J55" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="K55" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L55" t="s">
         <v>292</v>
       </c>
       <c r="M55" t="s">
+        <v>387</v>
+      </c>
+      <c r="N55" t="s">
         <v>388</v>
       </c>
-      <c r="N55" t="s">
+    </row>
+    <row r="56" hidden="1" spans="1:14">
+      <c r="A56" t="s">
         <v>389</v>
-      </c>
-    </row>
-    <row r="56" spans="1:14">
-      <c r="A56" t="s">
-        <v>390</v>
       </c>
       <c r="B56" t="s">
         <v>287</v>
       </c>
       <c r="C56" t="s">
+        <v>390</v>
+      </c>
+      <c r="D56" t="s">
         <v>391</v>
       </c>
-      <c r="D56" t="s">
+      <c r="E56" t="s">
         <v>392</v>
-      </c>
-      <c r="E56" t="s">
-        <v>393</v>
       </c>
       <c r="F56" t="s">
         <v>42</v>
@@ -6043,39 +6040,39 @@
         <v>61</v>
       </c>
       <c r="K56" t="s">
+        <v>393</v>
+      </c>
+      <c r="L56" t="s">
+        <v>292</v>
+      </c>
+      <c r="M56" t="s">
         <v>394</v>
       </c>
-      <c r="L56" t="s">
-        <v>35</v>
-      </c>
-      <c r="M56" t="s">
+      <c r="N56" t="s">
         <v>395</v>
-      </c>
-      <c r="N56" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="57" spans="1:14">
       <c r="A57" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B57" t="s">
         <v>287</v>
       </c>
       <c r="C57" t="s">
+        <v>397</v>
+      </c>
+      <c r="D57" t="s">
         <v>398</v>
       </c>
-      <c r="D57" t="s">
+      <c r="E57" t="s">
         <v>399</v>
-      </c>
-      <c r="E57" t="s">
-        <v>400</v>
       </c>
       <c r="F57" t="s">
         <v>42</v>
       </c>
       <c r="G57" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H57">
         <v>2</v>
@@ -6090,36 +6087,36 @@
         <v>305</v>
       </c>
       <c r="L57" t="s">
-        <v>306</v>
+        <v>35</v>
       </c>
       <c r="M57" t="s">
+        <v>401</v>
+      </c>
+      <c r="N57" t="s">
         <v>402</v>
       </c>
-      <c r="N57" t="s">
+    </row>
+    <row r="58" hidden="1" spans="1:14">
+      <c r="A58" t="s">
         <v>403</v>
-      </c>
-    </row>
-    <row r="58" spans="1:14">
-      <c r="A58" t="s">
-        <v>404</v>
       </c>
       <c r="B58" t="s">
         <v>287</v>
       </c>
       <c r="C58" t="s">
+        <v>404</v>
+      </c>
+      <c r="D58" t="s">
         <v>405</v>
       </c>
-      <c r="D58" t="s">
+      <c r="E58" t="s">
         <v>406</v>
-      </c>
-      <c r="E58" t="s">
-        <v>407</v>
       </c>
       <c r="F58" t="s">
         <v>42</v>
       </c>
       <c r="G58" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="H58">
         <v>2</v>
@@ -6131,39 +6128,39 @@
         <v>95</v>
       </c>
       <c r="K58" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="L58" t="s">
-        <v>35</v>
+        <v>292</v>
       </c>
       <c r="M58" t="s">
+        <v>408</v>
+      </c>
+      <c r="N58" t="s">
         <v>409</v>
       </c>
-      <c r="N58" t="s">
+    </row>
+    <row r="59" hidden="1" spans="1:14">
+      <c r="A59" t="s">
         <v>410</v>
-      </c>
-    </row>
-    <row r="59" spans="1:14">
-      <c r="A59" t="s">
-        <v>411</v>
       </c>
       <c r="B59" t="s">
         <v>287</v>
       </c>
       <c r="C59" t="s">
+        <v>411</v>
+      </c>
+      <c r="D59" t="s">
         <v>412</v>
       </c>
-      <c r="D59" t="s">
+      <c r="E59" t="s">
         <v>413</v>
-      </c>
-      <c r="E59" t="s">
-        <v>414</v>
       </c>
       <c r="F59" t="s">
         <v>42</v>
       </c>
       <c r="G59" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H59">
         <v>2</v>
@@ -6175,36 +6172,36 @@
         <v>121</v>
       </c>
       <c r="L59" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M59" t="s">
+        <v>414</v>
+      </c>
+      <c r="N59" t="s">
         <v>415</v>
       </c>
-      <c r="N59" t="s">
+    </row>
+    <row r="60" hidden="1" spans="1:14">
+      <c r="A60" t="s">
         <v>416</v>
-      </c>
-    </row>
-    <row r="60" spans="1:14">
-      <c r="A60" t="s">
-        <v>417</v>
       </c>
       <c r="B60" t="s">
         <v>287</v>
       </c>
       <c r="C60" t="s">
+        <v>417</v>
+      </c>
+      <c r="D60" t="s">
         <v>418</v>
       </c>
-      <c r="D60" t="s">
+      <c r="E60" t="s">
         <v>419</v>
-      </c>
-      <c r="E60" t="s">
-        <v>420</v>
       </c>
       <c r="F60" t="s">
         <v>170</v>
       </c>
       <c r="G60" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="H60">
         <v>2</v>
@@ -6225,30 +6222,30 @@
         <v>264</v>
       </c>
       <c r="N60" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="61" hidden="1" spans="1:14">
+      <c r="A61" t="s">
         <v>422</v>
-      </c>
-    </row>
-    <row r="61" spans="1:14">
-      <c r="A61" t="s">
-        <v>423</v>
       </c>
       <c r="B61" t="s">
         <v>287</v>
       </c>
       <c r="C61" t="s">
+        <v>423</v>
+      </c>
+      <c r="D61" t="s">
         <v>424</v>
       </c>
-      <c r="D61" t="s">
+      <c r="E61" t="s">
         <v>425</v>
-      </c>
-      <c r="E61" t="s">
-        <v>426</v>
       </c>
       <c r="F61" t="s">
         <v>170</v>
       </c>
       <c r="G61" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="H61">
         <v>3</v>
@@ -6266,33 +6263,33 @@
         <v>292</v>
       </c>
       <c r="M61" t="s">
+        <v>427</v>
+      </c>
+      <c r="N61" t="s">
         <v>428</v>
-      </c>
-      <c r="N61" t="s">
-        <v>429</v>
       </c>
     </row>
     <row r="62" spans="1:14">
       <c r="A62" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B62" t="s">
         <v>287</v>
       </c>
       <c r="C62" t="s">
+        <v>430</v>
+      </c>
+      <c r="D62" t="s">
         <v>431</v>
       </c>
-      <c r="D62" t="s">
+      <c r="E62" t="s">
         <v>432</v>
-      </c>
-      <c r="E62" t="s">
-        <v>433</v>
       </c>
       <c r="F62" t="s">
         <v>170</v>
       </c>
       <c r="G62" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="H62">
         <v>2</v>
@@ -6307,30 +6304,30 @@
         <v>305</v>
       </c>
       <c r="L62" t="s">
-        <v>306</v>
+        <v>35</v>
       </c>
       <c r="M62" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="N62" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="63" hidden="1" spans="1:14">
+      <c r="A63" t="s">
         <v>435</v>
-      </c>
-    </row>
-    <row r="63" spans="1:14">
-      <c r="A63" t="s">
-        <v>436</v>
       </c>
       <c r="B63" t="s">
         <v>287</v>
       </c>
       <c r="C63" t="s">
+        <v>436</v>
+      </c>
+      <c r="D63" t="s">
         <v>437</v>
       </c>
-      <c r="D63" t="s">
+      <c r="E63" t="s">
         <v>438</v>
-      </c>
-      <c r="E63" t="s">
-        <v>439</v>
       </c>
       <c r="F63" t="s">
         <v>170</v>
@@ -6351,36 +6348,36 @@
         <v>291</v>
       </c>
       <c r="L63" t="s">
-        <v>45</v>
+        <v>292</v>
       </c>
       <c r="M63" t="s">
+        <v>439</v>
+      </c>
+      <c r="N63" t="s">
         <v>440</v>
       </c>
-      <c r="N63" t="s">
+    </row>
+    <row r="64" hidden="1" spans="1:14">
+      <c r="A64" t="s">
         <v>441</v>
-      </c>
-    </row>
-    <row r="64" spans="1:14">
-      <c r="A64" t="s">
-        <v>442</v>
       </c>
       <c r="B64" t="s">
         <v>287</v>
       </c>
       <c r="C64" t="s">
+        <v>442</v>
+      </c>
+      <c r="D64" t="s">
         <v>443</v>
       </c>
-      <c r="D64" t="s">
+      <c r="E64" t="s">
         <v>444</v>
-      </c>
-      <c r="E64" t="s">
-        <v>445</v>
       </c>
       <c r="F64" t="s">
         <v>170</v>
       </c>
       <c r="G64" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H64">
         <v>2</v>
@@ -6395,33 +6392,33 @@
         <v>45</v>
       </c>
       <c r="M64" t="s">
+        <v>445</v>
+      </c>
+      <c r="N64" t="s">
         <v>446</v>
       </c>
-      <c r="N64" t="s">
+    </row>
+    <row r="65" hidden="1" spans="1:14">
+      <c r="A65" t="s">
         <v>447</v>
-      </c>
-    </row>
-    <row r="65" spans="1:14">
-      <c r="A65" t="s">
-        <v>448</v>
       </c>
       <c r="B65" t="s">
         <v>287</v>
       </c>
       <c r="C65" t="s">
+        <v>448</v>
+      </c>
+      <c r="D65" t="s">
         <v>449</v>
       </c>
-      <c r="D65" t="s">
+      <c r="E65" t="s">
         <v>450</v>
-      </c>
-      <c r="E65" t="s">
-        <v>451</v>
       </c>
       <c r="F65" t="s">
         <v>170</v>
       </c>
       <c r="G65" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="H65">
         <v>2</v>
@@ -6433,39 +6430,39 @@
         <v>172</v>
       </c>
       <c r="K65" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L65" t="s">
         <v>292</v>
       </c>
       <c r="M65" t="s">
+        <v>451</v>
+      </c>
+      <c r="N65" t="s">
         <v>452</v>
       </c>
-      <c r="N65" t="s">
+    </row>
+    <row r="66" hidden="1" spans="1:14">
+      <c r="A66" t="s">
         <v>453</v>
-      </c>
-    </row>
-    <row r="66" spans="1:14">
-      <c r="A66" t="s">
-        <v>454</v>
       </c>
       <c r="B66" t="s">
         <v>287</v>
       </c>
       <c r="C66" t="s">
+        <v>454</v>
+      </c>
+      <c r="D66" t="s">
         <v>455</v>
       </c>
-      <c r="D66" t="s">
+      <c r="E66" t="s">
         <v>456</v>
-      </c>
-      <c r="E66" t="s">
-        <v>457</v>
       </c>
       <c r="F66" t="s">
         <v>170</v>
       </c>
       <c r="G66" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="H66">
         <v>3</v>
@@ -6477,39 +6474,39 @@
         <v>61</v>
       </c>
       <c r="K66" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L66" t="s">
         <v>292</v>
       </c>
       <c r="M66" t="s">
+        <v>457</v>
+      </c>
+      <c r="N66" t="s">
         <v>458</v>
-      </c>
-      <c r="N66" t="s">
-        <v>459</v>
       </c>
     </row>
     <row r="67" spans="1:14">
       <c r="A67" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B67" t="s">
         <v>287</v>
       </c>
       <c r="C67" t="s">
+        <v>460</v>
+      </c>
+      <c r="D67" t="s">
         <v>461</v>
       </c>
-      <c r="D67" t="s">
+      <c r="E67" t="s">
         <v>462</v>
-      </c>
-      <c r="E67" t="s">
-        <v>463</v>
       </c>
       <c r="F67" t="s">
         <v>170</v>
       </c>
       <c r="G67" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="H67">
         <v>2</v>
@@ -6524,30 +6521,30 @@
         <v>305</v>
       </c>
       <c r="L67" t="s">
-        <v>306</v>
+        <v>35</v>
       </c>
       <c r="M67" t="s">
+        <v>463</v>
+      </c>
+      <c r="N67" t="s">
         <v>464</v>
       </c>
-      <c r="N67" t="s">
+    </row>
+    <row r="68" hidden="1" spans="1:14">
+      <c r="A68" t="s">
         <v>465</v>
-      </c>
-    </row>
-    <row r="68" spans="1:14">
-      <c r="A68" t="s">
-        <v>466</v>
       </c>
       <c r="B68" t="s">
         <v>287</v>
       </c>
       <c r="C68" t="s">
+        <v>466</v>
+      </c>
+      <c r="D68" t="s">
         <v>467</v>
       </c>
-      <c r="D68" t="s">
+      <c r="E68" t="s">
         <v>468</v>
-      </c>
-      <c r="E68" t="s">
-        <v>469</v>
       </c>
       <c r="F68" t="s">
         <v>170</v>
@@ -6565,39 +6562,39 @@
         <v>95</v>
       </c>
       <c r="K68" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L68" t="s">
         <v>292</v>
       </c>
       <c r="M68" t="s">
+        <v>469</v>
+      </c>
+      <c r="N68" t="s">
         <v>470</v>
       </c>
-      <c r="N68" t="s">
+    </row>
+    <row r="69" hidden="1" spans="1:14">
+      <c r="A69" t="s">
         <v>471</v>
-      </c>
-    </row>
-    <row r="69" spans="1:14">
-      <c r="A69" t="s">
-        <v>472</v>
       </c>
       <c r="B69" t="s">
         <v>287</v>
       </c>
       <c r="C69" t="s">
+        <v>472</v>
+      </c>
+      <c r="D69" t="s">
         <v>473</v>
       </c>
-      <c r="D69" t="s">
+      <c r="E69" t="s">
         <v>474</v>
-      </c>
-      <c r="E69" t="s">
-        <v>475</v>
       </c>
       <c r="F69" t="s">
         <v>170</v>
       </c>
       <c r="G69" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H69">
         <v>2</v>
@@ -6609,36 +6606,36 @@
         <v>121</v>
       </c>
       <c r="L69" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M69" t="s">
+        <v>475</v>
+      </c>
+      <c r="N69" t="s">
         <v>476</v>
       </c>
-      <c r="N69" t="s">
+    </row>
+    <row r="70" hidden="1" spans="1:14">
+      <c r="A70" t="s">
         <v>477</v>
-      </c>
-    </row>
-    <row r="70" spans="1:14">
-      <c r="A70" t="s">
-        <v>478</v>
       </c>
       <c r="B70" t="s">
         <v>287</v>
       </c>
       <c r="C70" t="s">
+        <v>478</v>
+      </c>
+      <c r="D70" t="s">
         <v>479</v>
       </c>
-      <c r="D70" t="s">
+      <c r="E70" t="s">
         <v>480</v>
-      </c>
-      <c r="E70" t="s">
-        <v>481</v>
       </c>
       <c r="F70" t="s">
         <v>170</v>
       </c>
       <c r="G70" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="H70">
         <v>2</v>
@@ -6650,39 +6647,39 @@
         <v>172</v>
       </c>
       <c r="K70" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L70" t="s">
         <v>292</v>
       </c>
       <c r="M70" t="s">
+        <v>481</v>
+      </c>
+      <c r="N70" t="s">
         <v>482</v>
       </c>
-      <c r="N70" t="s">
+    </row>
+    <row r="71" hidden="1" spans="1:14">
+      <c r="A71" t="s">
         <v>483</v>
-      </c>
-    </row>
-    <row r="71" spans="1:14">
-      <c r="A71" t="s">
-        <v>484</v>
       </c>
       <c r="B71" t="s">
         <v>287</v>
       </c>
       <c r="C71" t="s">
+        <v>484</v>
+      </c>
+      <c r="D71" t="s">
         <v>485</v>
       </c>
-      <c r="D71" t="s">
+      <c r="E71" t="s">
         <v>486</v>
-      </c>
-      <c r="E71" t="s">
-        <v>487</v>
       </c>
       <c r="F71" t="s">
         <v>170</v>
       </c>
       <c r="G71" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="H71">
         <v>3</v>
@@ -6694,39 +6691,39 @@
         <v>61</v>
       </c>
       <c r="K71" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L71" t="s">
         <v>292</v>
       </c>
       <c r="M71" t="s">
+        <v>488</v>
+      </c>
+      <c r="N71" t="s">
         <v>489</v>
-      </c>
-      <c r="N71" t="s">
-        <v>490</v>
       </c>
     </row>
     <row r="72" spans="1:14">
       <c r="A72" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="B72" t="s">
         <v>287</v>
       </c>
       <c r="C72" t="s">
+        <v>491</v>
+      </c>
+      <c r="D72" t="s">
         <v>492</v>
       </c>
-      <c r="D72" t="s">
+      <c r="E72" t="s">
         <v>493</v>
-      </c>
-      <c r="E72" t="s">
-        <v>494</v>
       </c>
       <c r="F72" t="s">
         <v>170</v>
       </c>
       <c r="G72" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="H72">
         <v>2</v>
@@ -6741,30 +6738,30 @@
         <v>305</v>
       </c>
       <c r="L72" t="s">
-        <v>306</v>
+        <v>35</v>
       </c>
       <c r="M72" t="s">
+        <v>494</v>
+      </c>
+      <c r="N72" t="s">
         <v>495</v>
       </c>
-      <c r="N72" t="s">
+    </row>
+    <row r="73" hidden="1" spans="1:14">
+      <c r="A73" t="s">
         <v>496</v>
-      </c>
-    </row>
-    <row r="73" spans="1:14">
-      <c r="A73" t="s">
-        <v>497</v>
       </c>
       <c r="B73" t="s">
         <v>287</v>
       </c>
       <c r="C73" t="s">
+        <v>497</v>
+      </c>
+      <c r="D73" t="s">
         <v>498</v>
       </c>
-      <c r="D73" t="s">
+      <c r="E73" t="s">
         <v>499</v>
-      </c>
-      <c r="E73" t="s">
-        <v>500</v>
       </c>
       <c r="F73" t="s">
         <v>170</v>
@@ -6782,39 +6779,39 @@
         <v>95</v>
       </c>
       <c r="K73" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L73" t="s">
         <v>292</v>
       </c>
       <c r="M73" t="s">
+        <v>500</v>
+      </c>
+      <c r="N73" t="s">
         <v>501</v>
       </c>
-      <c r="N73" t="s">
+    </row>
+    <row r="74" hidden="1" spans="1:14">
+      <c r="A74" t="s">
         <v>502</v>
-      </c>
-    </row>
-    <row r="74" spans="1:14">
-      <c r="A74" t="s">
-        <v>503</v>
       </c>
       <c r="B74" t="s">
         <v>287</v>
       </c>
       <c r="C74" t="s">
+        <v>503</v>
+      </c>
+      <c r="D74" t="s">
         <v>504</v>
       </c>
-      <c r="D74" t="s">
+      <c r="E74" t="s">
         <v>505</v>
-      </c>
-      <c r="E74" t="s">
-        <v>506</v>
       </c>
       <c r="F74" t="s">
         <v>170</v>
       </c>
       <c r="G74" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H74">
         <v>2</v>
@@ -6826,36 +6823,36 @@
         <v>121</v>
       </c>
       <c r="L74" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M74" t="s">
+        <v>506</v>
+      </c>
+      <c r="N74" t="s">
         <v>507</v>
       </c>
-      <c r="N74" t="s">
+    </row>
+    <row r="75" hidden="1" spans="1:14">
+      <c r="A75" t="s">
         <v>508</v>
-      </c>
-    </row>
-    <row r="75" spans="1:14">
-      <c r="A75" t="s">
-        <v>509</v>
       </c>
       <c r="B75" t="s">
         <v>287</v>
       </c>
       <c r="C75" t="s">
+        <v>509</v>
+      </c>
+      <c r="D75" t="s">
         <v>510</v>
       </c>
-      <c r="D75" t="s">
+      <c r="E75" t="s">
         <v>511</v>
-      </c>
-      <c r="E75" t="s">
-        <v>512</v>
       </c>
       <c r="F75" t="s">
         <v>170</v>
       </c>
       <c r="G75" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="H75">
         <v>2</v>
@@ -6864,42 +6861,42 @@
         <v>21</v>
       </c>
       <c r="J75" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="K75" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L75" t="s">
         <v>292</v>
       </c>
       <c r="M75" t="s">
+        <v>513</v>
+      </c>
+      <c r="N75" t="s">
         <v>514</v>
       </c>
-      <c r="N75" t="s">
+    </row>
+    <row r="76" hidden="1" spans="1:14">
+      <c r="A76" t="s">
         <v>515</v>
-      </c>
-    </row>
-    <row r="76" spans="1:14">
-      <c r="A76" t="s">
-        <v>516</v>
       </c>
       <c r="B76" t="s">
         <v>287</v>
       </c>
       <c r="C76" t="s">
+        <v>516</v>
+      </c>
+      <c r="D76" t="s">
         <v>517</v>
       </c>
-      <c r="D76" t="s">
+      <c r="E76" t="s">
         <v>518</v>
-      </c>
-      <c r="E76" t="s">
-        <v>519</v>
       </c>
       <c r="F76" t="s">
         <v>170</v>
       </c>
       <c r="G76" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="H76">
         <v>3</v>
@@ -6911,39 +6908,39 @@
         <v>61</v>
       </c>
       <c r="K76" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L76" t="s">
         <v>292</v>
       </c>
       <c r="M76" t="s">
+        <v>520</v>
+      </c>
+      <c r="N76" t="s">
         <v>521</v>
-      </c>
-      <c r="N76" t="s">
-        <v>522</v>
       </c>
     </row>
     <row r="77" spans="1:14">
       <c r="A77" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B77" t="s">
         <v>287</v>
       </c>
       <c r="C77" t="s">
+        <v>523</v>
+      </c>
+      <c r="D77" t="s">
         <v>524</v>
       </c>
-      <c r="D77" t="s">
+      <c r="E77" t="s">
         <v>525</v>
-      </c>
-      <c r="E77" t="s">
-        <v>526</v>
       </c>
       <c r="F77" t="s">
         <v>170</v>
       </c>
       <c r="G77" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="H77">
         <v>2</v>
@@ -6958,30 +6955,30 @@
         <v>305</v>
       </c>
       <c r="L77" t="s">
-        <v>306</v>
+        <v>35</v>
       </c>
       <c r="M77" t="s">
+        <v>526</v>
+      </c>
+      <c r="N77" t="s">
         <v>527</v>
       </c>
-      <c r="N77" t="s">
+    </row>
+    <row r="78" hidden="1" spans="1:14">
+      <c r="A78" t="s">
         <v>528</v>
-      </c>
-    </row>
-    <row r="78" spans="1:14">
-      <c r="A78" t="s">
-        <v>529</v>
       </c>
       <c r="B78" t="s">
         <v>287</v>
       </c>
       <c r="C78" t="s">
+        <v>529</v>
+      </c>
+      <c r="D78" t="s">
         <v>530</v>
       </c>
-      <c r="D78" t="s">
+      <c r="E78" t="s">
         <v>531</v>
-      </c>
-      <c r="E78" t="s">
-        <v>532</v>
       </c>
       <c r="F78" t="s">
         <v>170</v>
@@ -6999,36 +6996,36 @@
         <v>95</v>
       </c>
       <c r="L78" t="s">
-        <v>35</v>
+        <v>292</v>
       </c>
       <c r="M78" t="s">
+        <v>532</v>
+      </c>
+      <c r="N78" t="s">
         <v>533</v>
       </c>
-      <c r="N78" t="s">
+    </row>
+    <row r="79" hidden="1" spans="1:14">
+      <c r="A79" t="s">
         <v>534</v>
-      </c>
-    </row>
-    <row r="79" spans="1:14">
-      <c r="A79" t="s">
-        <v>535</v>
       </c>
       <c r="B79" t="s">
         <v>287</v>
       </c>
       <c r="C79" t="s">
+        <v>535</v>
+      </c>
+      <c r="D79" t="s">
         <v>536</v>
       </c>
-      <c r="D79" t="s">
+      <c r="E79" t="s">
         <v>537</v>
-      </c>
-      <c r="E79" t="s">
-        <v>538</v>
       </c>
       <c r="F79" t="s">
         <v>170</v>
       </c>
       <c r="G79" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H79">
         <v>2</v>
@@ -7043,33 +7040,33 @@
         <v>35</v>
       </c>
       <c r="M79" t="s">
+        <v>538</v>
+      </c>
+      <c r="N79" t="s">
         <v>539</v>
-      </c>
-      <c r="N79" t="s">
-        <v>540</v>
       </c>
     </row>
     <row r="80" spans="1:14">
       <c r="A80" t="s">
+        <v>540</v>
+      </c>
+      <c r="B80" t="s">
         <v>541</v>
       </c>
-      <c r="B80" t="s">
+      <c r="C80" t="s">
         <v>542</v>
       </c>
-      <c r="C80" t="s">
+      <c r="D80" t="s">
         <v>543</v>
       </c>
-      <c r="D80" t="s">
+      <c r="E80" t="s">
         <v>544</v>
-      </c>
-      <c r="E80" t="s">
-        <v>545</v>
       </c>
       <c r="F80" t="s">
         <v>42</v>
       </c>
       <c r="G80" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="H80">
         <v>3</v>
@@ -7084,36 +7081,36 @@
         <v>305</v>
       </c>
       <c r="L80" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M80" t="s">
         <v>300</v>
       </c>
       <c r="N80" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
     </row>
     <row r="81" spans="1:14">
       <c r="A81" t="s">
+        <v>547</v>
+      </c>
+      <c r="B81" t="s">
         <v>548</v>
       </c>
-      <c r="B81" t="s">
+      <c r="C81" t="s">
         <v>549</v>
       </c>
-      <c r="C81" t="s">
+      <c r="D81" t="s">
         <v>550</v>
       </c>
-      <c r="D81" t="s">
+      <c r="E81" t="s">
         <v>551</v>
-      </c>
-      <c r="E81" t="s">
-        <v>552</v>
       </c>
       <c r="F81" t="s">
         <v>42</v>
       </c>
       <c r="G81" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="H81">
         <v>3</v>
@@ -7128,36 +7125,36 @@
         <v>305</v>
       </c>
       <c r="L81" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="M81" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="N81" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
     </row>
     <row r="82" spans="1:14">
       <c r="A82" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="B82" t="s">
         <v>287</v>
       </c>
       <c r="C82" t="s">
+        <v>554</v>
+      </c>
+      <c r="D82" t="s">
         <v>555</v>
       </c>
-      <c r="D82" t="s">
+      <c r="E82" t="s">
         <v>556</v>
-      </c>
-      <c r="E82" t="s">
-        <v>557</v>
       </c>
       <c r="F82" t="s">
         <v>42</v>
       </c>
       <c r="G82" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="H82">
         <v>2</v>
@@ -7175,33 +7172,33 @@
         <v>35</v>
       </c>
       <c r="M82" t="s">
+        <v>558</v>
+      </c>
+      <c r="N82" t="s">
         <v>559</v>
-      </c>
-      <c r="N82" t="s">
-        <v>560</v>
       </c>
     </row>
     <row r="83" spans="1:14">
       <c r="A83" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="B83" t="s">
         <v>287</v>
       </c>
       <c r="C83" t="s">
+        <v>561</v>
+      </c>
+      <c r="D83" t="s">
         <v>562</v>
       </c>
-      <c r="D83" t="s">
+      <c r="E83" t="s">
         <v>563</v>
-      </c>
-      <c r="E83" t="s">
-        <v>564</v>
       </c>
       <c r="F83" t="s">
         <v>42</v>
       </c>
       <c r="G83" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="H83">
         <v>1</v>
@@ -7216,36 +7213,36 @@
         <v>305</v>
       </c>
       <c r="L83" t="s">
-        <v>35</v>
+        <v>292</v>
       </c>
       <c r="M83" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="N83" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="84" hidden="1" spans="1:14">
+      <c r="A84" t="s">
         <v>566</v>
       </c>
-    </row>
-    <row r="84" spans="1:14">
-      <c r="A84" t="s">
+      <c r="B84" t="s">
         <v>567</v>
       </c>
-      <c r="B84" t="s">
+      <c r="C84" t="s">
         <v>568</v>
       </c>
-      <c r="C84" t="s">
+      <c r="D84" t="s">
         <v>569</v>
       </c>
-      <c r="D84" t="s">
+      <c r="E84" t="s">
         <v>570</v>
-      </c>
-      <c r="E84" t="s">
-        <v>571</v>
       </c>
       <c r="F84" t="s">
         <v>42</v>
       </c>
       <c r="G84" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="H84">
         <v>2</v>
@@ -7257,39 +7254,39 @@
         <v>61</v>
       </c>
       <c r="K84" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L84" t="s">
         <v>292</v>
       </c>
       <c r="M84" t="s">
+        <v>572</v>
+      </c>
+      <c r="N84" t="s">
         <v>573</v>
       </c>
-      <c r="N84" t="s">
+    </row>
+    <row r="85" hidden="1" spans="1:14">
+      <c r="A85" t="s">
         <v>574</v>
       </c>
-    </row>
-    <row r="85" spans="1:14">
-      <c r="A85" t="s">
+      <c r="B85" t="s">
+        <v>541</v>
+      </c>
+      <c r="C85" t="s">
         <v>575</v>
       </c>
-      <c r="B85" t="s">
-        <v>542</v>
-      </c>
-      <c r="C85" t="s">
+      <c r="D85" t="s">
         <v>576</v>
       </c>
-      <c r="D85" t="s">
+      <c r="E85" t="s">
         <v>577</v>
-      </c>
-      <c r="E85" t="s">
-        <v>578</v>
       </c>
       <c r="F85" t="s">
         <v>42</v>
       </c>
       <c r="G85" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="H85">
         <v>3</v>
@@ -7301,39 +7298,39 @@
         <v>44</v>
       </c>
       <c r="K85" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L85" t="s">
         <v>292</v>
       </c>
       <c r="M85" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="N85" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="86" hidden="1" spans="1:14">
+      <c r="A86" t="s">
         <v>580</v>
       </c>
-    </row>
-    <row r="86" spans="1:14">
-      <c r="A86" t="s">
+      <c r="B86" t="s">
+        <v>548</v>
+      </c>
+      <c r="C86" t="s">
         <v>581</v>
       </c>
-      <c r="B86" t="s">
-        <v>549</v>
-      </c>
-      <c r="C86" t="s">
+      <c r="D86" t="s">
         <v>582</v>
       </c>
-      <c r="D86" t="s">
+      <c r="E86" t="s">
         <v>583</v>
-      </c>
-      <c r="E86" t="s">
-        <v>584</v>
       </c>
       <c r="F86" t="s">
         <v>42</v>
       </c>
       <c r="G86" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="H86">
         <v>3</v>
@@ -7345,39 +7342,39 @@
         <v>61</v>
       </c>
       <c r="K86" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L86" t="s">
         <v>292</v>
       </c>
       <c r="M86" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="N86" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="87" hidden="1" spans="1:14">
+      <c r="A87" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="87" spans="1:14">
-      <c r="A87" t="s">
+      <c r="B87" t="s">
+        <v>541</v>
+      </c>
+      <c r="C87" t="s">
         <v>587</v>
       </c>
-      <c r="B87" t="s">
-        <v>542</v>
-      </c>
-      <c r="C87" t="s">
+      <c r="D87" t="s">
         <v>588</v>
       </c>
-      <c r="D87" t="s">
+      <c r="E87" t="s">
         <v>589</v>
       </c>
-      <c r="E87" t="s">
+      <c r="F87" t="s">
         <v>590</v>
       </c>
-      <c r="F87" t="s">
+      <c r="G87" t="s">
         <v>591</v>
-      </c>
-      <c r="G87" t="s">
-        <v>592</v>
       </c>
       <c r="H87">
         <v>3</v>
@@ -7389,7 +7386,7 @@
         <v>44</v>
       </c>
       <c r="K87" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L87" t="s">
         <v>292</v>
@@ -7398,30 +7395,30 @@
         <v>24</v>
       </c>
       <c r="N87" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="88" hidden="1" spans="1:14">
+      <c r="A88" t="s">
         <v>593</v>
       </c>
-    </row>
-    <row r="88" spans="1:14">
-      <c r="A88" t="s">
+      <c r="B88" t="s">
+        <v>548</v>
+      </c>
+      <c r="C88" t="s">
         <v>594</v>
       </c>
-      <c r="B88" t="s">
-        <v>549</v>
-      </c>
-      <c r="C88" t="s">
+      <c r="D88" t="s">
         <v>595</v>
       </c>
-      <c r="D88" t="s">
+      <c r="E88" t="s">
         <v>596</v>
       </c>
-      <c r="E88" t="s">
+      <c r="F88" t="s">
+        <v>590</v>
+      </c>
+      <c r="G88" t="s">
         <v>597</v>
-      </c>
-      <c r="F88" t="s">
-        <v>591</v>
-      </c>
-      <c r="G88" t="s">
-        <v>598</v>
       </c>
       <c r="H88">
         <v>5</v>
@@ -7433,39 +7430,39 @@
         <v>61</v>
       </c>
       <c r="K88" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L88" t="s">
         <v>292</v>
       </c>
       <c r="M88" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="N88" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="89" hidden="1" spans="1:14">
+      <c r="A89" t="s">
         <v>599</v>
-      </c>
-    </row>
-    <row r="89" spans="1:14">
-      <c r="A89" t="s">
-        <v>600</v>
       </c>
       <c r="B89" t="s">
         <v>287</v>
       </c>
       <c r="C89" t="s">
+        <v>600</v>
+      </c>
+      <c r="D89" t="s">
         <v>601</v>
       </c>
-      <c r="D89" t="s">
+      <c r="E89" t="s">
         <v>602</v>
-      </c>
-      <c r="E89" t="s">
-        <v>603</v>
       </c>
       <c r="F89" t="s">
         <v>170</v>
       </c>
       <c r="G89" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H89">
         <v>3</v>
@@ -7477,39 +7474,39 @@
         <v>61</v>
       </c>
       <c r="K89" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L89" t="s">
         <v>292</v>
       </c>
       <c r="M89" t="s">
+        <v>603</v>
+      </c>
+      <c r="N89" t="s">
         <v>604</v>
       </c>
-      <c r="N89" t="s">
+    </row>
+    <row r="90" hidden="1" spans="1:14">
+      <c r="A90" t="s">
         <v>605</v>
       </c>
-    </row>
-    <row r="90" spans="1:14">
-      <c r="A90" t="s">
+      <c r="B90" t="s">
+        <v>548</v>
+      </c>
+      <c r="C90" t="s">
         <v>606</v>
       </c>
-      <c r="B90" t="s">
-        <v>549</v>
-      </c>
-      <c r="C90" t="s">
+      <c r="D90" t="s">
         <v>607</v>
       </c>
-      <c r="D90" t="s">
+      <c r="E90" t="s">
         <v>608</v>
       </c>
-      <c r="E90" t="s">
+      <c r="F90" t="s">
         <v>609</v>
       </c>
-      <c r="F90" t="s">
+      <c r="G90" t="s">
         <v>610</v>
-      </c>
-      <c r="G90" t="s">
-        <v>611</v>
       </c>
       <c r="H90">
         <v>5</v>
@@ -7521,7 +7518,7 @@
         <v>44</v>
       </c>
       <c r="K90" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="L90" t="s">
         <v>292</v>
@@ -7530,30 +7527,30 @@
         <v>24</v>
       </c>
       <c r="N90" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="91" hidden="1" spans="1:14">
+      <c r="A91" t="s">
         <v>612</v>
       </c>
-    </row>
-    <row r="91" spans="1:14">
-      <c r="A91" t="s">
+      <c r="B91" t="s">
+        <v>541</v>
+      </c>
+      <c r="C91" t="s">
         <v>613</v>
       </c>
-      <c r="B91" t="s">
-        <v>542</v>
-      </c>
-      <c r="C91" t="s">
+      <c r="D91" t="s">
         <v>614</v>
       </c>
-      <c r="D91" t="s">
+      <c r="E91" t="s">
         <v>615</v>
       </c>
-      <c r="E91" t="s">
+      <c r="F91" t="s">
         <v>616</v>
       </c>
-      <c r="F91" t="s">
+      <c r="G91" t="s">
         <v>617</v>
-      </c>
-      <c r="G91" t="s">
-        <v>618</v>
       </c>
       <c r="H91">
         <v>3</v>
@@ -7565,7 +7562,7 @@
         <v>95</v>
       </c>
       <c r="K91" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L91" t="s">
         <v>292</v>
@@ -7574,30 +7571,30 @@
         <v>24</v>
       </c>
       <c r="N91" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="92" hidden="1" spans="1:14">
+      <c r="A92" t="s">
         <v>619</v>
       </c>
-    </row>
-    <row r="92" spans="1:14">
-      <c r="A92" t="s">
+      <c r="B92" t="s">
+        <v>548</v>
+      </c>
+      <c r="C92" t="s">
         <v>620</v>
       </c>
-      <c r="B92" t="s">
-        <v>549</v>
-      </c>
-      <c r="C92" t="s">
+      <c r="D92" t="s">
         <v>621</v>
       </c>
-      <c r="D92" t="s">
+      <c r="E92" t="s">
         <v>622</v>
       </c>
-      <c r="E92" t="s">
+      <c r="F92" t="s">
+        <v>616</v>
+      </c>
+      <c r="G92" t="s">
         <v>623</v>
-      </c>
-      <c r="F92" t="s">
-        <v>617</v>
-      </c>
-      <c r="G92" t="s">
-        <v>624</v>
       </c>
       <c r="H92">
         <v>5</v>
@@ -7609,39 +7606,39 @@
         <v>61</v>
       </c>
       <c r="K92" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L92" t="s">
         <v>292</v>
       </c>
       <c r="M92" t="s">
+        <v>624</v>
+      </c>
+      <c r="N92" t="s">
         <v>625</v>
       </c>
-      <c r="N92" t="s">
+    </row>
+    <row r="93" hidden="1" spans="1:14">
+      <c r="A93" t="s">
         <v>626</v>
       </c>
-    </row>
-    <row r="93" spans="1:14">
-      <c r="A93" t="s">
+      <c r="B93" t="s">
+        <v>548</v>
+      </c>
+      <c r="C93" t="s">
         <v>627</v>
       </c>
-      <c r="B93" t="s">
-        <v>549</v>
-      </c>
-      <c r="C93" t="s">
+      <c r="D93" t="s">
         <v>628</v>
       </c>
-      <c r="D93" t="s">
+      <c r="E93" t="s">
         <v>629</v>
       </c>
-      <c r="E93" t="s">
+      <c r="F93" t="s">
         <v>630</v>
       </c>
-      <c r="F93" t="s">
+      <c r="G93" t="s">
         <v>631</v>
-      </c>
-      <c r="G93" t="s">
-        <v>632</v>
       </c>
       <c r="H93">
         <v>3</v>
@@ -7653,7 +7650,7 @@
         <v>206</v>
       </c>
       <c r="K93" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L93" t="s">
         <v>292</v>
@@ -7662,30 +7659,30 @@
         <v>24</v>
       </c>
       <c r="N93" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="94" hidden="1" spans="1:14">
+      <c r="A94" t="s">
         <v>633</v>
-      </c>
-    </row>
-    <row r="94" spans="1:14">
-      <c r="A94" t="s">
-        <v>634</v>
       </c>
       <c r="B94" t="s">
         <v>287</v>
       </c>
       <c r="C94" t="s">
+        <v>634</v>
+      </c>
+      <c r="D94" t="s">
         <v>635</v>
       </c>
-      <c r="D94" t="s">
+      <c r="E94" t="s">
         <v>636</v>
-      </c>
-      <c r="E94" t="s">
-        <v>637</v>
       </c>
       <c r="F94" t="s">
         <v>211</v>
       </c>
       <c r="G94" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="H94">
         <v>2</v>
@@ -7697,7 +7694,7 @@
         <v>44</v>
       </c>
       <c r="K94" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L94" t="s">
         <v>292</v>
@@ -7706,30 +7703,30 @@
         <v>24</v>
       </c>
       <c r="N94" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="95" hidden="1" spans="1:14">
+      <c r="A95" t="s">
         <v>639</v>
-      </c>
-    </row>
-    <row r="95" spans="1:14">
-      <c r="A95" t="s">
-        <v>640</v>
       </c>
       <c r="B95" t="s">
         <v>287</v>
       </c>
       <c r="C95" t="s">
+        <v>640</v>
+      </c>
+      <c r="D95" t="s">
         <v>641</v>
       </c>
-      <c r="D95" t="s">
+      <c r="E95" t="s">
         <v>642</v>
       </c>
-      <c r="E95" t="s">
+      <c r="F95" t="s">
+        <v>590</v>
+      </c>
+      <c r="G95" t="s">
         <v>643</v>
-      </c>
-      <c r="F95" t="s">
-        <v>591</v>
-      </c>
-      <c r="G95" t="s">
-        <v>644</v>
       </c>
       <c r="H95">
         <v>2</v>
@@ -7741,39 +7738,39 @@
         <v>44</v>
       </c>
       <c r="K95" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L95" t="s">
         <v>292</v>
       </c>
       <c r="M95" t="s">
+        <v>644</v>
+      </c>
+      <c r="N95" t="s">
         <v>645</v>
       </c>
-      <c r="N95" t="s">
+    </row>
+    <row r="96" hidden="1" spans="1:14">
+      <c r="A96" t="s">
         <v>646</v>
       </c>
-    </row>
-    <row r="96" spans="1:14">
-      <c r="A96" t="s">
+      <c r="B96" t="s">
+        <v>541</v>
+      </c>
+      <c r="C96" t="s">
         <v>647</v>
       </c>
-      <c r="B96" t="s">
-        <v>542</v>
-      </c>
-      <c r="C96" t="s">
+      <c r="D96" t="s">
         <v>648</v>
       </c>
-      <c r="D96" t="s">
+      <c r="E96" t="s">
         <v>649</v>
       </c>
-      <c r="E96" t="s">
+      <c r="F96" t="s">
         <v>650</v>
       </c>
-      <c r="F96" t="s">
-        <v>651</v>
-      </c>
       <c r="G96" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="H96">
         <v>3</v>
@@ -7785,39 +7782,39 @@
         <v>95</v>
       </c>
       <c r="K96" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L96" t="s">
         <v>292</v>
       </c>
       <c r="M96" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="N96" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="97" hidden="1" spans="1:14">
+      <c r="A97" t="s">
         <v>652</v>
-      </c>
-    </row>
-    <row r="97" spans="1:14">
-      <c r="A97" t="s">
-        <v>653</v>
       </c>
       <c r="B97" t="s">
         <v>287</v>
       </c>
       <c r="C97" t="s">
+        <v>653</v>
+      </c>
+      <c r="D97" t="s">
         <v>654</v>
       </c>
-      <c r="D97" t="s">
+      <c r="E97" t="s">
         <v>655</v>
       </c>
-      <c r="E97" t="s">
-        <v>656</v>
-      </c>
       <c r="F97" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="G97" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H97">
         <v>3</v>
@@ -7829,39 +7826,39 @@
         <v>61</v>
       </c>
       <c r="K97" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L97" t="s">
         <v>292</v>
       </c>
       <c r="M97" t="s">
+        <v>656</v>
+      </c>
+      <c r="N97" t="s">
         <v>657</v>
       </c>
-      <c r="N97" t="s">
+    </row>
+    <row r="98" hidden="1" spans="1:14">
+      <c r="A98" t="s">
         <v>658</v>
-      </c>
-    </row>
-    <row r="98" spans="1:14">
-      <c r="A98" t="s">
-        <v>659</v>
       </c>
       <c r="B98" t="s">
         <v>287</v>
       </c>
       <c r="C98" t="s">
+        <v>659</v>
+      </c>
+      <c r="D98" t="s">
         <v>660</v>
       </c>
-      <c r="D98" t="s">
+      <c r="E98" t="s">
         <v>661</v>
       </c>
-      <c r="E98" t="s">
+      <c r="F98" t="s">
+        <v>609</v>
+      </c>
+      <c r="G98" t="s">
         <v>662</v>
-      </c>
-      <c r="F98" t="s">
-        <v>610</v>
-      </c>
-      <c r="G98" t="s">
-        <v>663</v>
       </c>
       <c r="H98">
         <v>2</v>
@@ -7870,10 +7867,10 @@
         <v>21</v>
       </c>
       <c r="J98" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="K98" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L98" t="s">
         <v>292</v>
@@ -7882,30 +7879,30 @@
         <v>24</v>
       </c>
       <c r="N98" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="99" hidden="1" spans="1:14">
+      <c r="A99" t="s">
         <v>665</v>
-      </c>
-    </row>
-    <row r="99" spans="1:14">
-      <c r="A99" t="s">
-        <v>666</v>
       </c>
       <c r="B99" t="s">
         <v>287</v>
       </c>
       <c r="C99" t="s">
+        <v>666</v>
+      </c>
+      <c r="D99" t="s">
         <v>667</v>
       </c>
-      <c r="D99" t="s">
+      <c r="E99" t="s">
         <v>668</v>
-      </c>
-      <c r="E99" t="s">
-        <v>669</v>
       </c>
       <c r="F99" t="s">
         <v>42</v>
       </c>
       <c r="G99" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="H99">
         <v>1</v>
@@ -7917,39 +7914,39 @@
         <v>44</v>
       </c>
       <c r="K99" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L99" t="s">
         <v>292</v>
       </c>
       <c r="M99" t="s">
+        <v>670</v>
+      </c>
+      <c r="N99" t="s">
         <v>671</v>
       </c>
-      <c r="N99" t="s">
+    </row>
+    <row r="100" hidden="1" spans="1:14">
+      <c r="A100" t="s">
         <v>672</v>
-      </c>
-    </row>
-    <row r="100" spans="1:14">
-      <c r="A100" t="s">
-        <v>673</v>
       </c>
       <c r="B100" t="s">
         <v>287</v>
       </c>
       <c r="C100" t="s">
+        <v>673</v>
+      </c>
+      <c r="D100" t="s">
         <v>674</v>
       </c>
-      <c r="D100" t="s">
+      <c r="E100" t="s">
         <v>675</v>
-      </c>
-      <c r="E100" t="s">
-        <v>676</v>
       </c>
       <c r="F100" t="s">
         <v>42</v>
       </c>
       <c r="G100" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="H100">
         <v>1</v>
@@ -7961,39 +7958,39 @@
         <v>44</v>
       </c>
       <c r="K100" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L100" t="s">
         <v>292</v>
       </c>
       <c r="M100" t="s">
+        <v>677</v>
+      </c>
+      <c r="N100" t="s">
         <v>678</v>
       </c>
-      <c r="N100" t="s">
+    </row>
+    <row r="101" hidden="1" spans="1:14">
+      <c r="A101" t="s">
         <v>679</v>
-      </c>
-    </row>
-    <row r="101" spans="1:14">
-      <c r="A101" t="s">
-        <v>680</v>
       </c>
       <c r="B101" t="s">
         <v>287</v>
       </c>
       <c r="C101" t="s">
+        <v>680</v>
+      </c>
+      <c r="D101" t="s">
         <v>681</v>
       </c>
-      <c r="D101" t="s">
+      <c r="E101" t="s">
         <v>682</v>
-      </c>
-      <c r="E101" t="s">
-        <v>683</v>
       </c>
       <c r="F101" t="s">
         <v>42</v>
       </c>
       <c r="G101" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="H101">
         <v>1</v>
@@ -8005,39 +8002,39 @@
         <v>44</v>
       </c>
       <c r="K101" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L101" t="s">
         <v>292</v>
       </c>
       <c r="M101" t="s">
+        <v>684</v>
+      </c>
+      <c r="N101" t="s">
         <v>685</v>
       </c>
-      <c r="N101" t="s">
+    </row>
+    <row r="102" hidden="1" spans="1:14">
+      <c r="A102" t="s">
         <v>686</v>
-      </c>
-    </row>
-    <row r="102" spans="1:14">
-      <c r="A102" t="s">
-        <v>687</v>
       </c>
       <c r="B102" t="s">
         <v>287</v>
       </c>
       <c r="C102" t="s">
+        <v>687</v>
+      </c>
+      <c r="D102" t="s">
         <v>688</v>
       </c>
-      <c r="D102" t="s">
+      <c r="E102" t="s">
         <v>689</v>
-      </c>
-      <c r="E102" t="s">
-        <v>690</v>
       </c>
       <c r="F102" t="s">
         <v>42</v>
       </c>
       <c r="G102" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="H102">
         <v>2</v>
@@ -8049,39 +8046,39 @@
         <v>61</v>
       </c>
       <c r="K102" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L102" t="s">
         <v>292</v>
       </c>
       <c r="M102" t="s">
+        <v>691</v>
+      </c>
+      <c r="N102" t="s">
         <v>692</v>
       </c>
-      <c r="N102" t="s">
+    </row>
+    <row r="103" hidden="1" spans="1:14">
+      <c r="A103" t="s">
         <v>693</v>
-      </c>
-    </row>
-    <row r="103" spans="1:14">
-      <c r="A103" t="s">
-        <v>694</v>
       </c>
       <c r="B103" t="s">
         <v>287</v>
       </c>
       <c r="C103" t="s">
+        <v>694</v>
+      </c>
+      <c r="D103" t="s">
         <v>695</v>
       </c>
-      <c r="D103" t="s">
+      <c r="E103" t="s">
         <v>696</v>
-      </c>
-      <c r="E103" t="s">
-        <v>697</v>
       </c>
       <c r="F103" t="s">
         <v>42</v>
       </c>
       <c r="G103" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="H103">
         <v>2</v>
@@ -8093,39 +8090,39 @@
         <v>61</v>
       </c>
       <c r="K103" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L103" t="s">
         <v>292</v>
       </c>
       <c r="M103" t="s">
+        <v>698</v>
+      </c>
+      <c r="N103" t="s">
         <v>699</v>
       </c>
-      <c r="N103" t="s">
+    </row>
+    <row r="104" hidden="1" spans="1:14">
+      <c r="A104" t="s">
         <v>700</v>
-      </c>
-    </row>
-    <row r="104" spans="1:14">
-      <c r="A104" t="s">
-        <v>701</v>
       </c>
       <c r="B104" t="s">
         <v>287</v>
       </c>
       <c r="C104" t="s">
+        <v>701</v>
+      </c>
+      <c r="D104" t="s">
         <v>702</v>
       </c>
-      <c r="D104" t="s">
+      <c r="E104" t="s">
         <v>703</v>
-      </c>
-      <c r="E104" t="s">
-        <v>704</v>
       </c>
       <c r="F104" t="s">
         <v>42</v>
       </c>
       <c r="G104" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="H104">
         <v>2</v>
@@ -8137,39 +8134,39 @@
         <v>61</v>
       </c>
       <c r="K104" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L104" t="s">
         <v>292</v>
       </c>
       <c r="M104" t="s">
+        <v>705</v>
+      </c>
+      <c r="N104" t="s">
         <v>706</v>
       </c>
-      <c r="N104" t="s">
+    </row>
+    <row r="105" hidden="1" spans="1:14">
+      <c r="A105" t="s">
         <v>707</v>
-      </c>
-    </row>
-    <row r="105" spans="1:14">
-      <c r="A105" t="s">
-        <v>708</v>
       </c>
       <c r="B105" t="s">
         <v>287</v>
       </c>
       <c r="C105" t="s">
+        <v>708</v>
+      </c>
+      <c r="D105" t="s">
         <v>709</v>
       </c>
-      <c r="D105" t="s">
+      <c r="E105" t="s">
         <v>710</v>
-      </c>
-      <c r="E105" t="s">
-        <v>711</v>
       </c>
       <c r="F105" t="s">
         <v>42</v>
       </c>
       <c r="G105" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H105">
         <v>1</v>
@@ -8181,39 +8178,39 @@
         <v>121</v>
       </c>
       <c r="K105" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L105" t="s">
         <v>292</v>
       </c>
       <c r="M105" t="s">
+        <v>711</v>
+      </c>
+      <c r="N105" t="s">
         <v>712</v>
       </c>
-      <c r="N105" t="s">
+    </row>
+    <row r="106" hidden="1" spans="1:14">
+      <c r="A106" t="s">
         <v>713</v>
-      </c>
-    </row>
-    <row r="106" spans="1:14">
-      <c r="A106" t="s">
-        <v>714</v>
       </c>
       <c r="B106" t="s">
         <v>287</v>
       </c>
       <c r="C106" t="s">
+        <v>714</v>
+      </c>
+      <c r="D106" t="s">
         <v>715</v>
       </c>
-      <c r="D106" t="s">
+      <c r="E106" t="s">
         <v>716</v>
       </c>
-      <c r="E106" t="s">
+      <c r="F106" t="s">
+        <v>590</v>
+      </c>
+      <c r="G106" t="s">
         <v>717</v>
-      </c>
-      <c r="F106" t="s">
-        <v>591</v>
-      </c>
-      <c r="G106" t="s">
-        <v>718</v>
       </c>
       <c r="H106">
         <v>1</v>
@@ -8225,39 +8222,39 @@
         <v>44</v>
       </c>
       <c r="K106" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L106" t="s">
         <v>292</v>
       </c>
       <c r="M106" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="N106" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="107" hidden="1" spans="1:14">
+      <c r="A107" t="s">
         <v>719</v>
-      </c>
-    </row>
-    <row r="107" spans="1:14">
-      <c r="A107" t="s">
-        <v>720</v>
       </c>
       <c r="B107" t="s">
         <v>287</v>
       </c>
       <c r="C107" t="s">
+        <v>720</v>
+      </c>
+      <c r="D107" t="s">
         <v>721</v>
       </c>
-      <c r="D107" t="s">
+      <c r="E107" t="s">
         <v>722</v>
       </c>
-      <c r="E107" t="s">
+      <c r="F107" t="s">
+        <v>590</v>
+      </c>
+      <c r="G107" t="s">
         <v>723</v>
-      </c>
-      <c r="F107" t="s">
-        <v>591</v>
-      </c>
-      <c r="G107" t="s">
-        <v>724</v>
       </c>
       <c r="H107">
         <v>1</v>
@@ -8269,39 +8266,39 @@
         <v>44</v>
       </c>
       <c r="K107" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L107" t="s">
         <v>292</v>
       </c>
       <c r="M107" t="s">
+        <v>724</v>
+      </c>
+      <c r="N107" t="s">
         <v>725</v>
       </c>
-      <c r="N107" t="s">
+    </row>
+    <row r="108" hidden="1" spans="1:14">
+      <c r="A108" t="s">
         <v>726</v>
-      </c>
-    </row>
-    <row r="108" spans="1:14">
-      <c r="A108" t="s">
-        <v>727</v>
       </c>
       <c r="B108" t="s">
         <v>287</v>
       </c>
       <c r="C108" t="s">
+        <v>727</v>
+      </c>
+      <c r="D108" t="s">
         <v>728</v>
       </c>
-      <c r="D108" t="s">
+      <c r="E108" t="s">
         <v>729</v>
       </c>
-      <c r="E108" t="s">
+      <c r="F108" t="s">
+        <v>590</v>
+      </c>
+      <c r="G108" t="s">
         <v>730</v>
-      </c>
-      <c r="F108" t="s">
-        <v>591</v>
-      </c>
-      <c r="G108" t="s">
-        <v>731</v>
       </c>
       <c r="H108">
         <v>2</v>
@@ -8313,39 +8310,39 @@
         <v>61</v>
       </c>
       <c r="K108" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L108" t="s">
         <v>292</v>
       </c>
       <c r="M108" t="s">
+        <v>731</v>
+      </c>
+      <c r="N108" t="s">
         <v>732</v>
       </c>
-      <c r="N108" t="s">
+    </row>
+    <row r="109" hidden="1" spans="1:14">
+      <c r="A109" t="s">
         <v>733</v>
-      </c>
-    </row>
-    <row r="109" spans="1:14">
-      <c r="A109" t="s">
-        <v>734</v>
       </c>
       <c r="B109" t="s">
         <v>287</v>
       </c>
       <c r="C109" t="s">
+        <v>734</v>
+      </c>
+      <c r="D109" t="s">
         <v>735</v>
       </c>
-      <c r="D109" t="s">
+      <c r="E109" t="s">
         <v>736</v>
       </c>
-      <c r="E109" t="s">
+      <c r="F109" t="s">
+        <v>590</v>
+      </c>
+      <c r="G109" t="s">
         <v>737</v>
-      </c>
-      <c r="F109" t="s">
-        <v>591</v>
-      </c>
-      <c r="G109" t="s">
-        <v>738</v>
       </c>
       <c r="H109">
         <v>2</v>
@@ -8357,39 +8354,39 @@
         <v>61</v>
       </c>
       <c r="K109" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L109" t="s">
         <v>292</v>
       </c>
       <c r="M109" t="s">
+        <v>738</v>
+      </c>
+      <c r="N109" t="s">
         <v>739</v>
       </c>
-      <c r="N109" t="s">
+    </row>
+    <row r="110" hidden="1" spans="1:14">
+      <c r="A110" t="s">
         <v>740</v>
-      </c>
-    </row>
-    <row r="110" spans="1:14">
-      <c r="A110" t="s">
-        <v>741</v>
       </c>
       <c r="B110" t="s">
         <v>287</v>
       </c>
       <c r="C110" t="s">
+        <v>741</v>
+      </c>
+      <c r="D110" t="s">
         <v>742</v>
       </c>
-      <c r="D110" t="s">
+      <c r="E110" t="s">
         <v>743</v>
       </c>
-      <c r="E110" t="s">
+      <c r="F110" t="s">
+        <v>590</v>
+      </c>
+      <c r="G110" t="s">
         <v>744</v>
-      </c>
-      <c r="F110" t="s">
-        <v>591</v>
-      </c>
-      <c r="G110" t="s">
-        <v>745</v>
       </c>
       <c r="H110">
         <v>1</v>
@@ -8401,39 +8398,39 @@
         <v>121</v>
       </c>
       <c r="K110" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L110" t="s">
         <v>292</v>
       </c>
       <c r="M110" t="s">
+        <v>745</v>
+      </c>
+      <c r="N110" t="s">
         <v>746</v>
       </c>
-      <c r="N110" t="s">
+    </row>
+    <row r="111" hidden="1" spans="1:14">
+      <c r="A111" t="s">
         <v>747</v>
-      </c>
-    </row>
-    <row r="111" spans="1:14">
-      <c r="A111" t="s">
-        <v>748</v>
       </c>
       <c r="B111" t="s">
         <v>287</v>
       </c>
       <c r="C111" t="s">
+        <v>748</v>
+      </c>
+      <c r="D111" t="s">
         <v>749</v>
       </c>
-      <c r="D111" t="s">
+      <c r="E111" t="s">
         <v>750</v>
       </c>
-      <c r="E111" t="s">
+      <c r="F111" t="s">
+        <v>616</v>
+      </c>
+      <c r="G111" t="s">
         <v>751</v>
-      </c>
-      <c r="F111" t="s">
-        <v>617</v>
-      </c>
-      <c r="G111" t="s">
-        <v>752</v>
       </c>
       <c r="H111">
         <v>1</v>
@@ -8445,39 +8442,39 @@
         <v>95</v>
       </c>
       <c r="K111" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L111" t="s">
         <v>292</v>
       </c>
       <c r="M111" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="N111" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="112" hidden="1" spans="1:14">
+      <c r="A112" t="s">
         <v>753</v>
-      </c>
-    </row>
-    <row r="112" spans="1:14">
-      <c r="A112" t="s">
-        <v>754</v>
       </c>
       <c r="B112" t="s">
         <v>287</v>
       </c>
       <c r="C112" t="s">
+        <v>754</v>
+      </c>
+      <c r="D112" t="s">
         <v>755</v>
       </c>
-      <c r="D112" t="s">
+      <c r="E112" t="s">
         <v>756</v>
       </c>
-      <c r="E112" t="s">
+      <c r="F112" t="s">
+        <v>616</v>
+      </c>
+      <c r="G112" t="s">
         <v>757</v>
-      </c>
-      <c r="F112" t="s">
-        <v>617</v>
-      </c>
-      <c r="G112" t="s">
-        <v>758</v>
       </c>
       <c r="H112">
         <v>1</v>
@@ -8489,39 +8486,39 @@
         <v>95</v>
       </c>
       <c r="K112" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L112" t="s">
         <v>292</v>
       </c>
       <c r="M112" t="s">
+        <v>758</v>
+      </c>
+      <c r="N112" t="s">
         <v>759</v>
       </c>
-      <c r="N112" t="s">
+    </row>
+    <row r="113" hidden="1" spans="1:14">
+      <c r="A113" t="s">
         <v>760</v>
-      </c>
-    </row>
-    <row r="113" spans="1:14">
-      <c r="A113" t="s">
-        <v>761</v>
       </c>
       <c r="B113" t="s">
         <v>287</v>
       </c>
       <c r="C113" t="s">
+        <v>761</v>
+      </c>
+      <c r="D113" t="s">
         <v>762</v>
       </c>
-      <c r="D113" t="s">
+      <c r="E113" t="s">
         <v>763</v>
       </c>
-      <c r="E113" t="s">
+      <c r="F113" t="s">
+        <v>609</v>
+      </c>
+      <c r="G113" t="s">
         <v>764</v>
-      </c>
-      <c r="F113" t="s">
-        <v>610</v>
-      </c>
-      <c r="G113" t="s">
-        <v>765</v>
       </c>
       <c r="H113">
         <v>1</v>
@@ -8533,39 +8530,39 @@
         <v>44</v>
       </c>
       <c r="K113" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="L113" t="s">
         <v>292</v>
       </c>
       <c r="M113" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="N113" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="114" hidden="1" spans="1:14">
+      <c r="A114" t="s">
         <v>766</v>
-      </c>
-    </row>
-    <row r="114" spans="1:14">
-      <c r="A114" t="s">
-        <v>767</v>
       </c>
       <c r="B114" t="s">
         <v>287</v>
       </c>
       <c r="C114" t="s">
+        <v>767</v>
+      </c>
+      <c r="D114" t="s">
         <v>768</v>
       </c>
-      <c r="D114" t="s">
+      <c r="E114" t="s">
         <v>769</v>
       </c>
-      <c r="E114" t="s">
+      <c r="F114" t="s">
+        <v>609</v>
+      </c>
+      <c r="G114" t="s">
         <v>770</v>
-      </c>
-      <c r="F114" t="s">
-        <v>610</v>
-      </c>
-      <c r="G114" t="s">
-        <v>771</v>
       </c>
       <c r="H114">
         <v>2</v>
@@ -8577,39 +8574,39 @@
         <v>61</v>
       </c>
       <c r="K114" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="L114" t="s">
-        <v>35</v>
+        <v>292</v>
       </c>
       <c r="M114" t="s">
+        <v>771</v>
+      </c>
+      <c r="N114" t="s">
         <v>772</v>
       </c>
-      <c r="N114" t="s">
+    </row>
+    <row r="115" hidden="1" spans="1:14">
+      <c r="A115" t="s">
         <v>773</v>
-      </c>
-    </row>
-    <row r="115" spans="1:14">
-      <c r="A115" t="s">
-        <v>774</v>
       </c>
       <c r="B115" t="s">
         <v>287</v>
       </c>
       <c r="C115" t="s">
+        <v>774</v>
+      </c>
+      <c r="D115" t="s">
         <v>775</v>
       </c>
-      <c r="D115" t="s">
+      <c r="E115" t="s">
         <v>776</v>
       </c>
-      <c r="E115" t="s">
+      <c r="F115" t="s">
+        <v>609</v>
+      </c>
+      <c r="G115" t="s">
         <v>777</v>
-      </c>
-      <c r="F115" t="s">
-        <v>610</v>
-      </c>
-      <c r="G115" t="s">
-        <v>778</v>
       </c>
       <c r="H115">
         <v>2</v>
@@ -8621,39 +8618,39 @@
         <v>61</v>
       </c>
       <c r="K115" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="L115" t="s">
         <v>292</v>
       </c>
       <c r="M115" t="s">
+        <v>778</v>
+      </c>
+      <c r="N115" t="s">
         <v>779</v>
       </c>
-      <c r="N115" t="s">
+    </row>
+    <row r="116" hidden="1" spans="1:14">
+      <c r="A116" t="s">
         <v>780</v>
-      </c>
-    </row>
-    <row r="116" spans="1:14">
-      <c r="A116" t="s">
-        <v>781</v>
       </c>
       <c r="B116" t="s">
         <v>287</v>
       </c>
       <c r="C116" t="s">
+        <v>781</v>
+      </c>
+      <c r="D116" t="s">
         <v>782</v>
       </c>
-      <c r="D116" t="s">
+      <c r="E116" t="s">
         <v>783</v>
       </c>
-      <c r="E116" t="s">
+      <c r="F116" t="s">
+        <v>630</v>
+      </c>
+      <c r="G116" t="s">
         <v>784</v>
-      </c>
-      <c r="F116" t="s">
-        <v>631</v>
-      </c>
-      <c r="G116" t="s">
-        <v>785</v>
       </c>
       <c r="H116">
         <v>2</v>
@@ -8665,39 +8662,39 @@
         <v>206</v>
       </c>
       <c r="K116" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L116" t="s">
         <v>292</v>
       </c>
       <c r="M116" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="N116" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="117" hidden="1" spans="1:14">
+      <c r="A117" t="s">
         <v>786</v>
-      </c>
-    </row>
-    <row r="117" spans="1:14">
-      <c r="A117" t="s">
-        <v>787</v>
       </c>
       <c r="B117" t="s">
         <v>287</v>
       </c>
       <c r="C117" t="s">
+        <v>787</v>
+      </c>
+      <c r="D117" t="s">
         <v>788</v>
       </c>
-      <c r="D117" t="s">
+      <c r="E117" t="s">
         <v>789</v>
       </c>
-      <c r="E117" t="s">
+      <c r="F117" t="s">
+        <v>630</v>
+      </c>
+      <c r="G117" t="s">
         <v>790</v>
-      </c>
-      <c r="F117" t="s">
-        <v>631</v>
-      </c>
-      <c r="G117" t="s">
-        <v>791</v>
       </c>
       <c r="H117">
         <v>1</v>
@@ -8709,39 +8706,39 @@
         <v>206</v>
       </c>
       <c r="K117" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L117" t="s">
         <v>292</v>
       </c>
       <c r="M117" t="s">
+        <v>791</v>
+      </c>
+      <c r="N117" t="s">
         <v>792</v>
       </c>
-      <c r="N117" t="s">
+    </row>
+    <row r="118" hidden="1" spans="1:14">
+      <c r="A118" t="s">
         <v>793</v>
-      </c>
-    </row>
-    <row r="118" spans="1:14">
-      <c r="A118" t="s">
-        <v>794</v>
       </c>
       <c r="B118" t="s">
         <v>287</v>
       </c>
       <c r="C118" t="s">
+        <v>794</v>
+      </c>
+      <c r="D118" t="s">
         <v>795</v>
       </c>
-      <c r="D118" t="s">
+      <c r="E118" t="s">
         <v>796</v>
       </c>
-      <c r="E118" t="s">
+      <c r="F118" t="s">
+        <v>650</v>
+      </c>
+      <c r="G118" t="s">
         <v>797</v>
-      </c>
-      <c r="F118" t="s">
-        <v>651</v>
-      </c>
-      <c r="G118" t="s">
-        <v>798</v>
       </c>
       <c r="H118">
         <v>1</v>
@@ -8753,39 +8750,39 @@
         <v>95</v>
       </c>
       <c r="K118" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L118" t="s">
         <v>292</v>
       </c>
       <c r="M118" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="N118" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="119" hidden="1" spans="1:14">
+      <c r="A119" t="s">
         <v>799</v>
-      </c>
-    </row>
-    <row r="119" spans="1:14">
-      <c r="A119" t="s">
-        <v>800</v>
       </c>
       <c r="B119" t="s">
         <v>287</v>
       </c>
       <c r="C119" t="s">
+        <v>800</v>
+      </c>
+      <c r="D119" t="s">
         <v>801</v>
       </c>
-      <c r="D119" t="s">
+      <c r="E119" t="s">
         <v>802</v>
       </c>
-      <c r="E119" t="s">
+      <c r="F119" t="s">
+        <v>650</v>
+      </c>
+      <c r="G119" t="s">
         <v>803</v>
-      </c>
-      <c r="F119" t="s">
-        <v>651</v>
-      </c>
-      <c r="G119" t="s">
-        <v>804</v>
       </c>
       <c r="H119">
         <v>1</v>
@@ -8797,39 +8794,39 @@
         <v>95</v>
       </c>
       <c r="K119" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L119" t="s">
         <v>292</v>
       </c>
       <c r="M119" t="s">
+        <v>804</v>
+      </c>
+      <c r="N119" t="s">
         <v>805</v>
       </c>
-      <c r="N119" t="s">
+    </row>
+    <row r="120" hidden="1" spans="1:14">
+      <c r="A120" t="s">
         <v>806</v>
       </c>
-    </row>
-    <row r="120" spans="1:14">
-      <c r="A120" t="s">
+      <c r="B120" t="s">
+        <v>548</v>
+      </c>
+      <c r="C120" t="s">
         <v>807</v>
       </c>
-      <c r="B120" t="s">
-        <v>549</v>
-      </c>
-      <c r="C120" t="s">
+      <c r="D120" t="s">
         <v>808</v>
       </c>
-      <c r="D120" t="s">
+      <c r="E120" t="s">
         <v>809</v>
-      </c>
-      <c r="E120" t="s">
-        <v>810</v>
       </c>
       <c r="F120" t="s">
         <v>211</v>
       </c>
       <c r="G120" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="H120">
         <v>3</v>
@@ -8841,7 +8838,7 @@
         <v>44</v>
       </c>
       <c r="K120" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L120" t="s">
         <v>292</v>
@@ -8850,16 +8847,21 @@
         <v>24</v>
       </c>
       <c r="N120" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="121" hidden="1" spans="1:14">
+      <c r="D121" t="s">
         <v>812</v>
-      </c>
-    </row>
-    <row r="121" spans="1:14">
-      <c r="D121" t="s">
-        <v>813</v>
       </c>
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:N121" etc:filterBottomFollowUsedRange="0">
+    <filterColumn colId="10">
+      <filters>
+        <filter val="Sprint 3"/>
+      </filters>
+    </filterColumn>
     <extLst/>
   </autoFilter>
   <sortState ref="A2:N84">
@@ -8886,7 +8888,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L$1:L$1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L42 L47 L52 L57 L62 L67 L72 L77 L1:L41 L43:L46 L48:L51 L53:L56 L58:L61 L63:L66 L68:L71 L73:L76 L78:L1048576">
       <formula1>"Planned,Deferred,In-Progress,Completed,Draft,Blocked"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
backlog.xlsx now made readable to csv
</commit_message>
<xml_diff>
--- a/backlog/backlog.xlsx
+++ b/backlog/backlog.xlsx
@@ -10,7 +10,7 @@
     <sheet name="backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">backlog!$A$1:$N$128</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">backlog!$A$1:$N$138</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -9438,7 +9438,7 @@
         <v>61</v>
       </c>
       <c r="L126" t="s">
-        <v>186</v>
+        <v>45</v>
       </c>
       <c r="M126" t="s">
         <v>850</v>
@@ -9479,7 +9479,7 @@
         <v>61</v>
       </c>
       <c r="L127" t="s">
-        <v>35</v>
+        <v>186</v>
       </c>
       <c r="M127" t="s">
         <v>850</v>
@@ -9940,7 +9940,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:N128" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:N138" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <sortState ref="A2:N84">
@@ -9967,7 +9967,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L1:L120 L121:L122 L123:L129 L130:L138 L139:L1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L$1:L$1048576">
       <formula1>"Planned,Deferred,In-Progress,Completed,Draft,Blocked"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
test(PBI-131): validate auditor access history query flow
</commit_message>
<xml_diff>
--- a/backlog/backlog.xlsx
+++ b/backlog/backlog.xlsx
@@ -9684,7 +9684,7 @@
         <v>121</v>
       </c>
       <c r="L132" t="s">
-        <v>186</v>
+        <v>45</v>
       </c>
       <c r="M132" t="s">
         <v>888</v>
@@ -9725,7 +9725,7 @@
         <v>121</v>
       </c>
       <c r="L133" t="s">
-        <v>35</v>
+        <v>186</v>
       </c>
       <c r="M133" t="s">
         <v>895</v>

</xml_diff>

<commit_message>
docs(PBI-132): close auditor access history search story
</commit_message>
<xml_diff>
--- a/backlog/backlog.xlsx
+++ b/backlog/backlog.xlsx
@@ -9274,7 +9274,7 @@
         <v>95</v>
       </c>
       <c r="L122" t="s">
-        <v>186</v>
+        <v>45</v>
       </c>
       <c r="M122" t="s">
         <v>823</v>
@@ -9315,7 +9315,7 @@
         <v>95</v>
       </c>
       <c r="L123" t="s">
-        <v>35</v>
+        <v>186</v>
       </c>
       <c r="M123" t="s">
         <v>829</v>
@@ -9725,7 +9725,7 @@
         <v>121</v>
       </c>
       <c r="L133" t="s">
-        <v>186</v>
+        <v>45</v>
       </c>
       <c r="M133" t="s">
         <v>895</v>
@@ -9766,7 +9766,7 @@
         <v>95</v>
       </c>
       <c r="L134" t="s">
-        <v>35</v>
+        <v>186</v>
       </c>
       <c r="M134" t="s">
         <v>902</v>

</xml_diff>

<commit_message>
docs(PBI-133): define audit event inspection contract
</commit_message>
<xml_diff>
--- a/backlog/backlog.xlsx
+++ b/backlog/backlog.xlsx
@@ -9766,7 +9766,7 @@
         <v>95</v>
       </c>
       <c r="L134" t="s">
-        <v>186</v>
+        <v>45</v>
       </c>
       <c r="M134" t="s">
         <v>902</v>
@@ -9807,7 +9807,7 @@
         <v>61</v>
       </c>
       <c r="L135" t="s">
-        <v>35</v>
+        <v>186</v>
       </c>
       <c r="M135" t="s">
         <v>909</v>

</xml_diff>

<commit_message>
feat(PBI-134): add auditor access audit event detail retrieval
</commit_message>
<xml_diff>
--- a/backlog/backlog.xlsx
+++ b/backlog/backlog.xlsx
@@ -9807,7 +9807,7 @@
         <v>61</v>
       </c>
       <c r="L135" t="s">
-        <v>186</v>
+        <v>45</v>
       </c>
       <c r="M135" t="s">
         <v>909</v>
@@ -9848,7 +9848,7 @@
         <v>61</v>
       </c>
       <c r="L136" t="s">
-        <v>35</v>
+        <v>186</v>
       </c>
       <c r="M136" t="s">
         <v>915</v>

</xml_diff>

<commit_message>
feat(PBI-135): add auditor access audit event sequence retrieval
</commit_message>
<xml_diff>
--- a/backlog/backlog.xlsx
+++ b/backlog/backlog.xlsx
@@ -9848,7 +9848,7 @@
         <v>61</v>
       </c>
       <c r="L136" t="s">
-        <v>186</v>
+        <v>45</v>
       </c>
       <c r="M136" t="s">
         <v>915</v>
@@ -9889,7 +9889,7 @@
         <v>61</v>
       </c>
       <c r="L137" t="s">
-        <v>35</v>
+        <v>186</v>
       </c>
       <c r="M137" t="s">
         <v>921</v>

</xml_diff>

<commit_message>
test(PBI-136): harden missing and incomplete audit sequence behavior
</commit_message>
<xml_diff>
--- a/backlog/backlog.xlsx
+++ b/backlog/backlog.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9384"/>
+    <workbookView windowWidth="22188" windowHeight="8784"/>
   </bookViews>
   <sheets>
     <sheet name="backlog" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">backlog!$A$1:$N$138</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">backlog!$A$1:$N$148</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1742" uniqueCount="930">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1862" uniqueCount="996">
   <si>
     <t>PBI-###</t>
   </si>
@@ -2820,6 +2820,204 @@
   </si>
   <si>
     <t>Important: Story-closing task for PBI-122. Evidence should include single-event inspection, chronological sequence retrieval, and incomplete-history handling.</t>
+  </si>
+  <si>
+    <t>PBI-138</t>
+  </si>
+  <si>
+    <t>As an auditor, I want to search access history from the UI, so that I can investigate a selected user or resource without calling backend APIs manually</t>
+  </si>
+  <si>
+    <t>Context: PBI-121 delivers backend access-history query capability, but auditors still need a usable frontend workflow to apply filters and review results. Business problem: backend-only query capability leaves the investigation workflow incomplete for auditor-facing use. User role / actor: auditor. Expected behavior: auditor can enter supported filters and view matching access-history events in stable order from the UI. Business value: turns the access-history query capability into an operationally usable investigation workflow. In scope: search form, filter inputs, result list, empty state, validation feedback, and contract-driven query consumption. Out of scope: event-detail evidence view and chronological sequence inspection.</t>
+  </si>
+  <si>
+    <t>[ReqID: R22] Given an authorized auditor enters supported search filters, when the search is submitted, then the UI displays matching access-history events in the approved stable order. | [ReqID: R22] Given no matching events exist, when the search completes, then the UI shows an empty successful result state rather than an error. | [ReqID: R22] Given invalid filter input is supplied, when the search is attempted, then the UI displays validation or error feedback aligned to the backend contract.</t>
+  </si>
+  <si>
+    <t>Usability;Security;Audit;Maintainability</t>
+  </si>
+  <si>
+    <t>Draft</t>
+  </si>
+  <si>
+    <t>PBI-022;PBI-121;PBI-079;PBI-080;PBI-081;PBI-082</t>
+  </si>
+  <si>
+    <t>Important: Draft scope extension for PBI-022 if the feature is to be treated as a full auditor-facing workflow rather than backend-only audit capability. Consumes the PBI-121 backend query API.</t>
+  </si>
+  <si>
+    <t>PBI-139</t>
+  </si>
+  <si>
+    <t>As an auditor, I want to inspect event-level evidence from the UI, so that I can review who performed an action and what evidence was recorded</t>
+  </si>
+  <si>
+    <t>Context: PBI-122 delivers backend event-detail retrieval, but investigation remains backend-facing unless auditors can inspect evidence through the frontend. Business problem: backend-only event inspection leaves the evidence-review workflow incomplete for operational users. User role / actor: auditor. Expected behavior: auditor can open a selected audit event and review actor, target, outcome, timestamp, request correlation, and non-repudiation evidence fields from the UI. Business value: turns event-detail retrieval into a reviewable, usable investigation capability. In scope: event-detail screen or panel, evidence display, not-found handling, and contract-driven detail retrieval. Out of scope: chronological sequence or timeline view.</t>
+  </si>
+  <si>
+    <t>[ReqID: R22] Given an auditor selects an existing audit event, when the detail view is opened, then the UI displays the approved event evidence fields returned by the backend. | [ReqID: R22] Given a requested event no longer exists or is unavailable, when the detail view is requested, then the UI shows the correct not-found or unavailable state. | [ReqID: R22] Given the backend returns evidence fields for review, when the UI renders them, then the display does not redefine or omit required evidence semantics.</t>
+  </si>
+  <si>
+    <t>Usability;Security;Audit;NonRepudiation</t>
+  </si>
+  <si>
+    <t>PBI-022;PBI-122;PBI-138;PBI-079;PBI-080;PBI-081;PBI-082</t>
+  </si>
+  <si>
+    <t>Important: Draft scope extension for PBI-022. This story should start after the search UI is stable enough to hand off to event-detail inspection.</t>
+  </si>
+  <si>
+    <t>PBI-140</t>
+  </si>
+  <si>
+    <t>As an auditor, I want to view the chronological access sequence from the UI, so that I can understand how the audit trail unfolded around an actor or resource</t>
+  </si>
+  <si>
+    <t>Context: PBI-122 also delivers backend chronological sequence retrieval, but auditors need a readable frontend sequence or timeline to reconstruct investigations efficiently. Business problem: sequence inspection that exists only at API level is operationally weak for day-to-day investigation work. User role / actor: auditor. Expected behavior: auditor can view related audit events in chronological order for the selected actor or target and understand incomplete chains safely. Business value: completes the end-user investigation workflow for access logging and non-repudiation. In scope: sequence/timeline view, chronological ordering display, incomplete-sequence messaging, and contract-driven sequence retrieval. Out of scope: analytics dashboards and external export.</t>
+  </si>
+  <si>
+    <t>[ReqID: R22] Given related events exist for the same actor or target, when the sequence view is opened, then the UI displays the events in chronological order returned by the backend. | [ReqID: R22] Given the sequence is incomplete or limited by current scope, when the auditor views it, then the UI shows the available evidence without implying unsupported completeness. | [ReqID: R22] Given no additional related events exist, when the sequence is requested, then the UI shows the correct limited or empty sequence state without error.</t>
+  </si>
+  <si>
+    <t>PBI-022;PBI-122;PBI-139;PBI-079;PBI-080;PBI-081;PBI-082</t>
+  </si>
+  <si>
+    <t>Important: Draft scope extension for PBI-022. This story completes the auditor-facing workflow if the product owner wants frontend-complete investigation capability.</t>
+  </si>
+  <si>
+    <t>PBI-141</t>
+  </si>
+  <si>
+    <t>Do implement auditor access-history search UI and supported filter controls</t>
+  </si>
+  <si>
+    <t>Action to be performed: build the frontend search form and results list for auditor access-history lookup using the approved filter set from PBI-121. Why it is needed: auditors need a usable interface to query access-history events without relying on direct API use. Expected output: working search form, filter inputs, query submission flow, and result rendering. Scope: filter form, submit action, result list rendering, and backend contract consumption. Explicit exclusions: event-detail inspection and sequence timeline behavior.</t>
+  </si>
+  <si>
+    <t>[ReqID: R22] Given an authorized auditor enters supported search filters, when the form is submitted, then the UI calls the backend query API and renders matching events. | [ReqID: R22] Given matching events are returned, when the UI displays them, then the results preserve the approved ordering and visible summary fields required for investigation.</t>
+  </si>
+  <si>
+    <t>PBI-138;PBI-121;PBI-081</t>
+  </si>
+  <si>
+    <t>Important: First execution task for the auditor search UI slice. The UI must consume the approved query contract from PBI-121 without inventing additional filter semantics.</t>
+  </si>
+  <si>
+    <t>PBI-142</t>
+  </si>
+  <si>
+    <t>Do implement auditor search authorization, empty-state, and validation or error feedback handling</t>
+  </si>
+  <si>
+    <t>Action to be performed: add authorization-aware UI behavior, empty-result messaging, and validation/error handling to the access-history search workflow. Why it is needed: the search story is not complete if it only handles happy-path results. Expected output: stable empty-state, denied-state, and validation/error feedback aligned to backend behavior. Scope: unauthorized access handling, empty results, invalid filter input feedback, and generic error handling. Explicit exclusions: event-detail and sequence views.</t>
+  </si>
+  <si>
+    <t>[ReqID: R22] Given an unauthorized or disallowed actor reaches the search flow, when access is evaluated or the request is submitted, then the UI displays the correct blocked or denied state. | [ReqID: R22] Given no matching events exist, when the search completes, then the UI displays a clear empty-result state. | [ReqID: R22] Given invalid input or backend validation feedback is returned, when the search fails, then the UI displays the correct validation or error message.</t>
+  </si>
+  <si>
+    <t>Usability;Security;Audit</t>
+  </si>
+  <si>
+    <t>PBI-138;PBI-141</t>
+  </si>
+  <si>
+    <t>Important: Keeps negative-path behavior explicit for the UI slice and prevents happy-path-only completion.</t>
+  </si>
+  <si>
+    <t>PBI-143</t>
+  </si>
+  <si>
+    <t>Do execute auditor search UI validation, documentation updates, and demo evidence for PBI-138</t>
+  </si>
+  <si>
+    <t>Action to be performed: validate the full auditor access-history search UI flow, update docs, and collect evidence. Why it is needed: the story is not Done without proof across success, empty, and invalid or denied paths. Expected output: completed UI validation, updated docs, and reviewable evidence. Scope: functional checks, regression checks, screenshots or demo evidence, and documentation updates. Explicit exclusions: event-detail and timeline UI implementation.</t>
+  </si>
+  <si>
+    <t>[ReqID: R22] Given the search UI tasks are complete, when validation is executed, then success, empty, and validation or denied paths behave as documented. | [ReqID: R22] Given the story is prepared for review, when evidence is attached, then screenshots, test results, and updated documentation are available.</t>
+  </si>
+  <si>
+    <t>PBI-138;PBI-141;PBI-142</t>
+  </si>
+  <si>
+    <t>Important: Story-closing task for the auditor search UI. Evidence should include successful query, empty-result state, and denied or invalid-input behavior.</t>
+  </si>
+  <si>
+    <t>PBI-144</t>
+  </si>
+  <si>
+    <t>Do implement auditor event-detail inspection UI and evidence display</t>
+  </si>
+  <si>
+    <t>Action to be performed: build the frontend event-detail inspection view that displays the evidence fields returned by the PBI-122 backend detail API. Why it is needed: auditors need a readable frontend view of the recorded evidence to inspect individual audit events. Expected output: working event-detail view or panel with evidence display. Scope: detail request flow, evidence rendering, navigation from search results, and stable display of approved fields. Explicit exclusions: chronological sequence or timeline view.</t>
+  </si>
+  <si>
+    <t>[ReqID: R22] Given an auditor selects a search result or known event identifier, when the detail view opens, then the UI displays the approved event evidence fields returned by the backend. | [ReqID: R22] Given evidence fields are present, when the UI renders them, then the display preserves the backend-defined meanings for actor, target, outcome, timestamp, request correlation, and non-repudiation evidence.</t>
+  </si>
+  <si>
+    <t>Usability;Security;NonRepudiation;Maintainability</t>
+  </si>
+  <si>
+    <t>PBI-139;PBI-122;PBI-138</t>
+  </si>
+  <si>
+    <t>Important: First execution task for event-detail UI. This task must remain detail-focused and not absorb sequence/timeline work.</t>
+  </si>
+  <si>
+    <t>PBI-145</t>
+  </si>
+  <si>
+    <t>Do implement auditor sequence or timeline UI and navigation from detail inspection</t>
+  </si>
+  <si>
+    <t>Action to be performed: build the frontend sequence or timeline view for related audit events and connect it to the detail-inspection workflow. Why it is needed: auditors need a usable chronological view to reconstruct the access trail around an actor or resource. Expected output: working sequence or timeline UI with chronological event display and navigation from search or detail views. Scope: sequence retrieval trigger, ordered display, related-event rendering, and navigation. Explicit exclusions: analytics dashboards and external export.</t>
+  </si>
+  <si>
+    <t>[ReqID: R22] Given related events exist for the same actor or target, when the sequence view is opened, then the UI displays them in chronological order using the backend sequence response. | [ReqID: R22] Given the auditor moves from event-detail inspection into sequence view, when navigation occurs, then the relevant actor or target context is preserved correctly.</t>
+  </si>
+  <si>
+    <t>Usability;Maintainability;Audit</t>
+  </si>
+  <si>
+    <t>PBI-140;PBI-139;PBI-122</t>
+  </si>
+  <si>
+    <t>Important: This task implements the visible chronological investigation flow and should stay aligned to the backend ordering semantics.</t>
+  </si>
+  <si>
+    <t>PBI-147</t>
+  </si>
+  <si>
+    <t>Do execute auditor event-detail UI validation, documentation updates, and demo evidence for PBI-139</t>
+  </si>
+  <si>
+    <t>Action to be performed: validate the full auditor event-detail inspection UI flow, update docs, and collect evidence. Why it is needed: the story is not Done without proof that auditors can inspect event-level evidence correctly and safely. Expected output: completed UI validation, updated docs, and reviewable evidence for event-detail inspection. Scope: functional checks, regression checks, screenshots or demo evidence, missing-event handling verification, and documentation updates for the detail view. Explicit exclusions: chronological sequence or timeline UI implementation.</t>
+  </si>
+  <si>
+    <t>[ReqID: R22] Given the event-detail UI task is complete, when validation is executed, then event-detail retrieval, evidence display, and missing-event handling behave as documented. | [ReqID: R22] Given the story is prepared for review, when evidence is attached, then screenshots, test results, and updated documentation are available for the event-detail inspection flow.</t>
+  </si>
+  <si>
+    <t>PBI-139;PBI-144</t>
+  </si>
+  <si>
+    <t>Important: Story-closing evidence task for PBI-139 only. Evidence should include successful event-detail inspection and missing-event or unavailable-event handling.</t>
+  </si>
+  <si>
+    <t>PBI-148</t>
+  </si>
+  <si>
+    <t>Do execute auditor sequence or timeline UI validation, documentation updates, and demo evidence for PBI-140</t>
+  </si>
+  <si>
+    <t>Action to be performed: validate the full auditor chronological sequence or timeline UI flow, update docs, and collect evidence. Why it is needed: the story is not Done without proof that auditors can view chronological access trails safely, including incomplete or denied cases. Expected output: completed UI validation, updated docs, and reviewable evidence for sequence or timeline inspection. Scope: functional checks, regression checks, screenshots or demo evidence, incomplete-sequence handling verification, denied-state handling, and documentation updates for the sequence view. Explicit exclusions: new backend capability.</t>
+  </si>
+  <si>
+    <t>[ReqID: R22] Given the sequence or timeline UI tasks are complete, when validation is executed, then chronological sequence display, incomplete-sequence handling, and denied-state behavior match the approved backend contracts. | [ReqID: R22] Given the story is prepared for review, when evidence is attached, then screenshots, test results, and updated documentation are available for the sequence or timeline investigation flow.</t>
+  </si>
+  <si>
+    <t>PBI-140;PBI-145;PBI-146</t>
+  </si>
+  <si>
+    <t>Important: Story-closing evidence task for PBI-140 only. Evidence should include chronological sequence or timeline display, incomplete-sequence handling, and denied-state behavior.</t>
   </si>
 </sst>
 </file>
@@ -4023,7 +4221,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:N138"/>
+  <dimension ref="A1:N148"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:14">
@@ -9889,7 +10087,7 @@
         <v>61</v>
       </c>
       <c r="L137" t="s">
-        <v>186</v>
+        <v>45</v>
       </c>
       <c r="M137" t="s">
         <v>921</v>
@@ -9930,7 +10128,7 @@
         <v>121</v>
       </c>
       <c r="L138" t="s">
-        <v>35</v>
+        <v>186</v>
       </c>
       <c r="M138" t="s">
         <v>928</v>
@@ -9939,8 +10137,418 @@
         <v>929</v>
       </c>
     </row>
+    <row r="139" spans="1:14">
+      <c r="A139" t="s">
+        <v>930</v>
+      </c>
+      <c r="B139" t="s">
+        <v>243</v>
+      </c>
+      <c r="C139" t="s">
+        <v>931</v>
+      </c>
+      <c r="D139" t="s">
+        <v>932</v>
+      </c>
+      <c r="E139" t="s">
+        <v>933</v>
+      </c>
+      <c r="F139" t="s">
+        <v>184</v>
+      </c>
+      <c r="G139" t="s">
+        <v>934</v>
+      </c>
+      <c r="H139">
+        <v>3</v>
+      </c>
+      <c r="I139" t="s">
+        <v>32</v>
+      </c>
+      <c r="J139" t="s">
+        <v>150</v>
+      </c>
+      <c r="L139" t="s">
+        <v>935</v>
+      </c>
+      <c r="M139" t="s">
+        <v>936</v>
+      </c>
+      <c r="N139" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="140" spans="1:14">
+      <c r="A140" t="s">
+        <v>938</v>
+      </c>
+      <c r="B140" t="s">
+        <v>243</v>
+      </c>
+      <c r="C140" t="s">
+        <v>939</v>
+      </c>
+      <c r="D140" t="s">
+        <v>940</v>
+      </c>
+      <c r="E140" t="s">
+        <v>941</v>
+      </c>
+      <c r="F140" t="s">
+        <v>184</v>
+      </c>
+      <c r="G140" t="s">
+        <v>942</v>
+      </c>
+      <c r="H140">
+        <v>3</v>
+      </c>
+      <c r="I140" t="s">
+        <v>32</v>
+      </c>
+      <c r="J140" t="s">
+        <v>150</v>
+      </c>
+      <c r="L140" t="s">
+        <v>935</v>
+      </c>
+      <c r="M140" t="s">
+        <v>943</v>
+      </c>
+      <c r="N140" t="s">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="141" spans="1:14">
+      <c r="A141" t="s">
+        <v>945</v>
+      </c>
+      <c r="B141" t="s">
+        <v>243</v>
+      </c>
+      <c r="C141" t="s">
+        <v>946</v>
+      </c>
+      <c r="D141" t="s">
+        <v>947</v>
+      </c>
+      <c r="E141" t="s">
+        <v>948</v>
+      </c>
+      <c r="F141" t="s">
+        <v>184</v>
+      </c>
+      <c r="G141" t="s">
+        <v>934</v>
+      </c>
+      <c r="H141">
+        <v>3</v>
+      </c>
+      <c r="I141" t="s">
+        <v>21</v>
+      </c>
+      <c r="J141" t="s">
+        <v>150</v>
+      </c>
+      <c r="L141" t="s">
+        <v>935</v>
+      </c>
+      <c r="M141" t="s">
+        <v>949</v>
+      </c>
+      <c r="N141" t="s">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="142" spans="1:14">
+      <c r="A142" t="s">
+        <v>951</v>
+      </c>
+      <c r="B142" t="s">
+        <v>288</v>
+      </c>
+      <c r="C142" t="s">
+        <v>952</v>
+      </c>
+      <c r="D142" t="s">
+        <v>953</v>
+      </c>
+      <c r="E142" t="s">
+        <v>954</v>
+      </c>
+      <c r="F142" t="s">
+        <v>184</v>
+      </c>
+      <c r="G142" t="s">
+        <v>337</v>
+      </c>
+      <c r="H142">
+        <v>2</v>
+      </c>
+      <c r="I142" t="s">
+        <v>32</v>
+      </c>
+      <c r="J142" t="s">
+        <v>150</v>
+      </c>
+      <c r="L142" t="s">
+        <v>935</v>
+      </c>
+      <c r="M142" t="s">
+        <v>955</v>
+      </c>
+      <c r="N142" t="s">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="143" spans="1:14">
+      <c r="A143" t="s">
+        <v>957</v>
+      </c>
+      <c r="B143" t="s">
+        <v>288</v>
+      </c>
+      <c r="C143" t="s">
+        <v>958</v>
+      </c>
+      <c r="D143" t="s">
+        <v>959</v>
+      </c>
+      <c r="E143" t="s">
+        <v>960</v>
+      </c>
+      <c r="F143" t="s">
+        <v>184</v>
+      </c>
+      <c r="G143" t="s">
+        <v>961</v>
+      </c>
+      <c r="H143">
+        <v>2</v>
+      </c>
+      <c r="I143" t="s">
+        <v>32</v>
+      </c>
+      <c r="J143" t="s">
+        <v>150</v>
+      </c>
+      <c r="L143" t="s">
+        <v>935</v>
+      </c>
+      <c r="M143" t="s">
+        <v>962</v>
+      </c>
+      <c r="N143" t="s">
+        <v>963</v>
+      </c>
+    </row>
+    <row r="144" spans="1:14">
+      <c r="A144" t="s">
+        <v>964</v>
+      </c>
+      <c r="B144" t="s">
+        <v>288</v>
+      </c>
+      <c r="C144" t="s">
+        <v>965</v>
+      </c>
+      <c r="D144" t="s">
+        <v>966</v>
+      </c>
+      <c r="E144" t="s">
+        <v>967</v>
+      </c>
+      <c r="F144" t="s">
+        <v>184</v>
+      </c>
+      <c r="G144" t="s">
+        <v>319</v>
+      </c>
+      <c r="H144">
+        <v>2</v>
+      </c>
+      <c r="I144" t="s">
+        <v>32</v>
+      </c>
+      <c r="J144" t="s">
+        <v>121</v>
+      </c>
+      <c r="L144" t="s">
+        <v>935</v>
+      </c>
+      <c r="M144" t="s">
+        <v>968</v>
+      </c>
+      <c r="N144" t="s">
+        <v>969</v>
+      </c>
+    </row>
+    <row r="145" spans="1:14">
+      <c r="A145" t="s">
+        <v>970</v>
+      </c>
+      <c r="B145" t="s">
+        <v>288</v>
+      </c>
+      <c r="C145" t="s">
+        <v>971</v>
+      </c>
+      <c r="D145" t="s">
+        <v>972</v>
+      </c>
+      <c r="E145" t="s">
+        <v>973</v>
+      </c>
+      <c r="F145" t="s">
+        <v>184</v>
+      </c>
+      <c r="G145" t="s">
+        <v>974</v>
+      </c>
+      <c r="H145">
+        <v>2</v>
+      </c>
+      <c r="I145" t="s">
+        <v>32</v>
+      </c>
+      <c r="J145" t="s">
+        <v>150</v>
+      </c>
+      <c r="L145" t="s">
+        <v>935</v>
+      </c>
+      <c r="M145" t="s">
+        <v>975</v>
+      </c>
+      <c r="N145" t="s">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="146" spans="1:14">
+      <c r="A146" t="s">
+        <v>977</v>
+      </c>
+      <c r="B146" t="s">
+        <v>288</v>
+      </c>
+      <c r="C146" t="s">
+        <v>978</v>
+      </c>
+      <c r="D146" t="s">
+        <v>979</v>
+      </c>
+      <c r="E146" t="s">
+        <v>980</v>
+      </c>
+      <c r="F146" t="s">
+        <v>184</v>
+      </c>
+      <c r="G146" t="s">
+        <v>981</v>
+      </c>
+      <c r="H146">
+        <v>2</v>
+      </c>
+      <c r="I146" t="s">
+        <v>21</v>
+      </c>
+      <c r="J146" t="s">
+        <v>150</v>
+      </c>
+      <c r="L146" t="s">
+        <v>935</v>
+      </c>
+      <c r="M146" t="s">
+        <v>982</v>
+      </c>
+      <c r="N146" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="147" spans="1:14">
+      <c r="A147" t="s">
+        <v>984</v>
+      </c>
+      <c r="B147" t="s">
+        <v>288</v>
+      </c>
+      <c r="C147" t="s">
+        <v>985</v>
+      </c>
+      <c r="D147" t="s">
+        <v>986</v>
+      </c>
+      <c r="E147" t="s">
+        <v>987</v>
+      </c>
+      <c r="F147" t="s">
+        <v>184</v>
+      </c>
+      <c r="G147" t="s">
+        <v>744</v>
+      </c>
+      <c r="H147">
+        <v>2</v>
+      </c>
+      <c r="I147" t="s">
+        <v>32</v>
+      </c>
+      <c r="J147" t="s">
+        <v>121</v>
+      </c>
+      <c r="L147" t="s">
+        <v>935</v>
+      </c>
+      <c r="M147" t="s">
+        <v>988</v>
+      </c>
+      <c r="N147" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="148" spans="1:14">
+      <c r="A148" t="s">
+        <v>990</v>
+      </c>
+      <c r="B148" t="s">
+        <v>288</v>
+      </c>
+      <c r="C148" t="s">
+        <v>991</v>
+      </c>
+      <c r="D148" t="s">
+        <v>992</v>
+      </c>
+      <c r="E148" t="s">
+        <v>993</v>
+      </c>
+      <c r="F148" t="s">
+        <v>184</v>
+      </c>
+      <c r="G148" t="s">
+        <v>744</v>
+      </c>
+      <c r="H148">
+        <v>2</v>
+      </c>
+      <c r="I148" t="s">
+        <v>32</v>
+      </c>
+      <c r="J148" t="s">
+        <v>121</v>
+      </c>
+      <c r="L148" t="s">
+        <v>935</v>
+      </c>
+      <c r="M148" t="s">
+        <v>994</v>
+      </c>
+      <c r="N148" t="s">
+        <v>995</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:N138" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:N148" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <sortState ref="A2:N84">

</xml_diff>

<commit_message>
docs(PBI-137): close event inspection story
</commit_message>
<xml_diff>
--- a/backlog/backlog.xlsx
+++ b/backlog/backlog.xlsx
@@ -9513,7 +9513,7 @@
         <v>95</v>
       </c>
       <c r="L123" t="s">
-        <v>186</v>
+        <v>45</v>
       </c>
       <c r="M123" t="s">
         <v>829</v>
@@ -10128,7 +10128,7 @@
         <v>121</v>
       </c>
       <c r="L138" t="s">
-        <v>186</v>
+        <v>45</v>
       </c>
       <c r="M138" t="s">
         <v>928</v>

</xml_diff>